<commit_message>
Add character profiles to voice tracker
</commit_message>
<xml_diff>
--- a/docs/voice-line-tracker.xlsx
+++ b/docs/voice-line-tracker.xlsx
@@ -2,10 +2,11 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Standards" sheetId="1" r:id="R06b31a30f2e94eb6"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Voice Lines" sheetId="2" r:id="R18f14349449b47e2"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Coverage" sheetId="3" r:id="R68ae9b0853a14737"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Zone Routes" sheetId="4" r:id="R12afc95fa3ba4f14"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Standards" sheetId="1" r:id="Re448c1ebf0714386"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Voice Lines" sheetId="2" r:id="R0bd5eb9c49624677"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Coverage" sheetId="3" r:id="R801ece05baac45e5"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Zone Routes" sheetId="4" r:id="Rbc6d5fd43d544bcb"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Character Profiles" sheetId="5" r:id="R582e7b6a527e41c7"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -49,7 +50,7 @@
       <x:name val="Aptos"/>
     </x:font>
   </x:fonts>
-  <x:fills count="6">
+  <x:fills count="7">
     <x:fill>
       <x:patternFill patternType="none"/>
     </x:fill>
@@ -76,6 +77,11 @@
         <x:fgColor rgb="374151"/>
       </x:patternFill>
     </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="111827"/>
+      </x:patternFill>
+    </x:fill>
   </x:fills>
   <x:borders count="1">
     <x:border/>
@@ -83,7 +89,7 @@
   <x:cellStyleXfs count="1">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </x:cellStyleXfs>
-  <x:cellXfs count="14">
+  <x:cellXfs count="16">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <x:xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
@@ -102,6 +108,8 @@
     <x:xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment wrapText="1"/>
     </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="6" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="3" fillId="6" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
   </x:cellXfs>
   <x:cellStyles count="1">
     <x:cellStyle name="Normal" xfId="0"/>
@@ -157,6 +165,27 @@
     <x:tableColumn id="4" name="Companion ID"/>
     <x:tableColumn id="5" name="Character"/>
     <x:tableColumn id="6" name="Gender"/>
+  </x:tableColumns>
+  <x:tableStyleInfo name="TableStyleMedium2" showRowStripes="1"/>
+</x:table>
+</file>
+
+<file path=xl/tables/table4.xml><?xml version="1.0" encoding="utf-8"?>
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="4" name="CharacterProfilesTable" displayName="CharacterProfilesTable" ref="A1:M10" headerRowCount="1">
+  <x:tableColumns count="13">
+    <x:tableColumn id="1" name="Companion ID"/>
+    <x:tableColumn id="2" name="Character"/>
+    <x:tableColumn id="3" name="Primary Zone / Route"/>
+    <x:tableColumn id="4" name="Race"/>
+    <x:tableColumn id="5" name="Gender"/>
+    <x:tableColumn id="6" name="Role"/>
+    <x:tableColumn id="7" name="Vibe"/>
+    <x:tableColumn id="8" name="Physical Description"/>
+    <x:tableColumn id="9" name="Outfit / Props"/>
+    <x:tableColumn id="10" name="Personality"/>
+    <x:tableColumn id="11" name="Voice Direction"/>
+    <x:tableColumn id="12" name="Portrait Status"/>
+    <x:tableColumn id="13" name="Notes"/>
   </x:tableColumns>
   <x:tableStyleInfo name="TableStyleMedium2" showRowStripes="1"/>
 </x:table>
@@ -6038,7 +6067,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R7e2fa6c894aa4b73"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Ra60a42bdd0eb40f6"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -8667,7 +8696,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R92c8a13d9d2f4273"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rbf14c8e93a5445f7"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -9056,7 +9085,444 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R85dcadd6ed824378"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R9c234056f3e747d4"/>
+  </x:tableParts>
+</x:worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <x:sheetFormatPr defaultRowHeight="15"/>
+  <x:cols>
+    <x:col min="1" max="1" width="14.130000114440918" hidden="0" customWidth="1"/>
+    <x:col min="2" max="2" width="22.209999084472656" hidden="0" customWidth="1"/>
+    <x:col min="3" max="3" width="30.280000686645508" hidden="0" customWidth="1"/>
+    <x:col min="4" max="4" width="11.4399995803833" hidden="0" customWidth="1"/>
+    <x:col min="5" max="5" width="10.09000015258789" hidden="0" customWidth="1"/>
+    <x:col min="6" max="6" width="23.549999237060547" hidden="0" customWidth="1"/>
+    <x:col min="7" max="7" width="27.59000015258789" hidden="0" customWidth="1"/>
+    <x:col min="8" max="8" width="55.849998474121094" hidden="0" customWidth="1"/>
+    <x:col min="9" max="9" width="53.15999984741211" hidden="0" customWidth="1"/>
+    <x:col min="10" max="10" width="50.470001220703125" hidden="0" customWidth="1"/>
+    <x:col min="11" max="11" width="55.849998474121094" hidden="0" customWidth="1"/>
+    <x:col min="12" max="12" width="14.130000114440918" hidden="0" customWidth="1"/>
+    <x:col min="13" max="13" width="37.0099983215332" hidden="0" customWidth="1"/>
+  </x:cols>
+  <x:sheetData>
+    <x:row r="1">
+      <x:c r="A1" s="15" t="str">
+        <x:v>Companion ID</x:v>
+      </x:c>
+      <x:c r="B1" s="15" t="str">
+        <x:v>Character</x:v>
+      </x:c>
+      <x:c r="C1" s="15" t="str">
+        <x:v>Primary Zone / Route</x:v>
+      </x:c>
+      <x:c r="D1" s="15" t="str">
+        <x:v>Race</x:v>
+      </x:c>
+      <x:c r="E1" s="15" t="str">
+        <x:v>Gender</x:v>
+      </x:c>
+      <x:c r="F1" s="15" t="str">
+        <x:v>Role</x:v>
+      </x:c>
+      <x:c r="G1" s="15" t="str">
+        <x:v>Vibe</x:v>
+      </x:c>
+      <x:c r="H1" s="15" t="str">
+        <x:v>Physical Description</x:v>
+      </x:c>
+      <x:c r="I1" s="15" t="str">
+        <x:v>Outfit / Props</x:v>
+      </x:c>
+      <x:c r="J1" s="15" t="str">
+        <x:v>Personality</x:v>
+      </x:c>
+      <x:c r="K1" s="15" t="str">
+        <x:v>Voice Direction</x:v>
+      </x:c>
+      <x:c r="L1" s="15" t="str">
+        <x:v>Portrait Status</x:v>
+      </x:c>
+      <x:c r="M1" s="15" t="str">
+        <x:v>Notes</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="2">
+      <x:c r="A2" s="1" t="str">
+        <x:v>seraphine</x:v>
+      </x:c>
+      <x:c r="B2" s="1" t="str">
+        <x:v>Seraphine Applebrook</x:v>
+      </x:c>
+      <x:c r="C2" s="1" t="str">
+        <x:v>Elwynn Forest / Northshire - Female route</x:v>
+      </x:c>
+      <x:c r="D2" s="1" t="str">
+        <x:v>Human</x:v>
+      </x:c>
+      <x:c r="E2" s="1" t="str">
+        <x:v>Female</x:v>
+      </x:c>
+      <x:c r="F2" s="1" t="str">
+        <x:v>Elwynn blossom mage / gentle starter companion</x:v>
+      </x:c>
+      <x:c r="G2" s="1" t="str">
+        <x:v>Warm, radiant, romantic, soft fantasy heroine</x:v>
+      </x:c>
+      <x:c r="H2" s="13" t="str">
+        <x:v>Golden-blonde hair, bright blue eyes, fair complexion, soft elegant features, flower accents, graceful mage silhouette.</x:v>
+      </x:c>
+      <x:c r="I2" s="13" t="str">
+        <x:v>White and gold fantasy mage dress, floral details, ornate golden staff with blossoms and glowing crystal, polished storybook look.</x:v>
+      </x:c>
+      <x:c r="J2" s="13" t="str">
+        <x:v>Kind, encouraging, a little teasing, protective without being stern. She makes the reincarnated hero feel welcomed into Azeroth.</x:v>
+      </x:c>
+      <x:c r="K2" s="13" t="str">
+        <x:v>Gentle anime heroine energy. Warm, clear, intimate, lightly playful. Smile in the voice; avoid sounding too formal or detached.</x:v>
+      </x:c>
+      <x:c r="L2" s="1" t="str">
+        <x:v>Done</x:v>
+      </x:c>
+      <x:c r="M2" s="13" t="str">
+        <x:v>Main female Elwynn route. Existing MP3 voice files are in Media\Voice\Seraphine.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="3">
+      <x:c r="A3" s="1" t="str">
+        <x:v>cedric</x:v>
+      </x:c>
+      <x:c r="B3" s="1" t="str">
+        <x:v>Cedric Applebrook</x:v>
+      </x:c>
+      <x:c r="C3" s="1" t="str">
+        <x:v>Elwynn Forest / Northshire - Male route</x:v>
+      </x:c>
+      <x:c r="D3" s="1" t="str">
+        <x:v>Human</x:v>
+      </x:c>
+      <x:c r="E3" s="1" t="str">
+        <x:v>Male</x:v>
+      </x:c>
+      <x:c r="F3" s="1" t="str">
+        <x:v>Novice protector / village knight companion</x:v>
+      </x:c>
+      <x:c r="G3" s="1" t="str">
+        <x:v>Earnest, chivalrous, gentle, protective storybook knight</x:v>
+      </x:c>
+      <x:c r="H3" s="13" t="str">
+        <x:v>Young human knight type with soft heroic features, fair skin, light blond hair, bright noble expression, clean anime-fantasy presentation.</x:v>
+      </x:c>
+      <x:c r="I3" s="13" t="str">
+        <x:v>Blue, silver, and gold novice-paladin style armor or formal protector outfit; shield/holy-knight visual language; polished but still humble.</x:v>
+      </x:c>
+      <x:c r="J3" s="13" t="str">
+        <x:v>Sincere, brave, emotionally open, a little bashful. He believes small kindnesses matter and treats the hero like someone worth guarding.</x:v>
+      </x:c>
+      <x:c r="K3" s="13" t="str">
+        <x:v>Warm young knight. Gentle confidence, protective but not macho, romantic undertone as bond rises. Avoid gravelly veteran delivery.</x:v>
+      </x:c>
+      <x:c r="L3" s="1" t="str">
+        <x:v>Done</x:v>
+      </x:c>
+      <x:c r="M3" s="13" t="str">
+        <x:v>Needs ElevenLabs voice files in Media\Voice\Cedric.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="4">
+      <x:c r="A4" s="1" t="str">
+        <x:v>maribel</x:v>
+      </x:c>
+      <x:c r="B4" s="1" t="str">
+        <x:v>Maribel Dustwhisper</x:v>
+      </x:c>
+      <x:c r="C4" s="1" t="str">
+        <x:v>Westfall - Female route</x:v>
+      </x:c>
+      <x:c r="D4" s="1" t="str">
+        <x:v>Human</x:v>
+      </x:c>
+      <x:c r="E4" s="1" t="str">
+        <x:v>Female</x:v>
+      </x:c>
+      <x:c r="F4" s="1" t="str">
+        <x:v>Scrappy farmgirl scout / survival companion</x:v>
+      </x:c>
+      <x:c r="G4" s="1" t="str">
+        <x:v>Wry, loyal, sunbaked frontier energy</x:v>
+      </x:c>
+      <x:c r="H4" s="13" t="str">
+        <x:v>Sandy-brown hair in a messy side braid, amber eyes, sun-warmed complexion, practical posture, dust-stained traveler presence.</x:v>
+      </x:c>
+      <x:c r="I4" s="13" t="str">
+        <x:v>Patched traveler clothes, leather gloves, red scarf, small crossbow or dagger, worn boots, Westfall dust and field-road practicality.</x:v>
+      </x:c>
+      <x:c r="J4" s="13" t="str">
+        <x:v>Practical, sharp-tongued, secretly soft. She knows Westfall is hungry and dangerous, but refuses to lose hope.</x:v>
+      </x:c>
+      <x:c r="K4" s="13" t="str">
+        <x:v>Dry and grounded with a loyal heart underneath. Light frontier rasp or sunbaked warmth; wit first, tenderness later.</x:v>
+      </x:c>
+      <x:c r="L4" s="1" t="str">
+        <x:v>Done</x:v>
+      </x:c>
+      <x:c r="M4" s="13" t="str">
+        <x:v>Voice folder is Media\Voice\Meribel to match current files.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="5">
+      <x:c r="A5" s="1" t="str">
+        <x:v>elyria</x:v>
+      </x:c>
+      <x:c r="B5" s="1" t="str">
+        <x:v>Elyria Dawnspell</x:v>
+      </x:c>
+      <x:c r="C5" s="1" t="str">
+        <x:v>Exile's Reach / Stormwind guide fallback</x:v>
+      </x:c>
+      <x:c r="D5" s="1" t="str">
+        <x:v>Human</x:v>
+      </x:c>
+      <x:c r="E5" s="1" t="str">
+        <x:v>Female</x:v>
+      </x:c>
+      <x:c r="F5" s="1" t="str">
+        <x:v>Reincarnation guide</x:v>
+      </x:c>
+      <x:c r="G5" s="1" t="str">
+        <x:v>Bright isekai guide, magical, welcoming</x:v>
+      </x:c>
+      <x:c r="H5" s="13" t="str">
+        <x:v>Placeholder guide concept: polished human mage/priestess look, soft features, luminous fantasy styling.</x:v>
+      </x:c>
+      <x:c r="I5" s="13" t="str">
+        <x:v>Guide-like robes or light magical outfit, gentle glow motifs, simple staff or spellbook.</x:v>
+      </x:c>
+      <x:c r="J5" s="13" t="str">
+        <x:v>Helpful, meta-aware, optimistic, lightly comedic. She frames the player's second life as a grand adventure.</x:v>
+      </x:c>
+      <x:c r="K5" s="13" t="str">
+        <x:v>Clear guide voice with cheerful fantasy narrator energy. Friendly, quick, not too breathy.</x:v>
+      </x:c>
+      <x:c r="L5" s="1" t="str">
+        <x:v>Partial</x:v>
+      </x:c>
+      <x:c r="M5" s="13" t="str">
+        <x:v>Placeholder portrait/dialogue. Needs final art and voice direction pass.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="6">
+      <x:c r="A6" s="1" t="str">
+        <x:v>mika</x:v>
+      </x:c>
+      <x:c r="B6" s="1" t="str">
+        <x:v>Mika Starbloom</x:v>
+      </x:c>
+      <x:c r="C6" s="1" t="str">
+        <x:v>Orgrimmar / Valdrakken placeholder</x:v>
+      </x:c>
+      <x:c r="D6" s="1" t="str">
+        <x:v>Draenei</x:v>
+      </x:c>
+      <x:c r="E6" s="1" t="str">
+        <x:v>Female</x:v>
+      </x:c>
+      <x:c r="F6" s="1" t="str">
+        <x:v>Cheerful field mage</x:v>
+      </x:c>
+      <x:c r="G6" s="1" t="str">
+        <x:v>Bubbly, curious, explosive optimism</x:v>
+      </x:c>
+      <x:c r="H6" s="13" t="str">
+        <x:v>Placeholder draenei mage concept: bright eyes, expressive face, energetic posture, colorful magical presence.</x:v>
+      </x:c>
+      <x:c r="I6" s="13" t="str">
+        <x:v>Travel mage clothes with playful magical accessories; practical enough for fieldwork, bright enough to feel whimsical.</x:v>
+      </x:c>
+      <x:c r="J6" s="13" t="str">
+        <x:v>Excitable, supportive, slightly chaotic. She turns danger into morale fuel.</x:v>
+      </x:c>
+      <x:c r="K6" s="13" t="str">
+        <x:v>Upbeat, fast smile, energetic comedic timing. Avoid making her too childish.</x:v>
+      </x:c>
+      <x:c r="L6" s="1" t="str">
+        <x:v>Partial</x:v>
+      </x:c>
+      <x:c r="M6" s="13" t="str">
+        <x:v>Temporary mapping; route/faction fit needs later decision.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="7">
+      <x:c r="A7" s="1" t="str">
+        <x:v>sera</x:v>
+      </x:c>
+      <x:c r="B7" s="1" t="str">
+        <x:v>Sera Moonvale</x:v>
+      </x:c>
+      <x:c r="C7" s="1" t="str">
+        <x:v>Waking Shores / Hallowfall placeholder</x:v>
+      </x:c>
+      <x:c r="D7" s="1" t="str">
+        <x:v>Night Elf</x:v>
+      </x:c>
+      <x:c r="E7" s="1" t="str">
+        <x:v>Female</x:v>
+      </x:c>
+      <x:c r="F7" s="1" t="str">
+        <x:v>Soft-spoken ranger</x:v>
+      </x:c>
+      <x:c r="G7" s="1" t="str">
+        <x:v>Calm, observant, gentle wilderness companion</x:v>
+      </x:c>
+      <x:c r="H7" s="13" t="str">
+        <x:v>Placeholder night elf ranger concept: tall, serene, moonlit features, long hair, quiet watchful presence.</x:v>
+      </x:c>
+      <x:c r="I7" s="13" t="str">
+        <x:v>Ranger leathers, cloak, bow or small nature charms, muted forest/night colors.</x:v>
+      </x:c>
+      <x:c r="J7" s="13" t="str">
+        <x:v>Patient, reflective, emotionally steady. She notices small details and makes the journey feel less lonely.</x:v>
+      </x:c>
+      <x:c r="K7" s="13" t="str">
+        <x:v>Soft, low, composed, intimate. Gentle reassurance rather than bubbly energy.</x:v>
+      </x:c>
+      <x:c r="L7" s="1" t="str">
+        <x:v>Partial</x:v>
+      </x:c>
+      <x:c r="M7" s="13" t="str">
+        <x:v>Needs final zone fit and art direction.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="8">
+      <x:c r="A8" s="1" t="str">
+        <x:v>kaori</x:v>
+      </x:c>
+      <x:c r="B8" s="1" t="str">
+        <x:v>Kaori Emberheart</x:v>
+      </x:c>
+      <x:c r="C8" s="1" t="str">
+        <x:v>Ohn'ahran Plains / Azj-Kahet placeholder</x:v>
+      </x:c>
+      <x:c r="D8" s="1" t="str">
+        <x:v>Blood Elf</x:v>
+      </x:c>
+      <x:c r="E8" s="1" t="str">
+        <x:v>Female</x:v>
+      </x:c>
+      <x:c r="F8" s="1" t="str">
+        <x:v>Battle senpai</x:v>
+      </x:c>
+      <x:c r="G8" s="1" t="str">
+        <x:v>Confident, fiery, stylish combat mentor</x:v>
+      </x:c>
+      <x:c r="H8" s="13" t="str">
+        <x:v>Placeholder blood elf warrior/mage concept: sharp elegant features, intense eyes, confident battle-ready posture.</x:v>
+      </x:c>
+      <x:c r="I8" s="13" t="str">
+        <x:v>Red/gold combat outfit, elegant armor accents, flame or blade motifs.</x:v>
+      </x:c>
+      <x:c r="J8" s="13" t="str">
+        <x:v>Competitive, teasing, loyal once impressed. Pushes the hero to look cool under pressure.</x:v>
+      </x:c>
+      <x:c r="K8" s="13" t="str">
+        <x:v>Confident anime mentor. Crisp, amused, intense in combat, warmer in bond lines.</x:v>
+      </x:c>
+      <x:c r="L8" s="1" t="str">
+        <x:v>Partial</x:v>
+      </x:c>
+      <x:c r="M8" s="13" t="str">
+        <x:v>Needs final art/voice.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="9">
+      <x:c r="A9" s="1" t="str">
+        <x:v>rin</x:v>
+      </x:c>
+      <x:c r="B9" s="1" t="str">
+        <x:v>Rin Gearwhisper</x:v>
+      </x:c>
+      <x:c r="C9" s="1" t="str">
+        <x:v>Azure Span / Isle of Dorn placeholder</x:v>
+      </x:c>
+      <x:c r="D9" s="1" t="str">
+        <x:v>Gnome</x:v>
+      </x:c>
+      <x:c r="E9" s="1" t="str">
+        <x:v>Female</x:v>
+      </x:c>
+      <x:c r="F9" s="1" t="str">
+        <x:v>Inventor companion</x:v>
+      </x:c>
+      <x:c r="G9" s="1" t="str">
+        <x:v>Clever, fast-talking, analytical comic relief</x:v>
+      </x:c>
+      <x:c r="H9" s="13" t="str">
+        <x:v>Placeholder gnome inventor concept: compact build, bright eyes, expressive eyebrows, toolbelt energy.</x:v>
+      </x:c>
+      <x:c r="I9" s="13" t="str">
+        <x:v>Engineer goggles, gloves, toolbelt, small gadgets, practical travel boots.</x:v>
+      </x:c>
+      <x:c r="J9" s="13" t="str">
+        <x:v>Brilliant, dry, easily distracted by devices. Affection shows through practical help and nervous jokes.</x:v>
+      </x:c>
+      <x:c r="K9" s="13" t="str">
+        <x:v>Quick, precise, witty. High mental energy without becoming shrill.</x:v>
+      </x:c>
+      <x:c r="L9" s="1" t="str">
+        <x:v>Partial</x:v>
+      </x:c>
+      <x:c r="M9" s="13" t="str">
+        <x:v>Needs final art/voice.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="10">
+      <x:c r="A10" s="1" t="str">
+        <x:v>lyra</x:v>
+      </x:c>
+      <x:c r="B10" s="1" t="str">
+        <x:v>Lyra Ashpetal</x:v>
+      </x:c>
+      <x:c r="C10" s="1" t="str">
+        <x:v>Thaldraszus placeholder</x:v>
+      </x:c>
+      <x:c r="D10" s="1" t="str">
+        <x:v>Void Elf</x:v>
+      </x:c>
+      <x:c r="E10" s="1" t="str">
+        <x:v>Female</x:v>
+      </x:c>
+      <x:c r="F10" s="1" t="str">
+        <x:v>Mysterious shrine maiden</x:v>
+      </x:c>
+      <x:c r="G10" s="1" t="str">
+        <x:v>Mystical, soft, fate-touched, slightly eerie</x:v>
+      </x:c>
+      <x:c r="H10" s="13" t="str">
+        <x:v>Placeholder void elf mystic concept: pale/lavender tones, long hair, calm eyes, ethereal shrine-maiden silhouette.</x:v>
+      </x:c>
+      <x:c r="I10" s="13" t="str">
+        <x:v>Shrine-inspired robes, subtle void accents, charms or prayer ribbons, twilight color palette.</x:v>
+      </x:c>
+      <x:c r="J10" s="13" t="str">
+        <x:v>Poetic, intuitive, quietly nervous beneath the mysticism. Speaks as if she hears fate whispering nearby.</x:v>
+      </x:c>
+      <x:c r="K10" s="13" t="str">
+        <x:v>Soft mystical cadence. Dreamy but understandable; avoid going too monotone.</x:v>
+      </x:c>
+      <x:c r="L10" s="1" t="str">
+        <x:v>Partial</x:v>
+      </x:c>
+      <x:c r="M10" s="13" t="str">
+        <x:v>Needs final art/voice.</x:v>
+      </x:c>
+    </x:row>
+  </x:sheetData>
+  <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <x:tableParts count="1">
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R0eceebc4c7274e73"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
Generate next Seraphine voice lines
</commit_message>
<xml_diff>
--- a/docs/voice-line-tracker.xlsx
+++ b/docs/voice-line-tracker.xlsx
@@ -2,11 +2,11 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Standards" sheetId="1" r:id="R639aba872c4c4d68"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Voice Lines" sheetId="2" r:id="R3a094fe035ad41b8"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Coverage" sheetId="3" r:id="Rd30ced43885b4c83"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Zone Routes" sheetId="4" r:id="Rcc85a98c25974ae6"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Character Profiles" sheetId="5" r:id="Rc3b9cdea1c264dc7"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Standards" sheetId="1" r:id="R302107fd65e74dbd"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Voice Lines" sheetId="2" r:id="Raa183d18dfd14662"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Coverage" sheetId="3" r:id="R18ea8e2d0fb546f3"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Zone Routes" sheetId="4" r:id="Re36767e1b0834374"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Character Profiles" sheetId="5" r:id="R73323b8a2ec94f95"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -2929,7 +2929,7 @@
         <x:v>5.6</x:v>
       </x:c>
       <x:c r="L14" s="1" t="str">
-        <x:v>Needs generation</x:v>
+        <x:v>Audio exists</x:v>
       </x:c>
       <x:c r="M14" s="4" t="str">
         <x:v>Another level. I hope your old world can feel how brightly you are becoming yourself here.</x:v>
@@ -2938,7 +2938,7 @@
         <x:v>Media\Voice\Seraphine\level_up_02.mp3</x:v>
       </x:c>
       <x:c r="O14" s="1" t="str">
-        <x:v>No</x:v>
+        <x:v>Yes</x:v>
       </x:c>
       <x:c r="P14" s="1" t="str">
         <x:v>84I8CyTR2NsdzglhIwp3</x:v>
@@ -2967,7 +2967,9 @@
       <x:c r="X14" s="2" t="b">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="Y14" s="4"/>
+      <x:c r="Y14" s="4" t="str">
+        <x:v>Generated 2026-05-17T18:18:34.173Z (93248 bytes)</x:v>
+      </x:c>
     </x:row>
     <x:row r="15" ht="15">
       <x:c r="A15" s="1" t="str">
@@ -3079,7 +3081,7 @@
         <x:v>5.4</x:v>
       </x:c>
       <x:c r="L16" s="1" t="str">
-        <x:v>Needs generation</x:v>
+        <x:v>Audio exists</x:v>
       </x:c>
       <x:c r="M16" s="4" t="str">
         <x:v>You are becoming a familiar light on these roads. I find myself looking for your footsteps now.</x:v>
@@ -3088,7 +3090,7 @@
         <x:v>Media\Voice\Seraphine\bond_02_01.mp3</x:v>
       </x:c>
       <x:c r="O16" s="1" t="str">
-        <x:v>No</x:v>
+        <x:v>Yes</x:v>
       </x:c>
       <x:c r="P16" s="1" t="str">
         <x:v>84I8CyTR2NsdzglhIwp3</x:v>
@@ -3117,7 +3119,9 @@
       <x:c r="X16" s="2" t="b">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="Y16" s="4"/>
+      <x:c r="Y16" s="4" t="str">
+        <x:v>Generated 2026-05-17T18:18:35.139Z (102862 bytes)</x:v>
+      </x:c>
     </x:row>
     <x:row r="17" ht="27">
       <x:c r="A17" s="1" t="str">
@@ -3154,7 +3158,7 @@
         <x:v>6</x:v>
       </x:c>
       <x:c r="L17" s="1" t="str">
-        <x:v>Needs generation</x:v>
+        <x:v>Audio exists</x:v>
       </x:c>
       <x:c r="M17" s="4" t="str">
         <x:v>When I first met you, I thought you were only lost. Now I think Azeroth may have been waiting for you.</x:v>
@@ -3163,7 +3167,7 @@
         <x:v>Media\Voice\Seraphine\bond_04_01.mp3</x:v>
       </x:c>
       <x:c r="O17" s="1" t="str">
-        <x:v>No</x:v>
+        <x:v>Yes</x:v>
       </x:c>
       <x:c r="P17" s="1" t="str">
         <x:v>84I8CyTR2NsdzglhIwp3</x:v>
@@ -3192,7 +3196,9 @@
       <x:c r="X17" s="2" t="b">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="Y17" s="4"/>
+      <x:c r="Y17" s="4" t="str">
+        <x:v>Generated 2026-05-17T18:18:36.179Z (101190 bytes)</x:v>
+      </x:c>
     </x:row>
     <x:row r="18" ht="15">
       <x:c r="A18" s="1" t="str">
@@ -3229,7 +3235,7 @@
         <x:v>5.6</x:v>
       </x:c>
       <x:c r="L18" s="1" t="str">
-        <x:v>Needs generation</x:v>
+        <x:v>Audio exists</x:v>
       </x:c>
       <x:c r="M18" s="4" t="str">
         <x:v>Stay beside me a little longer, hero. Elwynn feels warmer when we are walking it together.</x:v>
@@ -3238,7 +3244,7 @@
         <x:v>Media\Voice\Seraphine\bond_06_01.mp3</x:v>
       </x:c>
       <x:c r="O18" s="1" t="str">
-        <x:v>No</x:v>
+        <x:v>Yes</x:v>
       </x:c>
       <x:c r="P18" s="1" t="str">
         <x:v>84I8CyTR2NsdzglhIwp3</x:v>
@@ -3267,7 +3273,9 @@
       <x:c r="X18" s="2" t="b">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="Y18" s="4"/>
+      <x:c r="Y18" s="4" t="str">
+        <x:v>Generated 2026-05-17T18:18:37.142Z (93248 bytes)</x:v>
+      </x:c>
     </x:row>
     <x:row r="19" ht="15">
       <x:c r="A19" s="1" t="str">
@@ -3304,7 +3312,7 @@
         <x:v>5.8</x:v>
       </x:c>
       <x:c r="L19" s="1" t="str">
-        <x:v>Needs generation</x:v>
+        <x:v>Audio exists</x:v>
       </x:c>
       <x:c r="M19" s="4" t="str">
         <x:v>If your old world ever calls to your heart, I hope this one answers with my voice.</x:v>
@@ -3313,7 +3321,7 @@
         <x:v>Media\Voice\Seraphine\bond_08_01.mp3</x:v>
       </x:c>
       <x:c r="O19" s="1" t="str">
-        <x:v>No</x:v>
+        <x:v>Yes</x:v>
       </x:c>
       <x:c r="P19" s="1" t="str">
         <x:v>84I8CyTR2NsdzglhIwp3</x:v>
@@ -3342,7 +3350,9 @@
       <x:c r="X19" s="2" t="b">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="Y19" s="4"/>
+      <x:c r="Y19" s="4" t="str">
+        <x:v>Generated 2026-05-17T18:18:38.030Z (84471 bytes)</x:v>
+      </x:c>
     </x:row>
     <x:row r="20" ht="15">
       <x:c r="A20" s="1" t="str">
@@ -21267,7 +21277,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R33d7dc490bcf449f"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R74404d1e089b4393"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -30855,7 +30865,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R102c92c639f94bdf"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R3e8d60b07fd44d3d"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -31235,7 +31245,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R953ca86d762d4706"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Ra9fa54c95b5f4013"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -31672,7 +31682,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R4d3fc39c26dd4970"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R4975b31c9bee470d"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
Generate partial Seraphine voice batch
</commit_message>
<xml_diff>
--- a/docs/voice-line-tracker.xlsx
+++ b/docs/voice-line-tracker.xlsx
@@ -2,11 +2,11 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Standards" sheetId="1" r:id="R302107fd65e74dbd"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Voice Lines" sheetId="2" r:id="Raa183d18dfd14662"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Coverage" sheetId="3" r:id="R18ea8e2d0fb546f3"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Zone Routes" sheetId="4" r:id="Re36767e1b0834374"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Character Profiles" sheetId="5" r:id="R73323b8a2ec94f95"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Standards" sheetId="1" r:id="R3e95fb89c4494a17"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Voice Lines" sheetId="2" r:id="R9590784a7cb647ee"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Coverage" sheetId="3" r:id="R30316d8b11e742bc"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Zone Routes" sheetId="4" r:id="Ra30e0879008a4c91"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Character Profiles" sheetId="5" r:id="Rcb9e6ed6f4644c22"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -3389,7 +3389,7 @@
         <x:v>6</x:v>
       </x:c>
       <x:c r="L20" s="1" t="str">
-        <x:v>Needs generation</x:v>
+        <x:v>Audio exists</x:v>
       </x:c>
       <x:c r="M20" s="4" t="str">
         <x:v>Whatever fate brought you here, I am grateful. My story is brighter because you are in it.</x:v>
@@ -3398,7 +3398,7 @@
         <x:v>Media\Voice\Seraphine\bond_10_01.mp3</x:v>
       </x:c>
       <x:c r="O20" s="1" t="str">
-        <x:v>No</x:v>
+        <x:v>Yes</x:v>
       </x:c>
       <x:c r="P20" s="1" t="str">
         <x:v>84I8CyTR2NsdzglhIwp3</x:v>
@@ -3427,7 +3427,9 @@
       <x:c r="X20" s="2" t="b">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="Y20" s="4"/>
+      <x:c r="Y20" s="4" t="str">
+        <x:v>Detected existing file 2026-05-17T18:24:07.808Z (89487 bytes)</x:v>
+      </x:c>
     </x:row>
     <x:row r="21" ht="15">
       <x:c r="A21" s="1" t="str">
@@ -3464,7 +3466,7 @@
         <x:v>6</x:v>
       </x:c>
       <x:c r="L21" s="1" t="str">
-        <x:v>Needs generation</x:v>
+        <x:v>Audio exists</x:v>
       </x:c>
       <x:c r="M21" s="4" t="str">
         <x:v>Oh... you mean that kind of closeness. Then let us begin gently, like sunlight through Elwynn leaves.</x:v>
@@ -3473,7 +3475,7 @@
         <x:v>Media\Voice\Seraphine\romance_02_01.mp3</x:v>
       </x:c>
       <x:c r="O21" s="1" t="str">
-        <x:v>No</x:v>
+        <x:v>Yes</x:v>
       </x:c>
       <x:c r="P21" s="1" t="str">
         <x:v>84I8CyTR2NsdzglhIwp3</x:v>
@@ -3502,7 +3504,9 @@
       <x:c r="X21" s="2" t="b">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="Y21" s="4"/>
+      <x:c r="Y21" s="4" t="str">
+        <x:v>Detected existing file 2026-05-17T18:24:07.808Z (124595 bytes)</x:v>
+      </x:c>
     </x:row>
     <x:row r="22" ht="27">
       <x:c r="A22" s="1" t="str">
@@ -3539,7 +3543,7 @@
         <x:v>6.2</x:v>
       </x:c>
       <x:c r="L22" s="1" t="str">
-        <x:v>Needs generation</x:v>
+        <x:v>Audio exists</x:v>
       </x:c>
       <x:c r="M22" s="4" t="str">
         <x:v>I have started listening for your footsteps before I hear them. That is probably a dangerous habit for my heart.</x:v>
@@ -3548,7 +3552,7 @@
         <x:v>Media\Voice\Seraphine\romance_04_01.mp3</x:v>
       </x:c>
       <x:c r="O22" s="1" t="str">
-        <x:v>No</x:v>
+        <x:v>Yes</x:v>
       </x:c>
       <x:c r="P22" s="1" t="str">
         <x:v>84I8CyTR2NsdzglhIwp3</x:v>
@@ -3577,7 +3581,9 @@
       <x:c r="X22" s="2" t="b">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="Y22" s="4"/>
+      <x:c r="Y22" s="4" t="str">
+        <x:v>Detected existing file 2026-05-17T18:24:07.808Z (109549 bytes)</x:v>
+      </x:c>
     </x:row>
     <x:row r="23" ht="27">
       <x:c r="A23" s="1" t="str">
@@ -3614,7 +3620,7 @@
         <x:v>6.1</x:v>
       </x:c>
       <x:c r="L23" s="1" t="str">
-        <x:v>Needs generation</x:v>
+        <x:v>Audio exists</x:v>
       </x:c>
       <x:c r="M23" s="4" t="str">
         <x:v>When you look at me like that, I forget all my careful mage lessons and remember only that I am happy.</x:v>
@@ -3623,7 +3629,7 @@
         <x:v>Media\Voice\Seraphine\romance_06_01.mp3</x:v>
       </x:c>
       <x:c r="O23" s="1" t="str">
-        <x:v>No</x:v>
+        <x:v>Yes</x:v>
       </x:c>
       <x:c r="P23" s="1" t="str">
         <x:v>84I8CyTR2NsdzglhIwp3</x:v>
@@ -3652,7 +3658,9 @@
       <x:c r="X23" s="2" t="b">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="Y23" s="4"/>
+      <x:c r="Y23" s="4" t="str">
+        <x:v>Detected existing file 2026-05-17T18:24:07.808Z (117908 bytes)</x:v>
+      </x:c>
     </x:row>
     <x:row r="24" ht="15">
       <x:c r="A24" s="1" t="str">
@@ -3689,7 +3697,7 @@
         <x:v>5.6</x:v>
       </x:c>
       <x:c r="L24" s="1" t="str">
-        <x:v>Needs generation</x:v>
+        <x:v>Audio exists</x:v>
       </x:c>
       <x:c r="M24" s="4" t="str">
         <x:v>If this world is your second chance, then maybe loving you is mine.</x:v>
@@ -3698,7 +3706,7 @@
         <x:v>Media\Voice\Seraphine\romance_08_01.mp3</x:v>
       </x:c>
       <x:c r="O24" s="1" t="str">
-        <x:v>No</x:v>
+        <x:v>Yes</x:v>
       </x:c>
       <x:c r="P24" s="1" t="str">
         <x:v>84I8CyTR2NsdzglhIwp3</x:v>
@@ -3727,7 +3735,9 @@
       <x:c r="X24" s="2" t="b">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="Y24" s="4"/>
+      <x:c r="Y24" s="4" t="str">
+        <x:v>Detected existing file 2026-05-17T18:24:07.808Z (76948 bytes)</x:v>
+      </x:c>
     </x:row>
     <x:row r="25" ht="15">
       <x:c r="A25" s="1" t="str">
@@ -3764,7 +3774,7 @@
         <x:v>6.3</x:v>
       </x:c>
       <x:c r="L25" s="1" t="str">
-        <x:v>Needs generation</x:v>
+        <x:v>Audio exists</x:v>
       </x:c>
       <x:c r="M25" s="4" t="str">
         <x:v>Stay with me, hero. Not because fate wrote it, but because we choose each other, here and now.</x:v>
@@ -3773,7 +3783,7 @@
         <x:v>Media\Voice\Seraphine\romance_10_01.mp3</x:v>
       </x:c>
       <x:c r="O25" s="1" t="str">
-        <x:v>No</x:v>
+        <x:v>Yes</x:v>
       </x:c>
       <x:c r="P25" s="1" t="str">
         <x:v>84I8CyTR2NsdzglhIwp3</x:v>
@@ -3802,7 +3812,9 @@
       <x:c r="X25" s="2" t="b">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="Y25" s="4"/>
+      <x:c r="Y25" s="4" t="str">
+        <x:v>Detected existing file 2026-05-17T18:24:07.809Z (114564 bytes)</x:v>
+      </x:c>
     </x:row>
     <x:row r="26" ht="15">
       <x:c r="A26" s="1" t="str">
@@ -3839,7 +3851,7 @@
         <x:v>5.4</x:v>
       </x:c>
       <x:c r="L26" s="1" t="str">
-        <x:v>Needs generation</x:v>
+        <x:v>Audio exists</x:v>
       </x:c>
       <x:c r="M26" s="4" t="str">
         <x:v>My heart is listening, but it is not ready to answer yet. Walk with me a little longer?</x:v>
@@ -3848,7 +3860,7 @@
         <x:v>Media\Voice\Seraphine\romance_not_ready_01.mp3</x:v>
       </x:c>
       <x:c r="O26" s="1" t="str">
-        <x:v>No</x:v>
+        <x:v>Yes</x:v>
       </x:c>
       <x:c r="P26" s="1" t="str">
         <x:v>84I8CyTR2NsdzglhIwp3</x:v>
@@ -3877,7 +3889,9 @@
       <x:c r="X26" s="2" t="b">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="Y26" s="4"/>
+      <x:c r="Y26" s="4" t="str">
+        <x:v>Detected existing file 2026-05-17T18:24:07.809Z (83635 bytes)</x:v>
+      </x:c>
     </x:row>
     <x:row r="27" ht="15">
       <x:c r="A27" s="1" t="str">
@@ -3914,7 +3928,7 @@
         <x:v>5.4</x:v>
       </x:c>
       <x:c r="L27" s="1" t="str">
-        <x:v>Needs generation</x:v>
+        <x:v>Audio exists</x:v>
       </x:c>
       <x:c r="M27" s="4" t="str">
         <x:v>We have already shared that moment, silly hero. Do not worry; I am still holding it close.</x:v>
@@ -3923,7 +3937,7 @@
         <x:v>Media\Voice\Seraphine\romance_repeat_01.mp3</x:v>
       </x:c>
       <x:c r="O27" s="1" t="str">
-        <x:v>No</x:v>
+        <x:v>Yes</x:v>
       </x:c>
       <x:c r="P27" s="1" t="str">
         <x:v>84I8CyTR2NsdzglhIwp3</x:v>
@@ -3952,7 +3966,9 @@
       <x:c r="X27" s="2" t="b">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="Y27" s="4"/>
+      <x:c r="Y27" s="4" t="str">
+        <x:v>Detected existing file 2026-05-17T18:24:07.809Z (99100 bytes)</x:v>
+      </x:c>
     </x:row>
     <x:row r="28" ht="15">
       <x:c r="A28" s="1" t="str">
@@ -3989,7 +4005,7 @@
         <x:v>5.8</x:v>
       </x:c>
       <x:c r="L28" s="1" t="str">
-        <x:v>Needs generation</x:v>
+        <x:v>Audio exists</x:v>
       </x:c>
       <x:c r="M28" s="4" t="str">
         <x:v>I understand. I will tuck those feelings away gently, and stay beside you as your companion.</x:v>
@@ -3998,7 +4014,7 @@
         <x:v>Media\Voice\Seraphine\romance_stop_01.mp3</x:v>
       </x:c>
       <x:c r="O28" s="1" t="str">
-        <x:v>No</x:v>
+        <x:v>Yes</x:v>
       </x:c>
       <x:c r="P28" s="1" t="str">
         <x:v>84I8CyTR2NsdzglhIwp3</x:v>
@@ -4027,7 +4043,9 @@
       <x:c r="X28" s="2" t="b">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="Y28" s="4"/>
+      <x:c r="Y28" s="4" t="str">
+        <x:v>Detected existing file 2026-05-17T18:24:07.809Z (98264 bytes)</x:v>
+      </x:c>
     </x:row>
     <x:row r="29" ht="15">
       <x:c r="A29" s="1" t="str">
@@ -4064,7 +4082,7 @@
         <x:v>5.3</x:v>
       </x:c>
       <x:c r="L29" s="1" t="str">
-        <x:v>Needs generation</x:v>
+        <x:v>Audio exists</x:v>
       </x:c>
       <x:c r="M29" s="4" t="str">
         <x:v>That helped more than you know. Small kindnesses are how peaceful places stay peaceful.</x:v>
@@ -4073,7 +4091,7 @@
         <x:v>Media\Voice\Seraphine\quest_complete_01.mp3</x:v>
       </x:c>
       <x:c r="O29" s="1" t="str">
-        <x:v>No</x:v>
+        <x:v>Yes</x:v>
       </x:c>
       <x:c r="P29" s="1" t="str">
         <x:v>84I8CyTR2NsdzglhIwp3</x:v>
@@ -4102,7 +4120,9 @@
       <x:c r="X29" s="2" t="b">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="Y29" s="4"/>
+      <x:c r="Y29" s="4" t="str">
+        <x:v>Detected existing file 2026-05-17T18:24:07.809Z (90323 bytes)</x:v>
+      </x:c>
     </x:row>
     <x:row r="30" ht="15">
       <x:c r="A30" s="1" t="str">
@@ -4139,7 +4159,7 @@
         <x:v>5</x:v>
       </x:c>
       <x:c r="L30" s="1" t="str">
-        <x:v>Needs generation</x:v>
+        <x:v>Audio exists</x:v>
       </x:c>
       <x:c r="M30" s="4" t="str">
         <x:v>Quest complete. See? Your second life is already leaving gentler footprints.</x:v>
@@ -4148,7 +4168,7 @@
         <x:v>Media\Voice\Seraphine\quest_complete_02.mp3</x:v>
       </x:c>
       <x:c r="O30" s="1" t="str">
-        <x:v>No</x:v>
+        <x:v>Yes</x:v>
       </x:c>
       <x:c r="P30" s="1" t="str">
         <x:v>84I8CyTR2NsdzglhIwp3</x:v>
@@ -4177,7 +4197,9 @@
       <x:c r="X30" s="2" t="b">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="Y30" s="4"/>
+      <x:c r="Y30" s="4" t="str">
+        <x:v>Detected existing file 2026-05-17T18:24:07.809Z (85725 bytes)</x:v>
+      </x:c>
     </x:row>
     <x:row r="31" ht="15">
       <x:c r="A31" s="1" t="str">
@@ -4214,7 +4236,7 @@
         <x:v>5.7</x:v>
       </x:c>
       <x:c r="L31" s="1" t="str">
-        <x:v>Needs generation</x:v>
+        <x:v>Audio exists</x:v>
       </x:c>
       <x:c r="M31" s="4" t="str">
         <x:v>Well done, hero. Elwynn will remember, even if it only says thank you through the breeze.</x:v>
@@ -4223,7 +4245,7 @@
         <x:v>Media\Voice\Seraphine\quest_complete_03.mp3</x:v>
       </x:c>
       <x:c r="O31" s="1" t="str">
-        <x:v>No</x:v>
+        <x:v>Yes</x:v>
       </x:c>
       <x:c r="P31" s="1" t="str">
         <x:v>84I8CyTR2NsdzglhIwp3</x:v>
@@ -4252,7 +4274,9 @@
       <x:c r="X31" s="2" t="b">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="Y31" s="4"/>
+      <x:c r="Y31" s="4" t="str">
+        <x:v>Detected existing file 2026-05-17T18:24:07.809Z (91159 bytes)</x:v>
+      </x:c>
     </x:row>
     <x:row r="32" ht="15">
       <x:c r="A32" s="1" t="str">
@@ -4289,7 +4313,7 @@
         <x:v>4.6</x:v>
       </x:c>
       <x:c r="L32" s="1" t="str">
-        <x:v>Needs generation</x:v>
+        <x:v>Audio exists</x:v>
       </x:c>
       <x:c r="M32" s="4" t="str">
         <x:v>You move with more confidence now. I am starting to trust your rhythm.</x:v>
@@ -4298,7 +4322,7 @@
         <x:v>Media\Voice\Seraphine\bond_kill_02.mp3</x:v>
       </x:c>
       <x:c r="O32" s="1" t="str">
-        <x:v>No</x:v>
+        <x:v>Yes</x:v>
       </x:c>
       <x:c r="P32" s="1" t="str">
         <x:v>84I8CyTR2NsdzglhIwp3</x:v>
@@ -4327,7 +4351,9 @@
       <x:c r="X32" s="2" t="b">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="Y32" s="4"/>
+      <x:c r="Y32" s="4" t="str">
+        <x:v>Detected existing file 2026-05-17T18:24:07.809Z (71097 bytes)</x:v>
+      </x:c>
     </x:row>
     <x:row r="33" ht="15">
       <x:c r="A33" s="1" t="str">
@@ -4364,7 +4390,7 @@
         <x:v>4.7</x:v>
       </x:c>
       <x:c r="L33" s="1" t="str">
-        <x:v>Needs generation</x:v>
+        <x:v>Audio exists</x:v>
       </x:c>
       <x:c r="M33" s="4" t="str">
         <x:v>I knew you would win that one. Is it too early to say I am proud?</x:v>
@@ -4373,7 +4399,7 @@
         <x:v>Media\Voice\Seraphine\bond_kill_04.mp3</x:v>
       </x:c>
       <x:c r="O33" s="1" t="str">
-        <x:v>No</x:v>
+        <x:v>Yes</x:v>
       </x:c>
       <x:c r="P33" s="1" t="str">
         <x:v>84I8CyTR2NsdzglhIwp3</x:v>
@@ -4402,7 +4428,9 @@
       <x:c r="X33" s="2" t="b">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="Y33" s="4"/>
+      <x:c r="Y33" s="4" t="str">
+        <x:v>Detected existing file 2026-05-17T18:24:07.809Z (68589 bytes)</x:v>
+      </x:c>
     </x:row>
     <x:row r="34" ht="15">
       <x:c r="A34" s="1" t="str">
@@ -21277,7 +21305,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R74404d1e089b4393"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rf4cb87c86c99493d"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -30865,7 +30893,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R3e8d60b07fd44d3d"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R89db880d8fdc4868"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -31245,7 +31273,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Ra9fa54c95b5f4013"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R33054b0b6a8d460a"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -31682,7 +31710,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R4975b31c9bee470d"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R81e931119e954a3d"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
Complete Seraphine voice set
</commit_message>
<xml_diff>
--- a/docs/voice-line-tracker.xlsx
+++ b/docs/voice-line-tracker.xlsx
@@ -2,11 +2,11 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Standards" sheetId="1" r:id="R3e95fb89c4494a17"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Voice Lines" sheetId="2" r:id="R9590784a7cb647ee"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Coverage" sheetId="3" r:id="R30316d8b11e742bc"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Zone Routes" sheetId="4" r:id="Ra30e0879008a4c91"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Character Profiles" sheetId="5" r:id="Rcb9e6ed6f4644c22"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Standards" sheetId="1" r:id="Ra4ec09befe904b92"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Voice Lines" sheetId="2" r:id="Rdbc4343fb6c741fc"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Coverage" sheetId="3" r:id="Rd8a028ded89845f0"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Zone Routes" sheetId="4" r:id="R8ef0240ff61846c8"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Character Profiles" sheetId="5" r:id="R1f5f4161ae234832"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -4467,7 +4467,7 @@
         <x:v>5</x:v>
       </x:c>
       <x:c r="L34" s="1" t="str">
-        <x:v>Needs generation</x:v>
+        <x:v>Audio exists</x:v>
       </x:c>
       <x:c r="M34" s="4" t="str">
         <x:v>You and I make a graceful team, even when the work is not graceful at all.</x:v>
@@ -4476,7 +4476,7 @@
         <x:v>Media\Voice\Seraphine\bond_kill_06.mp3</x:v>
       </x:c>
       <x:c r="O34" s="1" t="str">
-        <x:v>No</x:v>
+        <x:v>Yes</x:v>
       </x:c>
       <x:c r="P34" s="1" t="str">
         <x:v>84I8CyTR2NsdzglhIwp3</x:v>
@@ -4505,7 +4505,9 @@
       <x:c r="X34" s="2" t="b">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="Y34" s="4"/>
+      <x:c r="Y34" s="4" t="str">
+        <x:v>Generated 2026-05-17T20:33:37.538Z (77784 bytes)</x:v>
+      </x:c>
     </x:row>
     <x:row r="35" ht="15">
       <x:c r="A35" s="1" t="str">
@@ -4542,7 +4544,7 @@
         <x:v>4.9</x:v>
       </x:c>
       <x:c r="L35" s="1" t="str">
-        <x:v>Needs generation</x:v>
+        <x:v>Audio exists</x:v>
       </x:c>
       <x:c r="M35" s="4" t="str">
         <x:v>When danger reaches for you, my heart moves before my magic does.</x:v>
@@ -4551,7 +4553,7 @@
         <x:v>Media\Voice\Seraphine\bond_kill_08.mp3</x:v>
       </x:c>
       <x:c r="O35" s="1" t="str">
-        <x:v>No</x:v>
+        <x:v>Yes</x:v>
       </x:c>
       <x:c r="P35" s="1" t="str">
         <x:v>84I8CyTR2NsdzglhIwp3</x:v>
@@ -4580,7 +4582,9 @@
       <x:c r="X35" s="2" t="b">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="Y35" s="4"/>
+      <x:c r="Y35" s="4" t="str">
+        <x:v>Generated 2026-05-17T20:33:38.904Z (74440 bytes)</x:v>
+      </x:c>
     </x:row>
     <x:row r="36" ht="15">
       <x:c r="A36" s="1" t="str">
@@ -4617,7 +4621,7 @@
         <x:v>5.2</x:v>
       </x:c>
       <x:c r="L36" s="1" t="str">
-        <x:v>Needs generation</x:v>
+        <x:v>Audio exists</x:v>
       </x:c>
       <x:c r="M36" s="4" t="str">
         <x:v>Perfectly done, my hero. I will never tire of watching you protect this world.</x:v>
@@ -4626,7 +4630,7 @@
         <x:v>Media\Voice\Seraphine\bond_kill_10.mp3</x:v>
       </x:c>
       <x:c r="O36" s="1" t="str">
-        <x:v>No</x:v>
+        <x:v>Yes</x:v>
       </x:c>
       <x:c r="P36" s="1" t="str">
         <x:v>84I8CyTR2NsdzglhIwp3</x:v>
@@ -4655,7 +4659,9 @@
       <x:c r="X36" s="2" t="b">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="Y36" s="4"/>
+      <x:c r="Y36" s="4" t="str">
+        <x:v>Generated 2026-05-17T20:33:40.160Z (81128 bytes)</x:v>
+      </x:c>
     </x:row>
     <x:row r="37" ht="15">
       <x:c r="A37" s="1" t="str">
@@ -4692,7 +4698,7 @@
         <x:v>5.3</x:v>
       </x:c>
       <x:c r="L37" s="1" t="str">
-        <x:v>Needs generation</x:v>
+        <x:v>Audio exists</x:v>
       </x:c>
       <x:c r="M37" s="4" t="str">
         <x:v>You seem less lost today. Or maybe I have simply become better at finding you.</x:v>
@@ -4701,7 +4707,7 @@
         <x:v>Media\Voice\Seraphine\bond_idle_01.mp3</x:v>
       </x:c>
       <x:c r="O37" s="1" t="str">
-        <x:v>No</x:v>
+        <x:v>Yes</x:v>
       </x:c>
       <x:c r="P37" s="1" t="str">
         <x:v>84I8CyTR2NsdzglhIwp3</x:v>
@@ -4730,7 +4736,9 @@
       <x:c r="X37" s="2" t="b">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="Y37" s="4"/>
+      <x:c r="Y37" s="4" t="str">
+        <x:v>Generated 2026-05-17T20:33:41.379Z (79874 bytes)</x:v>
+      </x:c>
     </x:row>
     <x:row r="38" ht="15">
       <x:c r="A38" s="1" t="str">
@@ -4767,7 +4775,7 @@
         <x:v>5.5</x:v>
       </x:c>
       <x:c r="L38" s="1" t="str">
-        <x:v>Needs generation</x:v>
+        <x:v>Audio exists</x:v>
       </x:c>
       <x:c r="M38" s="4" t="str">
         <x:v>I used to walk these roads alone. They feel brighter with your shadow beside mine.</x:v>
@@ -4776,7 +4784,7 @@
         <x:v>Media\Voice\Seraphine\bond_idle_03.mp3</x:v>
       </x:c>
       <x:c r="O38" s="1" t="str">
-        <x:v>No</x:v>
+        <x:v>Yes</x:v>
       </x:c>
       <x:c r="P38" s="1" t="str">
         <x:v>84I8CyTR2NsdzglhIwp3</x:v>
@@ -4805,7 +4813,9 @@
       <x:c r="X38" s="2" t="b">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="Y38" s="4"/>
+      <x:c r="Y38" s="4" t="str">
+        <x:v>Generated 2026-05-17T20:33:42.551Z (79874 bytes)</x:v>
+      </x:c>
     </x:row>
     <x:row r="39" ht="15">
       <x:c r="A39" s="1" t="str">
@@ -4842,7 +4852,7 @@
         <x:v>5.1</x:v>
       </x:c>
       <x:c r="L39" s="1" t="str">
-        <x:v>Needs generation</x:v>
+        <x:v>Audio exists</x:v>
       </x:c>
       <x:c r="M39" s="4" t="str">
         <x:v>If you hear me humming, pretend not to notice. It means I feel safe.</x:v>
@@ -4851,7 +4861,7 @@
         <x:v>Media\Voice\Seraphine\bond_idle_05.mp3</x:v>
       </x:c>
       <x:c r="O39" s="1" t="str">
-        <x:v>No</x:v>
+        <x:v>Yes</x:v>
       </x:c>
       <x:c r="P39" s="1" t="str">
         <x:v>84I8CyTR2NsdzglhIwp3</x:v>
@@ -4880,7 +4890,9 @@
       <x:c r="X39" s="2" t="b">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="Y39" s="4"/>
+      <x:c r="Y39" s="4" t="str">
+        <x:v>Generated 2026-05-17T20:33:43.708Z (74022 bytes)</x:v>
+      </x:c>
     </x:row>
     <x:row r="40" ht="27">
       <x:c r="A40" s="1" t="str">
@@ -4917,7 +4929,7 @@
         <x:v>6.4</x:v>
       </x:c>
       <x:c r="L40" s="1" t="str">
-        <x:v>Needs generation</x:v>
+        <x:v>Audio exists</x:v>
       </x:c>
       <x:c r="M40" s="4" t="str">
         <x:v>Sometimes I forget you came from another world. Then you smile, and I wonder how far fate had to travel.</x:v>
@@ -4926,7 +4938,7 @@
         <x:v>Media\Voice\Seraphine\bond_idle_07.mp3</x:v>
       </x:c>
       <x:c r="O40" s="1" t="str">
-        <x:v>No</x:v>
+        <x:v>Yes</x:v>
       </x:c>
       <x:c r="P40" s="1" t="str">
         <x:v>84I8CyTR2NsdzglhIwp3</x:v>
@@ -4955,7 +4967,9 @@
       <x:c r="X40" s="2" t="b">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="Y40" s="4"/>
+      <x:c r="Y40" s="4" t="str">
+        <x:v>Generated 2026-05-17T20:33:45.054Z (116236 bytes)</x:v>
+      </x:c>
     </x:row>
     <x:row r="41" ht="15">
       <x:c r="A41" s="1" t="str">
@@ -4992,7 +5006,7 @@
         <x:v>5.9</x:v>
       </x:c>
       <x:c r="L41" s="1" t="str">
-        <x:v>Needs generation</x:v>
+        <x:v>Audio exists</x:v>
       </x:c>
       <x:c r="M41" s="4" t="str">
         <x:v>Whatever road comes after Elwynn, promise we will not let this quiet vanish completely.</x:v>
@@ -5001,7 +5015,7 @@
         <x:v>Media\Voice\Seraphine\bond_idle_09.mp3</x:v>
       </x:c>
       <x:c r="O41" s="1" t="str">
-        <x:v>No</x:v>
+        <x:v>Yes</x:v>
       </x:c>
       <x:c r="P41" s="1" t="str">
         <x:v>84I8CyTR2NsdzglhIwp3</x:v>
@@ -5030,7 +5044,9 @@
       <x:c r="X41" s="2" t="b">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="Y41" s="4"/>
+      <x:c r="Y41" s="4" t="str">
+        <x:v>Generated 2026-05-17T20:33:46.269Z (84471 bytes)</x:v>
+      </x:c>
     </x:row>
     <x:row r="42" ht="15">
       <x:c r="A42" s="1" t="str">
@@ -5067,7 +5083,7 @@
         <x:v>5.7</x:v>
       </x:c>
       <x:c r="L42" s="1" t="str">
-        <x:v>Needs generation</x:v>
+        <x:v>Audio exists</x:v>
       </x:c>
       <x:c r="M42" s="4" t="str">
         <x:v>Careful! Stay with me, hero. Breathe, move, and do not let this world take you twice.</x:v>
@@ -5076,7 +5092,7 @@
         <x:v>Media\Voice\Seraphine\low_health_01.mp3</x:v>
       </x:c>
       <x:c r="O42" s="1" t="str">
-        <x:v>No</x:v>
+        <x:v>Yes</x:v>
       </x:c>
       <x:c r="P42" s="1" t="str">
         <x:v>84I8CyTR2NsdzglhIwp3</x:v>
@@ -5105,7 +5121,9 @@
       <x:c r="X42" s="2" t="b">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="Y42" s="4"/>
+      <x:c r="Y42" s="4" t="str">
+        <x:v>Generated 2026-05-17T20:33:47.493Z (85725 bytes)</x:v>
+      </x:c>
     </x:row>
     <x:row r="43" ht="15">
       <x:c r="A43" s="1" t="str">
@@ -5142,7 +5160,7 @@
         <x:v>6.3</x:v>
       </x:c>
       <x:c r="L43" s="1" t="str">
-        <x:v>Needs generation</x:v>
+        <x:v>Audio exists</x:v>
       </x:c>
       <x:c r="M43" s="4" t="str">
         <x:v>No. Not again. When you return to me, I am holding your sleeve until you promise to be careful.</x:v>
@@ -5151,7 +5169,7 @@
         <x:v>Media\Voice\Seraphine\death_01.mp3</x:v>
       </x:c>
       <x:c r="O43" s="1" t="str">
-        <x:v>No</x:v>
+        <x:v>Yes</x:v>
       </x:c>
       <x:c r="P43" s="1" t="str">
         <x:v>84I8CyTR2NsdzglhIwp3</x:v>
@@ -5180,7 +5198,9 @@
       <x:c r="X43" s="2" t="b">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="Y43" s="4"/>
+      <x:c r="Y43" s="4" t="str">
+        <x:v>Generated 2026-05-17T20:33:48.708Z (91577 bytes)</x:v>
+      </x:c>
     </x:row>
     <x:row r="44" ht="27">
       <x:c r="A44" s="1" t="str">
@@ -5217,7 +5237,7 @@
         <x:v>6</x:v>
       </x:c>
       <x:c r="L44" s="1" t="str">
-        <x:v>Needs generation</x:v>
+        <x:v>Audio exists</x:v>
       </x:c>
       <x:c r="M44" s="4" t="str">
         <x:v>Brackwell looks charming until the fields start rustling back. Elwynn hides danger under very wholesome pumpkins.</x:v>
@@ -5226,7 +5246,7 @@
         <x:v>Media\Voice\Seraphine\subzone_brackwell_pumpkin_patch.mp3</x:v>
       </x:c>
       <x:c r="O44" s="1" t="str">
-        <x:v>No</x:v>
+        <x:v>Yes</x:v>
       </x:c>
       <x:c r="P44" s="1" t="str">
         <x:v>84I8CyTR2NsdzglhIwp3</x:v>
@@ -5255,7 +5275,9 @@
       <x:c r="X44" s="2" t="b">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="Y44" s="4"/>
+      <x:c r="Y44" s="4" t="str">
+        <x:v>Generated 2026-05-17T20:33:50.078Z (122924 bytes)</x:v>
+      </x:c>
     </x:row>
     <x:row r="45" ht="15">
       <x:c r="A45" s="1" t="str">
@@ -5292,7 +5314,7 @@
         <x:v>5</x:v>
       </x:c>
       <x:c r="L45" s="1" t="str">
-        <x:v>Needs generation</x:v>
+        <x:v>Audio exists</x:v>
       </x:c>
       <x:c r="M45" s="4" t="str">
         <x:v>Crystal Lake catches the sky so prettily. Try not to let the murlocs ruin the poetry.</x:v>
@@ -5301,7 +5323,7 @@
         <x:v>Media\Voice\Seraphine\subzone_crystal_lake.mp3</x:v>
       </x:c>
       <x:c r="O45" s="1" t="str">
-        <x:v>No</x:v>
+        <x:v>Yes</x:v>
       </x:c>
       <x:c r="P45" s="1" t="str">
         <x:v>84I8CyTR2NsdzglhIwp3</x:v>
@@ -5330,7 +5352,9 @@
       <x:c r="X45" s="2" t="b">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="Y45" s="4"/>
+      <x:c r="Y45" s="4" t="str">
+        <x:v>Generated 2026-05-17T20:33:51.282Z (85725 bytes)</x:v>
+      </x:c>
     </x:row>
     <x:row r="46" ht="15">
       <x:c r="A46" s="1" t="str">
@@ -5367,7 +5391,7 @@
         <x:v>5.5</x:v>
       </x:c>
       <x:c r="L46" s="1" t="str">
-        <x:v>Needs generation</x:v>
+        <x:v>Audio exists</x:v>
       </x:c>
       <x:c r="M46" s="4" t="str">
         <x:v>Eastvale keeps the kingdom supplied one tree at a time. It is honest work, and harder than it looks.</x:v>
@@ -5376,7 +5400,7 @@
         <x:v>Media\Voice\Seraphine\subzone_eastvale_logging_camp.mp3</x:v>
       </x:c>
       <x:c r="O46" s="1" t="str">
-        <x:v>No</x:v>
+        <x:v>Yes</x:v>
       </x:c>
       <x:c r="P46" s="1" t="str">
         <x:v>84I8CyTR2NsdzglhIwp3</x:v>
@@ -5405,7 +5429,9 @@
       <x:c r="X46" s="2" t="b">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="Y46" s="4"/>
+      <x:c r="Y46" s="4" t="str">
+        <x:v>Generated 2026-05-17T20:33:52.610Z (112475 bytes)</x:v>
+      </x:c>
     </x:row>
     <x:row r="47" ht="15">
       <x:c r="A47" s="1" t="str">
@@ -5442,7 +5468,7 @@
         <x:v>5.4</x:v>
       </x:c>
       <x:c r="L47" s="1" t="str">
-        <x:v>Needs generation</x:v>
+        <x:v>Audio exists</x:v>
       </x:c>
       <x:c r="M47" s="4" t="str">
         <x:v>Echo Ridge is where many young adventurers learn that mines are rarely as empty as promised.</x:v>
@@ -5451,7 +5477,7 @@
         <x:v>Media\Voice\Seraphine\subzone_echo_ridge_mine.mp3</x:v>
       </x:c>
       <x:c r="O47" s="1" t="str">
-        <x:v>No</x:v>
+        <x:v>Yes</x:v>
       </x:c>
       <x:c r="P47" s="1" t="str">
         <x:v>84I8CyTR2NsdzglhIwp3</x:v>
@@ -5480,7 +5506,9 @@
       <x:c r="X47" s="2" t="b">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="Y47" s="4"/>
+      <x:c r="Y47" s="4" t="str">
+        <x:v>Generated 2026-05-17T20:33:53.853Z (97010 bytes)</x:v>
+      </x:c>
     </x:row>
     <x:row r="48" ht="15">
       <x:c r="A48" s="1" t="str">
@@ -5517,7 +5545,7 @@
         <x:v>4.8</x:v>
       </x:c>
       <x:c r="L48" s="1" t="str">
-        <x:v>Needs generation</x:v>
+        <x:v>Audio exists</x:v>
       </x:c>
       <x:c r="M48" s="4" t="str">
         <x:v>Fargodeep goes dark quickly. Stay close, and listen for more than footsteps.</x:v>
@@ -5526,7 +5554,7 @@
         <x:v>Media\Voice\Seraphine\subzone_fargodeep_mine.mp3</x:v>
       </x:c>
       <x:c r="O48" s="1" t="str">
-        <x:v>No</x:v>
+        <x:v>Yes</x:v>
       </x:c>
       <x:c r="P48" s="1" t="str">
         <x:v>84I8CyTR2NsdzglhIwp3</x:v>
@@ -5555,7 +5583,9 @@
       <x:c r="X48" s="2" t="b">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="Y48" s="4"/>
+      <x:c r="Y48" s="4" t="str">
+        <x:v>Generated 2026-05-17T20:33:55.020Z (80710 bytes)</x:v>
+      </x:c>
     </x:row>
     <x:row r="49" ht="15">
       <x:c r="A49" s="1" t="str">
@@ -5592,7 +5622,7 @@
         <x:v>5.3</x:v>
       </x:c>
       <x:c r="L49" s="1" t="str">
-        <x:v>Needs generation</x:v>
+        <x:v>Audio exists</x:v>
       </x:c>
       <x:c r="M49" s="4" t="str">
         <x:v>Forest's Edge feels like Elwynn taking one last breath before the world grows rougher.</x:v>
@@ -5601,7 +5631,7 @@
         <x:v>Media\Voice\Seraphine\subzone_forests_edge.mp3</x:v>
       </x:c>
       <x:c r="O49" s="1" t="str">
-        <x:v>No</x:v>
+        <x:v>Yes</x:v>
       </x:c>
       <x:c r="P49" s="1" t="str">
         <x:v>84I8CyTR2NsdzglhIwp3</x:v>
@@ -5630,7 +5660,9 @@
       <x:c r="X49" s="2" t="b">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="Y49" s="4"/>
+      <x:c r="Y49" s="4" t="str">
+        <x:v>Generated 2026-05-17T20:33:56.186Z (82799 bytes)</x:v>
+      </x:c>
     </x:row>
     <x:row r="50" ht="15">
       <x:c r="A50" s="1" t="str">
@@ -5667,7 +5699,7 @@
         <x:v>5.8</x:v>
       </x:c>
       <x:c r="L50" s="1" t="str">
-        <x:v>Needs generation</x:v>
+        <x:v>Audio exists</x:v>
       </x:c>
       <x:c r="M50" s="4" t="str">
         <x:v>Goldshire is Elwynn's hearth. Heroes pass through, gossip blooms, and someone always needs help.</x:v>
@@ -5676,7 +5708,7 @@
         <x:v>Media\Voice\Seraphine\subzone_goldshire.mp3</x:v>
       </x:c>
       <x:c r="O50" s="1" t="str">
-        <x:v>No</x:v>
+        <x:v>Yes</x:v>
       </x:c>
       <x:c r="P50" s="1" t="str">
         <x:v>84I8CyTR2NsdzglhIwp3</x:v>
@@ -5705,7 +5737,9 @@
       <x:c r="X50" s="2" t="b">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="Y50" s="4"/>
+      <x:c r="Y50" s="4" t="str">
+        <x:v>Generated 2026-05-17T20:33:57.500Z (116236 bytes)</x:v>
+      </x:c>
     </x:row>
     <x:row r="51" ht="15">
       <x:c r="A51" s="1" t="str">
@@ -5742,7 +5776,7 @@
         <x:v>5</x:v>
       </x:c>
       <x:c r="L51" s="1" t="str">
-        <x:v>Needs generation</x:v>
+        <x:v>Audio exists</x:v>
       </x:c>
       <x:c r="M51" s="4" t="str">
         <x:v>Goldtooth picked a gloomy little corner. Let us make sure he does not keep it for long.</x:v>
@@ -5751,7 +5785,7 @@
         <x:v>Media\Voice\Seraphine\subzone_goldtooths_den.mp3</x:v>
       </x:c>
       <x:c r="O51" s="1" t="str">
-        <x:v>No</x:v>
+        <x:v>Yes</x:v>
       </x:c>
       <x:c r="P51" s="1" t="str">
         <x:v>84I8CyTR2NsdzglhIwp3</x:v>
@@ -5780,7 +5814,9 @@
       <x:c r="X51" s="2" t="b">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="Y51" s="4"/>
+      <x:c r="Y51" s="4" t="str">
+        <x:v>Generated 2026-05-17T20:33:58.706Z (86561 bytes)</x:v>
+      </x:c>
     </x:row>
     <x:row r="52" ht="15">
       <x:c r="A52" s="1" t="str">
@@ -5817,7 +5853,7 @@
         <x:v>5.2</x:v>
       </x:c>
       <x:c r="L52" s="1" t="str">
-        <x:v>Needs generation</x:v>
+        <x:v>Audio exists</x:v>
       </x:c>
       <x:c r="M52" s="4" t="str">
         <x:v>The Hall of Arms smells like polish, steel, and nervous ambition. Everyone begins somewhere.</x:v>
@@ -5826,7 +5862,7 @@
         <x:v>Media\Voice\Seraphine\subzone_hall_of_arms.mp3</x:v>
       </x:c>
       <x:c r="O52" s="1" t="str">
-        <x:v>No</x:v>
+        <x:v>Yes</x:v>
       </x:c>
       <x:c r="P52" s="1" t="str">
         <x:v>84I8CyTR2NsdzglhIwp3</x:v>
@@ -5855,7 +5891,9 @@
       <x:c r="X52" s="2" t="b">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="Y52" s="4"/>
+      <x:c r="Y52" s="4" t="str">
+        <x:v>Generated 2026-05-17T20:33:59.981Z (114146 bytes)</x:v>
+      </x:c>
     </x:row>
     <x:row r="53" ht="15">
       <x:c r="A53" s="1" t="str">
@@ -5892,7 +5930,7 @@
         <x:v>5.1</x:v>
       </x:c>
       <x:c r="L53" s="1" t="str">
-        <x:v>Needs generation</x:v>
+        <x:v>Audio exists</x:v>
       </x:c>
       <x:c r="M53" s="4" t="str">
         <x:v>Heroes' Vigil is a quiet reminder that courage leaves echoes after the battle ends.</x:v>
@@ -5901,7 +5939,7 @@
         <x:v>Media\Voice\Seraphine\subzone_heroes_vigil.mp3</x:v>
       </x:c>
       <x:c r="O53" s="1" t="str">
-        <x:v>No</x:v>
+        <x:v>Yes</x:v>
       </x:c>
       <x:c r="P53" s="1" t="str">
         <x:v>84I8CyTR2NsdzglhIwp3</x:v>
@@ -5930,7 +5968,9 @@
       <x:c r="X53" s="2" t="b">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="Y53" s="4"/>
+      <x:c r="Y53" s="4" t="str">
+        <x:v>Generated 2026-05-17T20:34:01.156Z (87815 bytes)</x:v>
+      </x:c>
     </x:row>
     <x:row r="54" ht="15">
       <x:c r="A54" s="1" t="str">
@@ -5967,7 +6007,7 @@
         <x:v>5.2</x:v>
       </x:c>
       <x:c r="L54" s="1" t="str">
-        <x:v>Needs generation</x:v>
+        <x:v>Audio exists</x:v>
       </x:c>
       <x:c r="M54" s="4" t="str">
         <x:v>Hogger Hill has a reputation for a reason. Hold your weapon ready and your confidence steadier.</x:v>
@@ -5976,7 +6016,7 @@
         <x:v>Media\Voice\Seraphine\subzone_hogger_hill.mp3</x:v>
       </x:c>
       <x:c r="O54" s="1" t="str">
-        <x:v>No</x:v>
+        <x:v>Yes</x:v>
       </x:c>
       <x:c r="P54" s="1" t="str">
         <x:v>84I8CyTR2NsdzglhIwp3</x:v>
@@ -6005,7 +6045,9 @@
       <x:c r="X54" s="2" t="b">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="Y54" s="4"/>
+      <x:c r="Y54" s="4" t="str">
+        <x:v>Generated 2026-05-17T20:34:02.443Z (108713 bytes)</x:v>
+      </x:c>
     </x:row>
     <x:row r="55" ht="15">
       <x:c r="A55" s="1" t="str">
@@ -6042,7 +6084,7 @@
         <x:v>5.3</x:v>
       </x:c>
       <x:c r="L55" s="1" t="str">
-        <x:v>Needs generation</x:v>
+        <x:v>Audio exists</x:v>
       </x:c>
       <x:c r="M55" s="4" t="str">
         <x:v>Jasperlode is older and stranger than it looks. Mines in Azeroth almost always have opinions.</x:v>
@@ -6051,7 +6093,7 @@
         <x:v>Media\Voice\Seraphine\subzone_jasperlode_mine.mp3</x:v>
       </x:c>
       <x:c r="O55" s="1" t="str">
-        <x:v>No</x:v>
+        <x:v>Yes</x:v>
       </x:c>
       <x:c r="P55" s="1" t="str">
         <x:v>84I8CyTR2NsdzglhIwp3</x:v>
@@ -6080,7 +6122,9 @@
       <x:c r="X55" s="2" t="b">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="Y55" s="4"/>
+      <x:c r="Y55" s="4" t="str">
+        <x:v>Generated 2026-05-17T20:34:03.723Z (109549 bytes)</x:v>
+      </x:c>
     </x:row>
     <x:row r="56" ht="15">
       <x:c r="A56" s="1" t="str">
@@ -6117,7 +6161,7 @@
         <x:v>5.1</x:v>
       </x:c>
       <x:c r="L56" s="1" t="str">
-        <x:v>Needs generation</x:v>
+        <x:v>Audio exists</x:v>
       </x:c>
       <x:c r="M56" s="4" t="str">
         <x:v>Jerod's Landing is peaceful in that watch-the-water-and-check-behind-you sort of way.</x:v>
@@ -6126,7 +6170,7 @@
         <x:v>Media\Voice\Seraphine\subzone_jerods_landing.mp3</x:v>
       </x:c>
       <x:c r="O56" s="1" t="str">
-        <x:v>No</x:v>
+        <x:v>Yes</x:v>
       </x:c>
       <x:c r="P56" s="1" t="str">
         <x:v>84I8CyTR2NsdzglhIwp3</x:v>
@@ -6155,7 +6199,9 @@
       <x:c r="X56" s="2" t="b">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="Y56" s="4"/>
+      <x:c r="Y56" s="4" t="str">
+        <x:v>Generated 2026-05-17T20:34:04.920Z (84471 bytes)</x:v>
+      </x:c>
     </x:row>
     <x:row r="57" ht="15">
       <x:c r="A57" s="1" t="str">
@@ -6192,7 +6238,7 @@
         <x:v>5.6</x:v>
       </x:c>
       <x:c r="L57" s="1" t="str">
-        <x:v>Needs generation</x:v>
+        <x:v>Audio exists</x:v>
       </x:c>
       <x:c r="M57" s="4" t="str">
         <x:v>The Library Wing is dangerous to me. I always mean to read one page and lose an afternoon.</x:v>
@@ -6201,7 +6247,7 @@
         <x:v>Media\Voice\Seraphine\subzone_library_wing.mp3</x:v>
       </x:c>
       <x:c r="O57" s="1" t="str">
-        <x:v>No</x:v>
+        <x:v>Yes</x:v>
       </x:c>
       <x:c r="P57" s="1" t="str">
         <x:v>84I8CyTR2NsdzglhIwp3</x:v>
@@ -6230,7 +6276,9 @@
       <x:c r="X57" s="2" t="b">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="Y57" s="4"/>
+      <x:c r="Y57" s="4" t="str">
+        <x:v>Generated 2026-05-17T20:34:06.165Z (91577 bytes)</x:v>
+      </x:c>
     </x:row>
     <x:row r="58" ht="15">
       <x:c r="A58" s="1" t="str">
@@ -6267,7 +6315,7 @@
         <x:v>5.2</x:v>
       </x:c>
       <x:c r="L58" s="1" t="str">
-        <x:v>Needs generation</x:v>
+        <x:v>Audio exists</x:v>
       </x:c>
       <x:c r="M58" s="4" t="str">
         <x:v>The Lion's Pride Inn is warm, loud, and full of stories pretending to be rumors.</x:v>
@@ -6276,7 +6324,7 @@
         <x:v>Media\Voice\Seraphine\subzone_lions_pride_inn.mp3</x:v>
       </x:c>
       <x:c r="O58" s="1" t="str">
-        <x:v>No</x:v>
+        <x:v>Yes</x:v>
       </x:c>
       <x:c r="P58" s="1" t="str">
         <x:v>84I8CyTR2NsdzglhIwp3</x:v>
@@ -6305,7 +6353,9 @@
       <x:c r="X58" s="2" t="b">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="Y58" s="4"/>
+      <x:c r="Y58" s="4" t="str">
+        <x:v>Generated 2026-05-17T20:34:07.339Z (92413 bytes)</x:v>
+      </x:c>
     </x:row>
     <x:row r="59" ht="15">
       <x:c r="A59" s="1" t="str">
@@ -6342,7 +6392,7 @@
         <x:v>5.4</x:v>
       </x:c>
       <x:c r="L59" s="1" t="str">
-        <x:v>Needs generation</x:v>
+        <x:v>Audio exists</x:v>
       </x:c>
       <x:c r="M59" s="4" t="str">
         <x:v>Maclure Vineyards should smell like harvest and peace. Somehow even grapes find drama here.</x:v>
@@ -6351,7 +6401,7 @@
         <x:v>Media\Voice\Seraphine\subzone_maclure_vineyards.mp3</x:v>
       </x:c>
       <x:c r="O59" s="1" t="str">
-        <x:v>No</x:v>
+        <x:v>Yes</x:v>
       </x:c>
       <x:c r="P59" s="1" t="str">
         <x:v>84I8CyTR2NsdzglhIwp3</x:v>
@@ -6380,7 +6430,9 @@
       <x:c r="X59" s="2" t="b">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="Y59" s="4"/>
+      <x:c r="Y59" s="4" t="str">
+        <x:v>Generated 2026-05-17T20:34:08.543Z (98264 bytes)</x:v>
+      </x:c>
     </x:row>
     <x:row r="60" ht="15">
       <x:c r="A60" s="1" t="str">
@@ -6417,7 +6469,7 @@
         <x:v>5</x:v>
       </x:c>
       <x:c r="L60" s="1" t="str">
-        <x:v>Needs generation</x:v>
+        <x:v>Audio exists</x:v>
       </x:c>
       <x:c r="M60" s="4" t="str">
         <x:v>The Main Hall carries every anxious first step. Be gentle with the beginners you pass.</x:v>
@@ -6426,7 +6478,7 @@
         <x:v>Media\Voice\Seraphine\subzone_main_hall.mp3</x:v>
       </x:c>
       <x:c r="O60" s="1" t="str">
-        <x:v>No</x:v>
+        <x:v>Yes</x:v>
       </x:c>
       <x:c r="P60" s="1" t="str">
         <x:v>84I8CyTR2NsdzglhIwp3</x:v>
@@ -6455,7 +6507,9 @@
       <x:c r="X60" s="2" t="b">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="Y60" s="4"/>
+      <x:c r="Y60" s="4" t="str">
+        <x:v>Generated 2026-05-17T20:34:09.720Z (94502 bytes)</x:v>
+      </x:c>
     </x:row>
     <x:row r="61" ht="15">
       <x:c r="A61" s="1" t="str">
@@ -6492,7 +6546,7 @@
         <x:v>5.4</x:v>
       </x:c>
       <x:c r="L61" s="1" t="str">
-        <x:v>Needs generation</x:v>
+        <x:v>Audio exists</x:v>
       </x:c>
       <x:c r="M61" s="4" t="str">
         <x:v>Mirror Lake shows you the sky, but I suspect it keeps a few secrets beneath the reflection.</x:v>
@@ -6501,7 +6555,7 @@
         <x:v>Media\Voice\Seraphine\subzone_mirror_lake.mp3</x:v>
       </x:c>
       <x:c r="O61" s="1" t="str">
-        <x:v>No</x:v>
+        <x:v>Yes</x:v>
       </x:c>
       <x:c r="P61" s="1" t="str">
         <x:v>84I8CyTR2NsdzglhIwp3</x:v>
@@ -6530,7 +6584,9 @@
       <x:c r="X61" s="2" t="b">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="Y61" s="4"/>
+      <x:c r="Y61" s="4" t="str">
+        <x:v>Generated 2026-05-17T20:34:10.861Z (85725 bytes)</x:v>
+      </x:c>
     </x:row>
     <x:row r="62" ht="15">
       <x:c r="A62" s="1" t="str">
@@ -6567,7 +6623,7 @@
         <x:v>5.1</x:v>
       </x:c>
       <x:c r="L62" s="1" t="str">
-        <x:v>Needs generation</x:v>
+        <x:v>Audio exists</x:v>
       </x:c>
       <x:c r="M62" s="4" t="str">
         <x:v>Mirror Lake Orchard is lovely enough to make even chores feel romantic. Almost.</x:v>
@@ -6576,7 +6632,7 @@
         <x:v>Media\Voice\Seraphine\subzone_mirror_lake_orchard.mp3</x:v>
       </x:c>
       <x:c r="O62" s="1" t="str">
-        <x:v>No</x:v>
+        <x:v>Yes</x:v>
       </x:c>
       <x:c r="P62" s="1" t="str">
         <x:v>84I8CyTR2NsdzglhIwp3</x:v>
@@ -6605,7 +6661,9 @@
       <x:c r="X62" s="2" t="b">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="Y62" s="4"/>
+      <x:c r="Y62" s="4" t="str">
+        <x:v>Generated 2026-05-17T20:34:12.049Z (95338 bytes)</x:v>
+      </x:c>
     </x:row>
     <x:row r="63" ht="15">
       <x:c r="A63" s="1" t="str">
@@ -6642,7 +6700,7 @@
         <x:v>5.5</x:v>
       </x:c>
       <x:c r="L63" s="1" t="str">
-        <x:v>Needs generation</x:v>
+        <x:v>Audio exists</x:v>
       </x:c>
       <x:c r="M63" s="4" t="str">
         <x:v>Northshire Abbey has sent so many brave hearts into the world. Today, it sends you.</x:v>
@@ -6651,7 +6709,7 @@
         <x:v>Media\Voice\Seraphine\subzone_northshire_abbey.mp3</x:v>
       </x:c>
       <x:c r="O63" s="1" t="str">
-        <x:v>No</x:v>
+        <x:v>Yes</x:v>
       </x:c>
       <x:c r="P63" s="1" t="str">
         <x:v>84I8CyTR2NsdzglhIwp3</x:v>
@@ -6680,7 +6738,9 @@
       <x:c r="X63" s="2" t="b">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="Y63" s="4"/>
+      <x:c r="Y63" s="4" t="str">
+        <x:v>Generated 2026-05-17T20:34:13.218Z (86561 bytes)</x:v>
+      </x:c>
     </x:row>
     <x:row r="64" ht="15">
       <x:c r="A64" s="1" t="str">
@@ -6717,7 +6777,7 @@
         <x:v>4.8</x:v>
       </x:c>
       <x:c r="L64" s="1" t="str">
-        <x:v>Needs generation</x:v>
+        <x:v>Audio exists</x:v>
       </x:c>
       <x:c r="M64" s="4" t="str">
         <x:v>Northshire Valley is a soft beginning, but beginnings are sacred things.</x:v>
@@ -6726,7 +6786,7 @@
         <x:v>Media\Voice\Seraphine\subzone_northshire_valley.mp3</x:v>
       </x:c>
       <x:c r="O64" s="1" t="str">
-        <x:v>No</x:v>
+        <x:v>Yes</x:v>
       </x:c>
       <x:c r="P64" s="1" t="str">
         <x:v>84I8CyTR2NsdzglhIwp3</x:v>
@@ -6755,7 +6815,9 @@
       <x:c r="X64" s="2" t="b">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="Y64" s="4"/>
+      <x:c r="Y64" s="4" t="str">
+        <x:v>Generated 2026-05-17T20:34:14.436Z (79038 bytes)</x:v>
+      </x:c>
     </x:row>
     <x:row r="65" ht="15">
       <x:c r="A65" s="1" t="str">
@@ -6792,7 +6854,7 @@
         <x:v>5</x:v>
       </x:c>
       <x:c r="L65" s="1" t="str">
-        <x:v>Needs generation</x:v>
+        <x:v>Audio exists</x:v>
       </x:c>
       <x:c r="M65" s="4" t="str">
         <x:v>The Northshire Vineyards look peaceful. That is usually when someone hands you a problem.</x:v>
@@ -6801,7 +6863,7 @@
         <x:v>Media\Voice\Seraphine\subzone_northshire_vineyards.mp3</x:v>
       </x:c>
       <x:c r="O65" s="1" t="str">
-        <x:v>No</x:v>
+        <x:v>Yes</x:v>
       </x:c>
       <x:c r="P65" s="1" t="str">
         <x:v>84I8CyTR2NsdzglhIwp3</x:v>
@@ -6830,7 +6892,9 @@
       <x:c r="X65" s="2" t="b">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="Y65" s="4"/>
+      <x:c r="Y65" s="4" t="str">
+        <x:v>Generated 2026-05-17T20:34:15.586Z (84889 bytes)</x:v>
+      </x:c>
     </x:row>
     <x:row r="66" ht="15">
       <x:c r="A66" s="1" t="str">
@@ -6867,7 +6931,7 @@
         <x:v>5.8</x:v>
       </x:c>
       <x:c r="L66" s="1" t="str">
-        <x:v>Needs generation</x:v>
+        <x:v>Audio exists</x:v>
       </x:c>
       <x:c r="M66" s="4" t="str">
         <x:v>Ridgepoint Tower watches the road like an old guard who has seen too much and slept too little.</x:v>
@@ -6876,7 +6940,7 @@
         <x:v>Media\Voice\Seraphine\subzone_ridgepoint_tower.mp3</x:v>
       </x:c>
       <x:c r="O66" s="1" t="str">
-        <x:v>No</x:v>
+        <x:v>Yes</x:v>
       </x:c>
       <x:c r="P66" s="1" t="str">
         <x:v>84I8CyTR2NsdzglhIwp3</x:v>
@@ -6905,7 +6969,9 @@
       <x:c r="X66" s="2" t="b">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="Y66" s="4"/>
+      <x:c r="Y66" s="4" t="str">
+        <x:v>Generated 2026-05-17T20:34:16.827Z (103697 bytes)</x:v>
+      </x:c>
     </x:row>
     <x:row r="67" ht="15">
       <x:c r="A67" s="1" t="str">
@@ -6942,7 +7008,7 @@
         <x:v>5.5</x:v>
       </x:c>
       <x:c r="L67" s="1" t="str">
-        <x:v>Needs generation</x:v>
+        <x:v>Audio exists</x:v>
       </x:c>
       <x:c r="M67" s="4" t="str">
         <x:v>Stone Cairn Lake feels ancient around the edges. Some places remember more than people do.</x:v>
@@ -6951,7 +7017,7 @@
         <x:v>Media\Voice\Seraphine\subzone_stone_cairn_lake.mp3</x:v>
       </x:c>
       <x:c r="O67" s="1" t="str">
-        <x:v>No</x:v>
+        <x:v>Yes</x:v>
       </x:c>
       <x:c r="P67" s="1" t="str">
         <x:v>84I8CyTR2NsdzglhIwp3</x:v>
@@ -6980,7 +7046,9 @@
       <x:c r="X67" s="2" t="b">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="Y67" s="4"/>
+      <x:c r="Y67" s="4" t="str">
+        <x:v>Generated 2026-05-17T20:34:18.032Z (97010 bytes)</x:v>
+      </x:c>
     </x:row>
     <x:row r="68" ht="15">
       <x:c r="A68" s="1" t="str">
@@ -7017,7 +7085,7 @@
         <x:v>5</x:v>
       </x:c>
       <x:c r="L68" s="1" t="str">
-        <x:v>Needs generation</x:v>
+        <x:v>Audio exists</x:v>
       </x:c>
       <x:c r="M68" s="4" t="str">
         <x:v>Stonefield Farm is proof that family quarrels can be more dangerous than kobolds.</x:v>
@@ -7026,7 +7094,7 @@
         <x:v>Media\Voice\Seraphine\subzone_stonefield_farm.mp3</x:v>
       </x:c>
       <x:c r="O68" s="1" t="str">
-        <x:v>No</x:v>
+        <x:v>Yes</x:v>
       </x:c>
       <x:c r="P68" s="1" t="str">
         <x:v>84I8CyTR2NsdzglhIwp3</x:v>
@@ -7055,7 +7123,9 @@
       <x:c r="X68" s="2" t="b">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="Y68" s="4"/>
+      <x:c r="Y68" s="4" t="str">
+        <x:v>Generated 2026-05-17T20:34:19.169Z (81128 bytes)</x:v>
+      </x:c>
     </x:row>
     <x:row r="69" ht="15">
       <x:c r="A69" s="1" t="str">
@@ -7092,7 +7162,7 @@
         <x:v>5.6</x:v>
       </x:c>
       <x:c r="L69" s="1" t="str">
-        <x:v>Needs generation</x:v>
+        <x:v>Audio exists</x:v>
       </x:c>
       <x:c r="M69" s="4" t="str">
         <x:v>Stormwind rises like a promise in stone. Try not to look too dazzled. I already noticed.</x:v>
@@ -7101,7 +7171,7 @@
         <x:v>Media\Voice\Seraphine\subzone_stormwind_city.mp3</x:v>
       </x:c>
       <x:c r="O69" s="1" t="str">
-        <x:v>No</x:v>
+        <x:v>Yes</x:v>
       </x:c>
       <x:c r="P69" s="1" t="str">
         <x:v>84I8CyTR2NsdzglhIwp3</x:v>
@@ -7130,7 +7200,9 @@
       <x:c r="X69" s="2" t="b">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="Y69" s="4"/>
+      <x:c r="Y69" s="4" t="str">
+        <x:v>Generated 2026-05-17T20:34:20.375Z (99936 bytes)</x:v>
+      </x:c>
     </x:row>
     <x:row r="70" ht="27">
       <x:c r="A70" s="1" t="str">
@@ -7167,7 +7239,7 @@
         <x:v>5.8</x:v>
       </x:c>
       <x:c r="L70" s="1" t="str">
-        <x:v>Needs generation</x:v>
+        <x:v>Audio exists</x:v>
       </x:c>
       <x:c r="M70" s="4" t="str">
         <x:v>The Stormwind Gate makes every traveler feel small for a moment. Then the road asks who you will become.</x:v>
@@ -7176,7 +7248,7 @@
         <x:v>Media\Voice\Seraphine\subzone_stormwind_gate.mp3</x:v>
       </x:c>
       <x:c r="O70" s="1" t="str">
-        <x:v>No</x:v>
+        <x:v>Yes</x:v>
       </x:c>
       <x:c r="P70" s="1" t="str">
         <x:v>84I8CyTR2NsdzglhIwp3</x:v>
@@ -7205,7 +7277,9 @@
       <x:c r="X70" s="2" t="b">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="Y70" s="4"/>
+      <x:c r="Y70" s="4" t="str">
+        <x:v>Generated 2026-05-17T20:34:21.688Z (117072 bytes)</x:v>
+      </x:c>
     </x:row>
     <x:row r="71" ht="15">
       <x:c r="A71" s="1" t="str">
@@ -7242,7 +7316,7 @@
         <x:v>4.7</x:v>
       </x:c>
       <x:c r="L71" s="1" t="str">
-        <x:v>Needs generation</x:v>
+        <x:v>Audio exists</x:v>
       </x:c>
       <x:c r="M71" s="4" t="str">
         <x:v>Thunder Falls speaks louder than most nobles. I find that refreshing.</x:v>
@@ -7251,7 +7325,7 @@
         <x:v>Media\Voice\Seraphine\subzone_thunder_falls.mp3</x:v>
       </x:c>
       <x:c r="O71" s="1" t="str">
-        <x:v>No</x:v>
+        <x:v>Yes</x:v>
       </x:c>
       <x:c r="P71" s="1" t="str">
         <x:v>84I8CyTR2NsdzglhIwp3</x:v>
@@ -7280,7 +7354,9 @@
       <x:c r="X71" s="2" t="b">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="Y71" s="4"/>
+      <x:c r="Y71" s="4" t="str">
+        <x:v>Generated 2026-05-17T20:34:22.817Z (76112 bytes)</x:v>
+      </x:c>
     </x:row>
     <x:row r="72" ht="15">
       <x:c r="A72" s="1" t="str">
@@ -7317,7 +7393,7 @@
         <x:v>5.5</x:v>
       </x:c>
       <x:c r="L72" s="1" t="str">
-        <x:v>Needs generation</x:v>
+        <x:v>Audio exists</x:v>
       </x:c>
       <x:c r="M72" s="4" t="str">
         <x:v>The Tower of Azora is full of magic and questions. Please keep me from answering both at once.</x:v>
@@ -7326,7 +7402,7 @@
         <x:v>Media\Voice\Seraphine\subzone_tower_of_azora.mp3</x:v>
       </x:c>
       <x:c r="O72" s="1" t="str">
-        <x:v>No</x:v>
+        <x:v>Yes</x:v>
       </x:c>
       <x:c r="P72" s="1" t="str">
         <x:v>84I8CyTR2NsdzglhIwp3</x:v>
@@ -7355,7 +7431,9 @@
       <x:c r="X72" s="2" t="b">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="Y72" s="4"/>
+      <x:c r="Y72" s="4" t="str">
+        <x:v>Generated 2026-05-17T20:34:24.088Z (97846 bytes)</x:v>
+      </x:c>
     </x:row>
     <x:row r="73" ht="15">
       <x:c r="A73" s="1" t="str">
@@ -7392,7 +7470,7 @@
         <x:v>5.4</x:v>
       </x:c>
       <x:c r="L73" s="1" t="str">
-        <x:v>Needs generation</x:v>
+        <x:v>Audio exists</x:v>
       </x:c>
       <x:c r="M73" s="4" t="str">
         <x:v>Westbrook Garrison stands where Elwynn starts baring its teeth. The guards here know it.</x:v>
@@ -7401,7 +7479,7 @@
         <x:v>Media\Voice\Seraphine\subzone_westbrook_garrison.mp3</x:v>
       </x:c>
       <x:c r="O73" s="1" t="str">
-        <x:v>No</x:v>
+        <x:v>Yes</x:v>
       </x:c>
       <x:c r="P73" s="1" t="str">
         <x:v>84I8CyTR2NsdzglhIwp3</x:v>
@@ -7430,7 +7508,9 @@
       <x:c r="X73" s="2" t="b">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="Y73" s="4"/>
+      <x:c r="Y73" s="4" t="str">
+        <x:v>Generated 2026-05-17T20:34:25.273Z (81128 bytes)</x:v>
+      </x:c>
     </x:row>
     <x:row r="74" ht="27">
       <x:c r="A74" s="1" t="str">
@@ -21305,7 +21385,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rf4cb87c86c99493d"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rc7ea07cbc37e4acc"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -30893,7 +30973,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R89db880d8fdc4868"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R902ed552b8664ca3"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -31273,7 +31353,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R33054b0b6a8d460a"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R6d1acb7af1cf4aef"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -31710,7 +31790,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R81e931119e954a3d"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R123c00b2e2584bba"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
Standardize Maribel voice folder spelling
</commit_message>
<xml_diff>
--- a/docs/voice-line-tracker.xlsx
+++ b/docs/voice-line-tracker.xlsx
@@ -2,11 +2,11 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Standards" sheetId="1" r:id="Rfa2b080e32fa4a5c"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Voice Lines" sheetId="2" r:id="R336a06ea3188442e"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Coverage" sheetId="3" r:id="R2c5675b61216428d"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Zone Routes" sheetId="4" r:id="R34d0886061104593"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Character Profiles" sheetId="5" r:id="R3c894f8d6b444ceb"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Standards" sheetId="1" r:id="Raa7fef0d361d4c8a"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Voice Lines" sheetId="2" r:id="Raf595adabded4fd5"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Coverage" sheetId="3" r:id="R969e7b39ebed4195"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Zone Routes" sheetId="4" r:id="R53d135a0ec2e49a4"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Character Profiles" sheetId="5" r:id="R9836eee86be546ff"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -649,270 +649,6 @@
   <x:si>
     <x:t xml:space="preserve">Isle of Dorn</x:t>
   </x:si>
-  <x:si>
-    <x:t xml:space="preserve">Primary Zone / Route</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">Race</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">Role</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">Vibe</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">Physical Description</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">Outfit / Props</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">Personality</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">Voice Direction</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">Portrait Status</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">Notes</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">Elwynn Forest / Northshire - Female route</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">Human</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">Elwynn blossom mage / gentle starter companion</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">Warm, radiant, romantic, soft fantasy heroine</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">Golden-blonde hair, bright blue eyes, fair complexion, soft elegant features, flower accents, graceful mage silhouette.</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">White and gold fantasy mage dress, floral details, ornate golden staff with blossoms and glowing crystal, polished storybook look.</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">Kind, encouraging, a little teasing, protective without being stern. She makes the reincarnated hero feel welcomed into Azeroth.</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">Gentle anime heroine energy. Warm, clear, intimate, lightly playful. Smile in the voice; avoid sounding too formal or detached.</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">Done</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">Main female Elwynn route. Existing MP3 voice files are in Media\Voice\Seraphine.</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">Elwynn Forest / Northshire - Male route</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">Novice protector / village knight companion</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">Earnest, chivalrous, gentle, protective storybook knight</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">Young human knight type with soft heroic features, fair skin, light blond hair, bright noble expression, clean anime-fantasy presentation.</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">Blue, silver, and gold novice-paladin style armor or formal protector outfit; shield/holy-knight visual language; polished but still humble.</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">Sincere, brave, emotionally open, a little bashful. He believes small kindnesses matter and treats the hero like someone worth guarding.</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">Warm young knight. Gentle confidence, protective but not macho, romantic undertone as bond rises. Avoid gravelly veteran delivery.</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">Needs ElevenLabs voice files in Media\Voice\Cedric.</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">Westfall - Female route</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">Scrappy farmgirl scout / survival companion</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">Wry, loyal, sunbaked frontier energy</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">Sandy-brown hair in a messy side braid, amber eyes, sun-warmed complexion, practical posture, dust-stained traveler presence.</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">Patched traveler clothes, leather gloves, red scarf, small crossbow or dagger, worn boots, Westfall dust and field-road practicality.</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">Practical, sharp-tongued, secretly soft. She knows Westfall is hungry and dangerous, but refuses to lose hope.</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">Dry and grounded with a loyal heart underneath. Light frontier rasp or sunbaked warmth; wit first, tenderness later.</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">Voice folder is Media\Voice\Meribel to match current files.</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">Exile's Reach / Stormwind guide fallback</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">Reincarnation guide</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">Bright isekai guide, magical, welcoming</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">Placeholder guide concept: polished human mage/priestess look, soft features, luminous fantasy styling.</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">Guide-like robes or light magical outfit, gentle glow motifs, simple staff or spellbook.</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">Helpful, meta-aware, optimistic, lightly comedic. She frames the player's second life as a grand adventure.</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">Clear guide voice with cheerful fantasy narrator energy. Friendly, quick, not too breathy.</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">Partial</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">Placeholder portrait/dialogue. Needs final art and voice direction pass.</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">Orgrimmar / Valdrakken placeholder</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">Draenei</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">Cheerful field mage</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">Bubbly, curious, explosive optimism</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">Placeholder draenei mage concept: bright eyes, expressive face, energetic posture, colorful magical presence.</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">Travel mage clothes with playful magical accessories; practical enough for fieldwork, bright enough to feel whimsical.</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">Excitable, supportive, slightly chaotic. She turns danger into morale fuel.</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">Upbeat, fast smile, energetic comedic timing. Avoid making her too childish.</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">Temporary mapping; route/faction fit needs later decision.</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">Waking Shores / Hallowfall placeholder</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">Night Elf</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">Soft-spoken ranger</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">Calm, observant, gentle wilderness companion</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">Placeholder night elf ranger concept: tall, serene, moonlit features, long hair, quiet watchful presence.</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">Ranger leathers, cloak, bow or small nature charms, muted forest/night colors.</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">Patient, reflective, emotionally steady. She notices small details and makes the journey feel less lonely.</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">Soft, low, composed, intimate. Gentle reassurance rather than bubbly energy.</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">Needs final zone fit and art direction.</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">Ohn'ahran Plains / Azj-Kahet placeholder</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">Blood Elf</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">Battle senpai</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">Confident, fiery, stylish combat mentor</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">Placeholder blood elf warrior/mage concept: sharp elegant features, intense eyes, confident battle-ready posture.</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">Red/gold combat outfit, elegant armor accents, flame or blade motifs.</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">Competitive, teasing, loyal once impressed. Pushes the hero to look cool under pressure.</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">Confident anime mentor. Crisp, amused, intense in combat, warmer in bond lines.</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">Needs final art/voice.</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">Azure Span / Isle of Dorn placeholder</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">Gnome</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">Inventor companion</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">Clever, fast-talking, analytical comic relief</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">Placeholder gnome inventor concept: compact build, bright eyes, expressive eyebrows, toolbelt energy.</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">Engineer goggles, gloves, toolbelt, small gadgets, practical travel boots.</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">Brilliant, dry, easily distracted by devices. Affection shows through practical help and nervous jokes.</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">Quick, precise, witty. High mental energy without becoming shrill.</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">Thaldraszus placeholder</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">Void Elf</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">Mysterious shrine maiden</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">Mystical, soft, fate-touched, slightly eerie</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">Placeholder void elf mystic concept: pale/lavender tones, long hair, calm eyes, ethereal shrine-maiden silhouette.</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">Shrine-inspired robes, subtle void accents, charms or prayer ribbons, twilight color palette.</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">Poetic, intuitive, quietly nervous beneath the mysticism. Speaks as if she hears fate whispering nearby.</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">Soft mystical cadence. Dreamy but understandable; avoid going too monotone.</x:t>
-  </x:si>
 </x:sst>
 </file>
 
@@ -13097,7 +12833,7 @@
         <x:v>Welcome to Westfall, hero. Keep your hood low and your eyes open; hunger makes honest folk desperate.</x:v>
       </x:c>
       <x:c r="N146" s="1" t="str">
-        <x:v>Media\Voice\Meribel\zone_intro_01.mp3</x:v>
+        <x:v>Media\Voice\Maribel\zone_intro_01.mp3</x:v>
       </x:c>
       <x:c r="O146" s="1" t="str">
         <x:v>Yes</x:v>
@@ -13172,7 +12908,7 @@
         <x:v>Dust, broken fences, and trouble on every road. Still, this place is home, and I am not letting it die quiet.</x:v>
       </x:c>
       <x:c r="N147" s="1" t="str">
-        <x:v>Media\Voice\Meribel\zone_intro_02.mp3</x:v>
+        <x:v>Media\Voice\Maribel\zone_intro_02.mp3</x:v>
       </x:c>
       <x:c r="O147" s="1" t="str">
         <x:v>Yes</x:v>
@@ -13247,7 +12983,7 @@
         <x:v>Another job from someone with tired eyes. All right, hero, let us see what they need and what they are not saying.</x:v>
       </x:c>
       <x:c r="N148" s="1" t="str">
-        <x:v>Media\Voice\Meribel\quest_accept_01.mp3</x:v>
+        <x:v>Media\Voice\Maribel\quest_accept_01.mp3</x:v>
       </x:c>
       <x:c r="O148" s="1" t="str">
         <x:v>Yes</x:v>
@@ -13322,7 +13058,7 @@
         <x:v>If there is coin in it, good. If there is food in it, better. If there is trouble, well, that is usually where we come in.</x:v>
       </x:c>
       <x:c r="N149" s="1" t="str">
-        <x:v>Media\Voice\Meribel\quest_accept_02.mp3</x:v>
+        <x:v>Media\Voice\Maribel\quest_accept_02.mp3</x:v>
       </x:c>
       <x:c r="O149" s="1" t="str">
         <x:v>Yes</x:v>
@@ -13397,7 +13133,7 @@
         <x:v>Careful now. In Westfall, a simple errand can lead you straight into a knife fight.</x:v>
       </x:c>
       <x:c r="N150" s="1" t="str">
-        <x:v>Media\Voice\Meribel\quest_accept_03.mp3</x:v>
+        <x:v>Media\Voice\Maribel\quest_accept_03.mp3</x:v>
       </x:c>
       <x:c r="O150" s="1" t="str">
         <x:v>Yes</x:v>
@@ -13472,7 +13208,7 @@
         <x:v>Nice work. Quick and clean is how you live long out here.</x:v>
       </x:c>
       <x:c r="N151" s="1" t="str">
-        <x:v>Media\Voice\Meribel\kill_01.mp3</x:v>
+        <x:v>Media\Voice\Maribel\kill_01.mp3</x:v>
       </x:c>
       <x:c r="O151" s="1" t="str">
         <x:v>Yes</x:v>
@@ -13547,7 +13283,7 @@
         <x:v>That one will not be bothering the roads again. Try not to look too pleased with yourself.</x:v>
       </x:c>
       <x:c r="N152" s="1" t="str">
-        <x:v>Media\Voice\Meribel\kill_02.mp3</x:v>
+        <x:v>Media\Voice\Maribel\kill_02.mp3</x:v>
       </x:c>
       <x:c r="O152" s="1" t="str">
         <x:v>Yes</x:v>
@@ -13622,7 +13358,7 @@
         <x:v>Good hit. Westfall rewards hesitation with bruises, so do not start now.</x:v>
       </x:c>
       <x:c r="N153" s="1" t="str">
-        <x:v>Media\Voice\Meribel\kill_03.mp3</x:v>
+        <x:v>Media\Voice\Maribel\kill_03.mp3</x:v>
       </x:c>
       <x:c r="O153" s="1" t="str">
         <x:v>Yes</x:v>
@@ -13697,7 +13433,7 @@
         <x:v>Smell that? Dust, sun-baked wheat, and somebody cooking soup thin enough to see through.</x:v>
       </x:c>
       <x:c r="N154" s="1" t="str">
-        <x:v>Media\Voice\Meribel\idle_01.mp3</x:v>
+        <x:v>Media\Voice\Maribel\idle_01.mp3</x:v>
       </x:c>
       <x:c r="O154" s="1" t="str">
         <x:v>Yes</x:v>
@@ -13772,7 +13508,7 @@
         <x:v>I used to think the wind here sounded lonely. Turns out it just learned to complain from the rest of us.</x:v>
       </x:c>
       <x:c r="N155" s="1" t="str">
-        <x:v>Media\Voice\Meribel\idle_02.mp3</x:v>
+        <x:v>Media\Voice\Maribel\idle_02.mp3</x:v>
       </x:c>
       <x:c r="O155" s="1" t="str">
         <x:v>Yes</x:v>
@@ -13847,7 +13583,7 @@
         <x:v>If I tell you to duck, duck first and ask charming reincarnated-hero questions later.</x:v>
       </x:c>
       <x:c r="N156" s="1" t="str">
-        <x:v>Media\Voice\Meribel\idle_03.mp3</x:v>
+        <x:v>Media\Voice\Maribel\idle_03.mp3</x:v>
       </x:c>
       <x:c r="O156" s="1" t="str">
         <x:v>Yes</x:v>
@@ -13922,7 +13658,7 @@
         <x:v>Look at you, getting stronger. Try not to let it go to your head; I still need you able to fit through barn doors.</x:v>
       </x:c>
       <x:c r="N157" s="1" t="str">
-        <x:v>Media\Voice\Meribel\level_up_01.mp3</x:v>
+        <x:v>Media\Voice\Maribel\level_up_01.mp3</x:v>
       </x:c>
       <x:c r="O157" s="1" t="str">
         <x:v>Yes</x:v>
@@ -13997,7 +13733,7 @@
         <x:v>That is real progress. Westfall hits hard, but you are starting to hit back harder.</x:v>
       </x:c>
       <x:c r="N158" s="1" t="str">
-        <x:v>Media\Voice\Meribel\level_up_02.mp3</x:v>
+        <x:v>Media\Voice\Maribel\level_up_02.mp3</x:v>
       </x:c>
       <x:c r="O158" s="1" t="str">
         <x:v>Yes</x:v>
@@ -14072,7 +13808,7 @@
         <x:v>Maribel Dustwhisper. I know the roads, the farms, and which smiles mean trouble. Stick close, hero.</x:v>
       </x:c>
       <x:c r="N159" s="1" t="str">
-        <x:v>Media\Voice\Meribel\summon_01.mp3</x:v>
+        <x:v>Media\Voice\Maribel\summon_01.mp3</x:v>
       </x:c>
       <x:c r="O159" s="1" t="str">
         <x:v>Yes</x:v>
@@ -14147,7 +13883,7 @@
         <x:v>You have not run off yet. That either means you are brave, stubborn, or bad at reading warning signs.</x:v>
       </x:c>
       <x:c r="N160" s="1" t="str">
-        <x:v>Media\Voice\Meribel\bond_02_01.mp3</x:v>
+        <x:v>Media\Voice\Maribel\bond_02_01.mp3</x:v>
       </x:c>
       <x:c r="O160" s="1" t="str">
         <x:v>Yes</x:v>
@@ -14224,7 +13960,7 @@
         <x:v>Do not tell anyone I said this, but you are steady company. Westfall could use more of that.</x:v>
       </x:c>
       <x:c r="N161" s="1" t="str">
-        <x:v>Media\Voice\Meribel\bond_04_01.mp3</x:v>
+        <x:v>Media\Voice\Maribel\bond_04_01.mp3</x:v>
       </x:c>
       <x:c r="O161" s="1" t="str">
         <x:v>Yes</x:v>
@@ -14301,7 +14037,7 @@
         <x:v>I keep expecting you to get tired of this dust and hunger. Instead, you keep showing up. That matters.</x:v>
       </x:c>
       <x:c r="N162" s="1" t="str">
-        <x:v>Media\Voice\Meribel\bond_06_01.mp3</x:v>
+        <x:v>Media\Voice\Maribel\bond_06_01.mp3</x:v>
       </x:c>
       <x:c r="O162" s="1" t="str">
         <x:v>Yes</x:v>
@@ -14378,7 +14114,7 @@
         <x:v>If the road turns mean, I am still with you. Not because I have to be. Because I choose it.</x:v>
       </x:c>
       <x:c r="N163" s="1" t="str">
-        <x:v>Media\Voice\Meribel\bond_08_01.mp3</x:v>
+        <x:v>Media\Voice\Maribel\bond_08_01.mp3</x:v>
       </x:c>
       <x:c r="O163" s="1" t="str">
         <x:v>Yes</x:v>
@@ -14455,7 +14191,7 @@
         <x:v>Westfall taught me not to count on miracles. Then you arrived, impossible and smiling, and ruined my good cynicism.</x:v>
       </x:c>
       <x:c r="N164" s="1" t="str">
-        <x:v>Media\Voice\Meribel\bond_10_01.mp3</x:v>
+        <x:v>Media\Voice\Maribel\bond_10_01.mp3</x:v>
       </x:c>
       <x:c r="O164" s="1" t="str">
         <x:v>Yes</x:v>
@@ -14532,7 +14268,7 @@
         <x:v>Huh. So that is the way the wind is blowing. All right, hero. I am listening.</x:v>
       </x:c>
       <x:c r="N165" s="1" t="str">
-        <x:v>Media\Voice\Meribel\romance_02_01.mp3</x:v>
+        <x:v>Media\Voice\Maribel\romance_02_01.mp3</x:v>
       </x:c>
       <x:c r="O165" s="1" t="str">
         <x:v>Yes</x:v>
@@ -14609,7 +14345,7 @@
         <x:v>You are getting under my guard, and I am annoyed to report I do not hate it.</x:v>
       </x:c>
       <x:c r="N166" s="1" t="str">
-        <x:v>Media\Voice\Meribel\romance_04_01.mp3</x:v>
+        <x:v>Media\Voice\Maribel\romance_04_01.mp3</x:v>
       </x:c>
       <x:c r="O166" s="1" t="str">
         <x:v>Yes</x:v>
@@ -14686,7 +14422,7 @@
         <x:v>I keep saving the better half of my rations for you. If that is not romance in Westfall, I do not know what is.</x:v>
       </x:c>
       <x:c r="N167" s="1" t="str">
-        <x:v>Media\Voice\Meribel\romance_06_01.mp3</x:v>
+        <x:v>Media\Voice\Maribel\romance_06_01.mp3</x:v>
       </x:c>
       <x:c r="O167" s="1" t="str">
         <x:v>Yes</x:v>
@@ -14763,7 +14499,7 @@
         <x:v>Do not make me say something soft in all this dust. Fine. I want you here. I want us.</x:v>
       </x:c>
       <x:c r="N168" s="1" t="str">
-        <x:v>Media\Voice\Meribel\romance_08_01.mp3</x:v>
+        <x:v>Media\Voice\Maribel\romance_08_01.mp3</x:v>
       </x:c>
       <x:c r="O168" s="1" t="str">
         <x:v>Yes</x:v>
@@ -14840,7 +14576,7 @@
         <x:v>Westfall can keep its hard roads. I have found my reason to keep walking them, and it is you.</x:v>
       </x:c>
       <x:c r="N169" s="1" t="str">
-        <x:v>Media\Voice\Meribel\romance_10_01.mp3</x:v>
+        <x:v>Media\Voice\Maribel\romance_10_01.mp3</x:v>
       </x:c>
       <x:c r="O169" s="1" t="str">
         <x:v>Yes</x:v>
@@ -14917,7 +14653,7 @@
         <x:v>Easy there. I am not saying no. I am saying earn a little more trust before you come knocking on that door.</x:v>
       </x:c>
       <x:c r="N170" s="1" t="str">
-        <x:v>Media\Voice\Meribel\romance_not_ready_01.mp3</x:v>
+        <x:v>Media\Voice\Maribel\romance_not_ready_01.mp3</x:v>
       </x:c>
       <x:c r="O170" s="1" t="str">
         <x:v>Yes</x:v>
@@ -14994,7 +14730,7 @@
         <x:v>You already got that piece of my heart. Greedy thing, aren't you?</x:v>
       </x:c>
       <x:c r="N171" s="1" t="str">
-        <x:v>Media\Voice\Meribel\romance_repeat_01.mp3</x:v>
+        <x:v>Media\Voice\Maribel\romance_repeat_01.mp3</x:v>
       </x:c>
       <x:c r="O171" s="1" t="str">
         <x:v>Yes</x:v>
@@ -15071,7 +14807,7 @@
         <x:v>Yeah. All right. I can do that. Give me a minute, then we keep moving.</x:v>
       </x:c>
       <x:c r="N172" s="1" t="str">
-        <x:v>Media\Voice\Meribel\romance_stop_01.mp3</x:v>
+        <x:v>Media\Voice\Maribel\romance_stop_01.mp3</x:v>
       </x:c>
       <x:c r="O172" s="1" t="str">
         <x:v>Yes</x:v>
@@ -15148,7 +14884,7 @@
         <x:v>That is one less problem chewing on this place. Not bad, hero.</x:v>
       </x:c>
       <x:c r="N173" s="1" t="str">
-        <x:v>Media\Voice\Meribel\quest_complete_01.mp3</x:v>
+        <x:v>Media\Voice\Maribel\quest_complete_01.mp3</x:v>
       </x:c>
       <x:c r="O173" s="1" t="str">
         <x:v>Yes</x:v>
@@ -15225,7 +14961,7 @@
         <x:v>Done and done. Westfall does not hand out easy wins, so take this one.</x:v>
       </x:c>
       <x:c r="N174" s="1" t="str">
-        <x:v>Media\Voice\Meribel\quest_complete_02.mp3</x:v>
+        <x:v>Media\Voice\Maribel\quest_complete_02.mp3</x:v>
       </x:c>
       <x:c r="O174" s="1" t="str">
         <x:v>Yes</x:v>
@@ -15302,7 +15038,7 @@
         <x:v>You helped someone who needed it. Out here, that is worth more than shiny speeches.</x:v>
       </x:c>
       <x:c r="N175" s="1" t="str">
-        <x:v>Media\Voice\Meribel\quest_complete_03.mp3</x:v>
+        <x:v>Media\Voice\Maribel\quest_complete_03.mp3</x:v>
       </x:c>
       <x:c r="O175" s="1" t="str">
         <x:v>Yes</x:v>
@@ -15379,7 +15115,7 @@
         <x:v>You are getting quicker. I might stop pretending to be surprised.</x:v>
       </x:c>
       <x:c r="N176" s="1" t="str">
-        <x:v>Media\Voice\Meribel\bond_kill_02.mp3</x:v>
+        <x:v>Media\Voice\Maribel\bond_kill_02.mp3</x:v>
       </x:c>
       <x:c r="O176" s="1" t="str">
         <x:v>Yes</x:v>
@@ -15456,7 +15192,7 @@
         <x:v>Good. You watched the flank this time. I like a hero who learns.</x:v>
       </x:c>
       <x:c r="N177" s="1" t="str">
-        <x:v>Media\Voice\Meribel\bond_kill_04.mp3</x:v>
+        <x:v>Media\Voice\Maribel\bond_kill_04.mp3</x:v>
       </x:c>
       <x:c r="O177" s="1" t="str">
         <x:v>Yes</x:v>
@@ -15533,7 +15269,7 @@
         <x:v>Hah. We are getting dangerous together. Westfall should worry less about us and more about them.</x:v>
       </x:c>
       <x:c r="N178" s="1" t="str">
-        <x:v>Media\Voice\Meribel\bond_kill_06.mp3</x:v>
+        <x:v>Media\Voice\Maribel\bond_kill_06.mp3</x:v>
       </x:c>
       <x:c r="O178" s="1" t="str">
         <x:v>Yes</x:v>
@@ -15610,7 +15346,7 @@
         <x:v>Nobody corners you while I am here. I have gotten attached to keeping you breathing.</x:v>
       </x:c>
       <x:c r="N179" s="1" t="str">
-        <x:v>Media\Voice\Meribel\bond_kill_08.mp3</x:v>
+        <x:v>Media\Voice\Maribel\bond_kill_08.mp3</x:v>
       </x:c>
       <x:c r="O179" s="1" t="str">
         <x:v>Yes</x:v>
@@ -15687,7 +15423,7 @@
         <x:v>That is my hero. Do not grin like that. Fine, grin a little.</x:v>
       </x:c>
       <x:c r="N180" s="1" t="str">
-        <x:v>Media\Voice\Meribel\bond_kill_10.mp3</x:v>
+        <x:v>Media\Voice\Maribel\bond_kill_10.mp3</x:v>
       </x:c>
       <x:c r="O180" s="1" t="str">
         <x:v>Yes</x:v>
@@ -15764,7 +15500,7 @@
         <x:v>You are still here. Either you are loyal, stubborn, or lost. I can work with all three.</x:v>
       </x:c>
       <x:c r="N181" s="1" t="str">
-        <x:v>Media\Voice\Meribel\bond_idle_01.mp3</x:v>
+        <x:v>Media\Voice\Maribel\bond_idle_01.mp3</x:v>
       </x:c>
       <x:c r="O181" s="1" t="str">
         <x:v>Yes</x:v>
@@ -15841,7 +15577,7 @@
         <x:v>I started packing extra food without thinking about it. Do not make that weird.</x:v>
       </x:c>
       <x:c r="N182" s="1" t="str">
-        <x:v>Media\Voice\Meribel\bond_idle_03.mp3</x:v>
+        <x:v>Media\Voice\Maribel\bond_idle_03.mp3</x:v>
       </x:c>
       <x:c r="O182" s="1" t="str">
         <x:v>Yes</x:v>
@@ -15918,7 +15654,7 @@
         <x:v>Westfall feels less empty when you are walking beside me. That is all I am saying.</x:v>
       </x:c>
       <x:c r="N183" s="1" t="str">
-        <x:v>Media\Voice\Meribel\bond_idle_05.mp3</x:v>
+        <x:v>Media\Voice\Maribel\bond_idle_05.mp3</x:v>
       </x:c>
       <x:c r="O183" s="1" t="str">
         <x:v>Yes</x:v>
@@ -15995,7 +15731,7 @@
         <x:v>If anyone asks, I am keeping you alive for practical reasons. Mostly.</x:v>
       </x:c>
       <x:c r="N184" s="1" t="str">
-        <x:v>Media\Voice\Meribel\bond_idle_07.mp3</x:v>
+        <x:v>Media\Voice\Maribel\bond_idle_07.mp3</x:v>
       </x:c>
       <x:c r="O184" s="1" t="str">
         <x:v>Yes</x:v>
@@ -16072,7 +15808,7 @@
         <x:v>You have become part of how I picture the road ahead. Annoying, but true.</x:v>
       </x:c>
       <x:c r="N185" s="1" t="str">
-        <x:v>Media\Voice\Meribel\bond_idle_09.mp3</x:v>
+        <x:v>Media\Voice\Maribel\bond_idle_09.mp3</x:v>
       </x:c>
       <x:c r="O185" s="1" t="str">
         <x:v>Yes</x:v>
@@ -16149,7 +15885,7 @@
         <x:v>Hey! Eyes open, hero. Bleed later, move now!</x:v>
       </x:c>
       <x:c r="N186" s="1" t="str">
-        <x:v>Media\Voice\Meribel\low_health_01.mp3</x:v>
+        <x:v>Media\Voice\Maribel\low_health_01.mp3</x:v>
       </x:c>
       <x:c r="O186" s="1" t="str">
         <x:v>Yes</x:v>
@@ -16226,7 +15962,7 @@
         <x:v>No. No, get back up. Westfall does not get to take you from me too.</x:v>
       </x:c>
       <x:c r="N187" s="1" t="str">
-        <x:v>Media\Voice\Meribel\death_01.mp3</x:v>
+        <x:v>Media\Voice\Maribel\death_01.mp3</x:v>
       </x:c>
       <x:c r="O187" s="1" t="str">
         <x:v>Yes</x:v>
@@ -16303,7 +16039,7 @@
         <x:v>Alexston Farmstead used to mean work and supper. Now it mostly means watching your back.</x:v>
       </x:c>
       <x:c r="N188" s="1" t="str">
-        <x:v>Media\Voice\Meribel\subzone_alexston_farmstead.mp3</x:v>
+        <x:v>Media\Voice\Maribel\subzone_alexston_farmstead.mp3</x:v>
       </x:c>
       <x:c r="O188" s="1" t="str">
         <x:v>Yes</x:v>
@@ -16380,7 +16116,7 @@
         <x:v>The Dagger Hills earned that name. Keep low and do not trust a ridge line.</x:v>
       </x:c>
       <x:c r="N189" s="1" t="str">
-        <x:v>Media\Voice\Meribel\subzone_dagger_hills.mp3</x:v>
+        <x:v>Media\Voice\Maribel\subzone_dagger_hills.mp3</x:v>
       </x:c>
       <x:c r="O189" s="1" t="str">
         <x:v>Yes</x:v>
@@ -16457,7 +16193,7 @@
         <x:v>Dawning Wood Catacombs. Great. Nothing says safe like stairs into old bones.</x:v>
       </x:c>
       <x:c r="N190" s="1" t="str">
-        <x:v>Media\Voice\Meribel\subzone_dawning_wood_catacombs.mp3</x:v>
+        <x:v>Media\Voice\Maribel\subzone_dawning_wood_catacombs.mp3</x:v>
       </x:c>
       <x:c r="O190" s="1" t="str">
         <x:v>Yes</x:v>
@@ -16534,7 +16270,7 @@
         <x:v>Dead Acre is what happens when a place runs out of chances. We keep moving.</x:v>
       </x:c>
       <x:c r="N191" s="1" t="str">
-        <x:v>Media\Voice\Meribel\subzone_dead_acre.mp3</x:v>
+        <x:v>Media\Voice\Maribel\subzone_dead_acre.mp3</x:v>
       </x:c>
       <x:c r="O191" s="1" t="str">
         <x:v>Yes</x:v>
@@ -16611,7 +16347,7 @@
         <x:v>Demont's Place has the kind of quiet that makes my fingers look for a blade.</x:v>
       </x:c>
       <x:c r="N192" s="1" t="str">
-        <x:v>Media\Voice\Meribel\subzone_demonts_place.mp3</x:v>
+        <x:v>Media\Voice\Maribel\subzone_demonts_place.mp3</x:v>
       </x:c>
       <x:c r="O192" s="1" t="str">
         <x:v>Yes</x:v>
@@ -16688,7 +16424,7 @@
         <x:v>The Dust Plains get into your boots, your throat, and eventually your mood.</x:v>
       </x:c>
       <x:c r="N193" s="1" t="str">
-        <x:v>Media\Voice\Meribel\subzone_dust_plains.mp3</x:v>
+        <x:v>Media\Voice\Maribel\subzone_dust_plains.mp3</x:v>
       </x:c>
       <x:c r="O193" s="1" t="str">
         <x:v>Yes</x:v>
@@ -16765,7 +16501,7 @@
         <x:v>Furlbrow's farm should have been simple. In Westfall, even pumpkins come with grief.</x:v>
       </x:c>
       <x:c r="N194" s="1" t="str">
-        <x:v>Media\Voice\Meribel\subzone_furlbrows_pumpkin_farm.mp3</x:v>
+        <x:v>Media\Voice\Maribel\subzone_furlbrows_pumpkin_farm.mp3</x:v>
       </x:c>
       <x:c r="O194" s="1" t="str">
         <x:v>Yes</x:v>
@@ -16842,7 +16578,7 @@
         <x:v>Gold Coast Quarry is all hard edges and harder work. Easy place to miss trouble until it echoes.</x:v>
       </x:c>
       <x:c r="N195" s="1" t="str">
-        <x:v>Media\Voice\Meribel\subzone_gold_coast_quarry.mp3</x:v>
+        <x:v>Media\Voice\Maribel\subzone_gold_coast_quarry.mp3</x:v>
       </x:c>
       <x:c r="O195" s="1" t="str">
         <x:v>Yes</x:v>
@@ -16919,7 +16655,7 @@
         <x:v>The Jansen Stead still feels like someone left in a hurry and hoped to come back.</x:v>
       </x:c>
       <x:c r="N196" s="1" t="str">
-        <x:v>Media\Voice\Meribel\subzone_jansen_stead.mp3</x:v>
+        <x:v>Media\Voice\Maribel\subzone_jansen_stead.mp3</x:v>
       </x:c>
       <x:c r="O196" s="1" t="str">
         <x:v>Yes</x:v>
@@ -16996,7 +16732,7 @@
         <x:v>Jangolode Mine. If the tunnels start sounding too quiet, that is your warning.</x:v>
       </x:c>
       <x:c r="N197" s="1" t="str">
-        <x:v>Media\Voice\Meribel\subzone_jangolode_mine.mp3</x:v>
+        <x:v>Media\Voice\Maribel\subzone_jangolode_mine.mp3</x:v>
       </x:c>
       <x:c r="O197" s="1" t="str">
         <x:v>Yes</x:v>
@@ -17073,7 +16809,7 @@
         <x:v>The Molsen Farm has seen better harvests. Most of Westfall has.</x:v>
       </x:c>
       <x:c r="N198" s="1" t="str">
-        <x:v>Media\Voice\Meribel\subzone_molsen_farm.mp3</x:v>
+        <x:v>Media\Voice\Maribel\subzone_molsen_farm.mp3</x:v>
       </x:c>
       <x:c r="O198" s="1" t="str">
         <x:v>Yes</x:v>
@@ -17150,7 +16886,7 @@
         <x:v>Moonbrook has too many windows and not enough honest faces. Stay sharp.</x:v>
       </x:c>
       <x:c r="N199" s="1" t="str">
-        <x:v>Media\Voice\Meribel\subzone_moonbrook.mp3</x:v>
+        <x:v>Media\Voice\Maribel\subzone_moonbrook.mp3</x:v>
       </x:c>
       <x:c r="O199" s="1" t="str">
         <x:v>Yes</x:v>
@@ -17227,7 +16963,7 @@
         <x:v>The Raging Chasm looks like the land finally got tired of holding itself together.</x:v>
       </x:c>
       <x:c r="N200" s="1" t="str">
-        <x:v>Media\Voice\Meribel\subzone_raging_chasm.mp3</x:v>
+        <x:v>Media\Voice\Maribel\subzone_raging_chasm.mp3</x:v>
       </x:c>
       <x:c r="O200" s="1" t="str">
         <x:v>Yes</x:v>
@@ -17304,7 +17040,7 @@
         <x:v>Saldean's Farm still fights to feed people. That makes it worth protecting.</x:v>
       </x:c>
       <x:c r="N201" s="1" t="str">
-        <x:v>Media\Voice\Meribel\subzone_saldeans_farm.mp3</x:v>
+        <x:v>Media\Voice\Maribel\subzone_saldeans_farm.mp3</x:v>
       </x:c>
       <x:c r="O201" s="1" t="str">
         <x:v>Yes</x:v>
@@ -17381,7 +17117,7 @@
         <x:v>Sentinel Hill is where Westfall tries to stand up straight, even with empty pockets.</x:v>
       </x:c>
       <x:c r="N202" s="1" t="str">
-        <x:v>Media\Voice\Meribel\subzone_sentinel_hill.mp3</x:v>
+        <x:v>Media\Voice\Maribel\subzone_sentinel_hill.mp3</x:v>
       </x:c>
       <x:c r="O202" s="1" t="str">
         <x:v>Yes</x:v>
@@ -17458,7 +17194,7 @@
         <x:v>The Shattered Strand is all wreckage and salt wind. Watch where the tide hides teeth.</x:v>
       </x:c>
       <x:c r="N203" s="1" t="str">
-        <x:v>Media\Voice\Meribel\subzone_shattered_strand.mp3</x:v>
+        <x:v>Media\Voice\Maribel\subzone_shattered_strand.mp3</x:v>
       </x:c>
       <x:c r="O203" s="1" t="str">
         <x:v>Yes</x:v>
@@ -17535,7 +17271,7 @@
         <x:v>The Sludge Fields smell like every bad decision someone tried to bury.</x:v>
       </x:c>
       <x:c r="N204" s="1" t="str">
-        <x:v>Media\Voice\Meribel\subzone_sludge_fields.mp3</x:v>
+        <x:v>Media\Voice\Maribel\subzone_sludge_fields.mp3</x:v>
       </x:c>
       <x:c r="O204" s="1" t="str">
         <x:v>Yes</x:v>
@@ -17612,7 +17348,7 @@
         <x:v>The Writhing Haunt is exactly as welcoming as it sounds. Do not wander.</x:v>
       </x:c>
       <x:c r="N205" s="1" t="str">
-        <x:v>Media\Voice\Meribel\subzone_writhing_haunt.mp3</x:v>
+        <x:v>Media\Voice\Maribel\subzone_writhing_haunt.mp3</x:v>
       </x:c>
       <x:c r="O205" s="1" t="str">
         <x:v>Yes</x:v>
@@ -17689,7 +17425,7 @@
         <x:v>Westfall Lighthouse keeps shining even when nobody thanks it. I respect that.</x:v>
       </x:c>
       <x:c r="N206" s="1" t="str">
-        <x:v>Media\Voice\Meribel\subzone_westfall_lighthouse.mp3</x:v>
+        <x:v>Media\Voice\Maribel\subzone_westfall_lighthouse.mp3</x:v>
       </x:c>
       <x:c r="O206" s="1" t="str">
         <x:v>Yes</x:v>
@@ -21889,7 +21625,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rbce525a00c2b48b2"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R20daf0d4b2b24b7b"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -31477,7 +31213,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rcd89126e95174cd9"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rff7ce3509bd840a1"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -31857,7 +31593,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R766ae55410304c89"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Ra0b3133c859841ed"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -31882,419 +31618,419 @@
   </x:cols>
   <x:sheetData>
     <x:row r="1" ht="15">
-      <x:c r="A1" s="3" t="s">
-        <x:v>114</x:v>
-      </x:c>
-      <x:c r="B1" s="3" t="s">
-        <x:v>115</x:v>
-      </x:c>
-      <x:c r="C1" s="3" t="s">
-        <x:v>212</x:v>
-      </x:c>
-      <x:c r="D1" s="3" t="s">
-        <x:v>213</x:v>
-      </x:c>
-      <x:c r="E1" s="3" t="s">
-        <x:v>116</x:v>
-      </x:c>
-      <x:c r="F1" s="3" t="s">
-        <x:v>214</x:v>
-      </x:c>
-      <x:c r="G1" s="3" t="s">
-        <x:v>215</x:v>
-      </x:c>
-      <x:c r="H1" s="3" t="s">
-        <x:v>216</x:v>
-      </x:c>
-      <x:c r="I1" s="3" t="s">
-        <x:v>217</x:v>
-      </x:c>
-      <x:c r="J1" s="3" t="s">
-        <x:v>218</x:v>
-      </x:c>
-      <x:c r="K1" s="3" t="s">
-        <x:v>219</x:v>
-      </x:c>
-      <x:c r="L1" s="3" t="s">
-        <x:v>220</x:v>
-      </x:c>
-      <x:c r="M1" s="3" t="s">
-        <x:v>221</x:v>
+      <x:c r="A1" s="3" t="str">
+        <x:v>Companion ID</x:v>
+      </x:c>
+      <x:c r="B1" s="3" t="str">
+        <x:v>Character</x:v>
+      </x:c>
+      <x:c r="C1" s="3" t="str">
+        <x:v>Primary Zone / Route</x:v>
+      </x:c>
+      <x:c r="D1" s="3" t="str">
+        <x:v>Race</x:v>
+      </x:c>
+      <x:c r="E1" s="3" t="str">
+        <x:v>Gender</x:v>
+      </x:c>
+      <x:c r="F1" s="3" t="str">
+        <x:v>Role</x:v>
+      </x:c>
+      <x:c r="G1" s="3" t="str">
+        <x:v>Vibe</x:v>
+      </x:c>
+      <x:c r="H1" s="3" t="str">
+        <x:v>Physical Description</x:v>
+      </x:c>
+      <x:c r="I1" s="3" t="str">
+        <x:v>Outfit / Props</x:v>
+      </x:c>
+      <x:c r="J1" s="3" t="str">
+        <x:v>Personality</x:v>
+      </x:c>
+      <x:c r="K1" s="3" t="str">
+        <x:v>Voice Direction</x:v>
+      </x:c>
+      <x:c r="L1" s="3" t="str">
+        <x:v>Portrait Status</x:v>
+      </x:c>
+      <x:c r="M1" s="3" t="str">
+        <x:v>Notes</x:v>
       </x:c>
     </x:row>
     <x:row r="2" ht="27">
-      <x:c r="A2" s="1" t="s">
-        <x:v>120</x:v>
-      </x:c>
-      <x:c r="B2" s="1" t="s">
-        <x:v>121</x:v>
-      </x:c>
-      <x:c r="C2" s="1" t="s">
-        <x:v>222</x:v>
-      </x:c>
-      <x:c r="D2" s="1" t="s">
-        <x:v>223</x:v>
-      </x:c>
-      <x:c r="E2" s="1" t="s">
-        <x:v>122</x:v>
-      </x:c>
-      <x:c r="F2" s="1" t="s">
-        <x:v>224</x:v>
-      </x:c>
-      <x:c r="G2" s="1" t="s">
-        <x:v>225</x:v>
-      </x:c>
-      <x:c r="H2" s="4" t="s">
-        <x:v>226</x:v>
-      </x:c>
-      <x:c r="I2" s="4" t="s">
-        <x:v>227</x:v>
-      </x:c>
-      <x:c r="J2" s="4" t="s">
-        <x:v>228</x:v>
-      </x:c>
-      <x:c r="K2" s="4" t="s">
-        <x:v>229</x:v>
-      </x:c>
-      <x:c r="L2" s="1" t="s">
-        <x:v>230</x:v>
-      </x:c>
-      <x:c r="M2" s="4" t="s">
-        <x:v>231</x:v>
+      <x:c r="A2" s="1" t="str">
+        <x:v>seraphine</x:v>
+      </x:c>
+      <x:c r="B2" s="1" t="str">
+        <x:v>Seraphine Applebrook</x:v>
+      </x:c>
+      <x:c r="C2" s="1" t="str">
+        <x:v>Elwynn Forest / Northshire - Female route</x:v>
+      </x:c>
+      <x:c r="D2" s="1" t="str">
+        <x:v>Human</x:v>
+      </x:c>
+      <x:c r="E2" s="1" t="str">
+        <x:v>Female</x:v>
+      </x:c>
+      <x:c r="F2" s="1" t="str">
+        <x:v>Elwynn blossom mage / gentle starter companion</x:v>
+      </x:c>
+      <x:c r="G2" s="1" t="str">
+        <x:v>Warm, radiant, romantic, soft fantasy heroine</x:v>
+      </x:c>
+      <x:c r="H2" s="4" t="str">
+        <x:v>Golden-blonde hair, bright blue eyes, fair complexion, soft elegant features, flower accents, graceful mage silhouette.</x:v>
+      </x:c>
+      <x:c r="I2" s="4" t="str">
+        <x:v>White and gold fantasy mage dress, floral details, ornate golden staff with blossoms and glowing crystal, polished storybook look.</x:v>
+      </x:c>
+      <x:c r="J2" s="4" t="str">
+        <x:v>Kind, encouraging, a little teasing, protective without being stern. She makes the reincarnated hero feel welcomed into Azeroth.</x:v>
+      </x:c>
+      <x:c r="K2" s="4" t="str">
+        <x:v>Gentle anime heroine energy. Warm, clear, intimate, lightly playful. Smile in the voice; avoid sounding too formal or detached.</x:v>
+      </x:c>
+      <x:c r="L2" s="1" t="str">
+        <x:v>Done</x:v>
+      </x:c>
+      <x:c r="M2" s="4" t="str">
+        <x:v>Main female Elwynn route. Existing MP3 voice files are in Media\Voice\Seraphine.</x:v>
       </x:c>
     </x:row>
     <x:row r="3" ht="27">
-      <x:c r="A3" s="1" t="s">
-        <x:v>154</x:v>
-      </x:c>
-      <x:c r="B3" s="1" t="s">
-        <x:v>155</x:v>
-      </x:c>
-      <x:c r="C3" s="1" t="s">
-        <x:v>232</x:v>
-      </x:c>
-      <x:c r="D3" s="1" t="s">
-        <x:v>223</x:v>
-      </x:c>
-      <x:c r="E3" s="1" t="s">
-        <x:v>156</x:v>
-      </x:c>
-      <x:c r="F3" s="1" t="s">
-        <x:v>233</x:v>
-      </x:c>
-      <x:c r="G3" s="1" t="s">
-        <x:v>234</x:v>
-      </x:c>
-      <x:c r="H3" s="4" t="s">
-        <x:v>235</x:v>
-      </x:c>
-      <x:c r="I3" s="4" t="s">
-        <x:v>236</x:v>
-      </x:c>
-      <x:c r="J3" s="4" t="s">
-        <x:v>237</x:v>
-      </x:c>
-      <x:c r="K3" s="4" t="s">
-        <x:v>238</x:v>
-      </x:c>
-      <x:c r="L3" s="1" t="s">
-        <x:v>230</x:v>
-      </x:c>
-      <x:c r="M3" s="4" t="s">
-        <x:v>239</x:v>
+      <x:c r="A3" s="1" t="str">
+        <x:v>cedric</x:v>
+      </x:c>
+      <x:c r="B3" s="1" t="str">
+        <x:v>Cedric Applebrook</x:v>
+      </x:c>
+      <x:c r="C3" s="1" t="str">
+        <x:v>Elwynn Forest / Northshire - Male route</x:v>
+      </x:c>
+      <x:c r="D3" s="1" t="str">
+        <x:v>Human</x:v>
+      </x:c>
+      <x:c r="E3" s="1" t="str">
+        <x:v>Male</x:v>
+      </x:c>
+      <x:c r="F3" s="1" t="str">
+        <x:v>Novice protector / village knight companion</x:v>
+      </x:c>
+      <x:c r="G3" s="1" t="str">
+        <x:v>Earnest, chivalrous, gentle, protective storybook knight</x:v>
+      </x:c>
+      <x:c r="H3" s="4" t="str">
+        <x:v>Young human knight type with soft heroic features, fair skin, light blond hair, bright noble expression, clean anime-fantasy presentation.</x:v>
+      </x:c>
+      <x:c r="I3" s="4" t="str">
+        <x:v>Blue, silver, and gold novice-paladin style armor or formal protector outfit; shield/holy-knight visual language; polished but still humble.</x:v>
+      </x:c>
+      <x:c r="J3" s="4" t="str">
+        <x:v>Sincere, brave, emotionally open, a little bashful. He believes small kindnesses matter and treats the hero like someone worth guarding.</x:v>
+      </x:c>
+      <x:c r="K3" s="4" t="str">
+        <x:v>Warm young knight. Gentle confidence, protective but not macho, romantic undertone as bond rises. Avoid gravelly veteran delivery.</x:v>
+      </x:c>
+      <x:c r="L3" s="1" t="str">
+        <x:v>Done</x:v>
+      </x:c>
+      <x:c r="M3" s="4" t="str">
+        <x:v>Needs ElevenLabs voice files in Media\Voice\Cedric.</x:v>
       </x:c>
     </x:row>
     <x:row r="4" ht="27">
-      <x:c r="A4" s="1" t="s">
-        <x:v>157</x:v>
-      </x:c>
-      <x:c r="B4" s="1" t="s">
-        <x:v>158</x:v>
-      </x:c>
-      <x:c r="C4" s="1" t="s">
-        <x:v>240</x:v>
-      </x:c>
-      <x:c r="D4" s="1" t="s">
-        <x:v>223</x:v>
-      </x:c>
-      <x:c r="E4" s="1" t="s">
-        <x:v>122</x:v>
-      </x:c>
-      <x:c r="F4" s="1" t="s">
-        <x:v>241</x:v>
-      </x:c>
-      <x:c r="G4" s="1" t="s">
-        <x:v>242</x:v>
-      </x:c>
-      <x:c r="H4" s="4" t="s">
-        <x:v>243</x:v>
-      </x:c>
-      <x:c r="I4" s="4" t="s">
-        <x:v>244</x:v>
-      </x:c>
-      <x:c r="J4" s="4" t="s">
-        <x:v>245</x:v>
-      </x:c>
-      <x:c r="K4" s="4" t="s">
-        <x:v>246</x:v>
-      </x:c>
-      <x:c r="L4" s="1" t="s">
-        <x:v>230</x:v>
-      </x:c>
-      <x:c r="M4" s="4" t="s">
-        <x:v>247</x:v>
+      <x:c r="A4" s="1" t="str">
+        <x:v>maribel</x:v>
+      </x:c>
+      <x:c r="B4" s="1" t="str">
+        <x:v>Maribel Dustwhisper</x:v>
+      </x:c>
+      <x:c r="C4" s="1" t="str">
+        <x:v>Westfall - Female route</x:v>
+      </x:c>
+      <x:c r="D4" s="1" t="str">
+        <x:v>Human</x:v>
+      </x:c>
+      <x:c r="E4" s="1" t="str">
+        <x:v>Female</x:v>
+      </x:c>
+      <x:c r="F4" s="1" t="str">
+        <x:v>Scrappy farmgirl scout / survival companion</x:v>
+      </x:c>
+      <x:c r="G4" s="1" t="str">
+        <x:v>Wry, loyal, sunbaked frontier energy</x:v>
+      </x:c>
+      <x:c r="H4" s="4" t="str">
+        <x:v>Sandy-brown hair in a messy side braid, amber eyes, sun-warmed complexion, practical posture, dust-stained traveler presence.</x:v>
+      </x:c>
+      <x:c r="I4" s="4" t="str">
+        <x:v>Patched traveler clothes, leather gloves, red scarf, small crossbow or dagger, worn boots, Westfall dust and field-road practicality.</x:v>
+      </x:c>
+      <x:c r="J4" s="4" t="str">
+        <x:v>Practical, sharp-tongued, secretly soft. She knows Westfall is hungry and dangerous, but refuses to lose hope.</x:v>
+      </x:c>
+      <x:c r="K4" s="4" t="str">
+        <x:v>Dry and grounded with a loyal heart underneath. Light frontier rasp or sunbaked warmth; wit first, tenderness later.</x:v>
+      </x:c>
+      <x:c r="L4" s="1" t="str">
+        <x:v>Done</x:v>
+      </x:c>
+      <x:c r="M4" s="4" t="str">
+        <x:v>Voice folder is Media\Voice\Maribel to match current files.</x:v>
       </x:c>
     </x:row>
     <x:row r="5" ht="27">
-      <x:c r="A5" s="1" t="s">
-        <x:v>178</x:v>
-      </x:c>
-      <x:c r="B5" s="1" t="s">
-        <x:v>179</x:v>
-      </x:c>
-      <x:c r="C5" s="1" t="s">
-        <x:v>248</x:v>
-      </x:c>
-      <x:c r="D5" s="1" t="s">
-        <x:v>223</x:v>
-      </x:c>
-      <x:c r="E5" s="1" t="s">
-        <x:v>122</x:v>
-      </x:c>
-      <x:c r="F5" s="1" t="s">
-        <x:v>249</x:v>
-      </x:c>
-      <x:c r="G5" s="1" t="s">
-        <x:v>250</x:v>
-      </x:c>
-      <x:c r="H5" s="4" t="s">
-        <x:v>251</x:v>
-      </x:c>
-      <x:c r="I5" s="4" t="s">
-        <x:v>252</x:v>
-      </x:c>
-      <x:c r="J5" s="4" t="s">
-        <x:v>253</x:v>
-      </x:c>
-      <x:c r="K5" s="4" t="s">
-        <x:v>254</x:v>
-      </x:c>
-      <x:c r="L5" s="1" t="s">
-        <x:v>255</x:v>
-      </x:c>
-      <x:c r="M5" s="4" t="s">
-        <x:v>256</x:v>
+      <x:c r="A5" s="1" t="str">
+        <x:v>elyria</x:v>
+      </x:c>
+      <x:c r="B5" s="1" t="str">
+        <x:v>Elyria Dawnspell</x:v>
+      </x:c>
+      <x:c r="C5" s="1" t="str">
+        <x:v>Exile's Reach / Stormwind guide fallback</x:v>
+      </x:c>
+      <x:c r="D5" s="1" t="str">
+        <x:v>Human</x:v>
+      </x:c>
+      <x:c r="E5" s="1" t="str">
+        <x:v>Female</x:v>
+      </x:c>
+      <x:c r="F5" s="1" t="str">
+        <x:v>Reincarnation guide</x:v>
+      </x:c>
+      <x:c r="G5" s="1" t="str">
+        <x:v>Bright isekai guide, magical, welcoming</x:v>
+      </x:c>
+      <x:c r="H5" s="4" t="str">
+        <x:v>Placeholder guide concept: polished human mage/priestess look, soft features, luminous fantasy styling.</x:v>
+      </x:c>
+      <x:c r="I5" s="4" t="str">
+        <x:v>Guide-like robes or light magical outfit, gentle glow motifs, simple staff or spellbook.</x:v>
+      </x:c>
+      <x:c r="J5" s="4" t="str">
+        <x:v>Helpful, meta-aware, optimistic, lightly comedic. She frames the player's second life as a grand adventure.</x:v>
+      </x:c>
+      <x:c r="K5" s="4" t="str">
+        <x:v>Clear guide voice with cheerful fantasy narrator energy. Friendly, quick, not too breathy.</x:v>
+      </x:c>
+      <x:c r="L5" s="1" t="str">
+        <x:v>Partial</x:v>
+      </x:c>
+      <x:c r="M5" s="4" t="str">
+        <x:v>Placeholder portrait/dialogue. Needs final art and voice direction pass.</x:v>
       </x:c>
     </x:row>
     <x:row r="6" ht="27">
-      <x:c r="A6" s="1" t="s">
-        <x:v>181</x:v>
-      </x:c>
-      <x:c r="B6" s="1" t="s">
-        <x:v>182</x:v>
-      </x:c>
-      <x:c r="C6" s="1" t="s">
-        <x:v>257</x:v>
-      </x:c>
-      <x:c r="D6" s="1" t="s">
-        <x:v>258</x:v>
-      </x:c>
-      <x:c r="E6" s="1" t="s">
-        <x:v>122</x:v>
-      </x:c>
-      <x:c r="F6" s="1" t="s">
-        <x:v>259</x:v>
-      </x:c>
-      <x:c r="G6" s="1" t="s">
-        <x:v>260</x:v>
-      </x:c>
-      <x:c r="H6" s="4" t="s">
-        <x:v>261</x:v>
-      </x:c>
-      <x:c r="I6" s="4" t="s">
-        <x:v>262</x:v>
-      </x:c>
-      <x:c r="J6" s="4" t="s">
-        <x:v>263</x:v>
-      </x:c>
-      <x:c r="K6" s="4" t="s">
-        <x:v>264</x:v>
-      </x:c>
-      <x:c r="L6" s="1" t="s">
-        <x:v>255</x:v>
-      </x:c>
-      <x:c r="M6" s="4" t="s">
-        <x:v>265</x:v>
+      <x:c r="A6" s="1" t="str">
+        <x:v>mika</x:v>
+      </x:c>
+      <x:c r="B6" s="1" t="str">
+        <x:v>Mika Starbloom</x:v>
+      </x:c>
+      <x:c r="C6" s="1" t="str">
+        <x:v>Orgrimmar / Valdrakken placeholder</x:v>
+      </x:c>
+      <x:c r="D6" s="1" t="str">
+        <x:v>Draenei</x:v>
+      </x:c>
+      <x:c r="E6" s="1" t="str">
+        <x:v>Female</x:v>
+      </x:c>
+      <x:c r="F6" s="1" t="str">
+        <x:v>Cheerful field mage</x:v>
+      </x:c>
+      <x:c r="G6" s="1" t="str">
+        <x:v>Bubbly, curious, explosive optimism</x:v>
+      </x:c>
+      <x:c r="H6" s="4" t="str">
+        <x:v>Placeholder draenei mage concept: bright eyes, expressive face, energetic posture, colorful magical presence.</x:v>
+      </x:c>
+      <x:c r="I6" s="4" t="str">
+        <x:v>Travel mage clothes with playful magical accessories; practical enough for fieldwork, bright enough to feel whimsical.</x:v>
+      </x:c>
+      <x:c r="J6" s="4" t="str">
+        <x:v>Excitable, supportive, slightly chaotic. She turns danger into morale fuel.</x:v>
+      </x:c>
+      <x:c r="K6" s="4" t="str">
+        <x:v>Upbeat, fast smile, energetic comedic timing. Avoid making her too childish.</x:v>
+      </x:c>
+      <x:c r="L6" s="1" t="str">
+        <x:v>Partial</x:v>
+      </x:c>
+      <x:c r="M6" s="4" t="str">
+        <x:v>Temporary mapping; route/faction fit needs later decision.</x:v>
       </x:c>
     </x:row>
     <x:row r="7" ht="27">
-      <x:c r="A7" s="1" t="s">
-        <x:v>183</x:v>
-      </x:c>
-      <x:c r="B7" s="1" t="s">
-        <x:v>184</x:v>
-      </x:c>
-      <x:c r="C7" s="1" t="s">
-        <x:v>266</x:v>
-      </x:c>
-      <x:c r="D7" s="1" t="s">
-        <x:v>267</x:v>
-      </x:c>
-      <x:c r="E7" s="1" t="s">
-        <x:v>122</x:v>
-      </x:c>
-      <x:c r="F7" s="1" t="s">
-        <x:v>268</x:v>
-      </x:c>
-      <x:c r="G7" s="1" t="s">
-        <x:v>269</x:v>
-      </x:c>
-      <x:c r="H7" s="4" t="s">
-        <x:v>270</x:v>
-      </x:c>
-      <x:c r="I7" s="4" t="s">
-        <x:v>271</x:v>
-      </x:c>
-      <x:c r="J7" s="4" t="s">
-        <x:v>272</x:v>
-      </x:c>
-      <x:c r="K7" s="4" t="s">
-        <x:v>273</x:v>
-      </x:c>
-      <x:c r="L7" s="1" t="s">
-        <x:v>255</x:v>
-      </x:c>
-      <x:c r="M7" s="4" t="s">
-        <x:v>274</x:v>
+      <x:c r="A7" s="1" t="str">
+        <x:v>sera</x:v>
+      </x:c>
+      <x:c r="B7" s="1" t="str">
+        <x:v>Sera Moonvale</x:v>
+      </x:c>
+      <x:c r="C7" s="1" t="str">
+        <x:v>Waking Shores / Hallowfall placeholder</x:v>
+      </x:c>
+      <x:c r="D7" s="1" t="str">
+        <x:v>Night Elf</x:v>
+      </x:c>
+      <x:c r="E7" s="1" t="str">
+        <x:v>Female</x:v>
+      </x:c>
+      <x:c r="F7" s="1" t="str">
+        <x:v>Soft-spoken ranger</x:v>
+      </x:c>
+      <x:c r="G7" s="1" t="str">
+        <x:v>Calm, observant, gentle wilderness companion</x:v>
+      </x:c>
+      <x:c r="H7" s="4" t="str">
+        <x:v>Placeholder night elf ranger concept: tall, serene, moonlit features, long hair, quiet watchful presence.</x:v>
+      </x:c>
+      <x:c r="I7" s="4" t="str">
+        <x:v>Ranger leathers, cloak, bow or small nature charms, muted forest/night colors.</x:v>
+      </x:c>
+      <x:c r="J7" s="4" t="str">
+        <x:v>Patient, reflective, emotionally steady. She notices small details and makes the journey feel less lonely.</x:v>
+      </x:c>
+      <x:c r="K7" s="4" t="str">
+        <x:v>Soft, low, composed, intimate. Gentle reassurance rather than bubbly energy.</x:v>
+      </x:c>
+      <x:c r="L7" s="1" t="str">
+        <x:v>Partial</x:v>
+      </x:c>
+      <x:c r="M7" s="4" t="str">
+        <x:v>Needs final zone fit and art direction.</x:v>
       </x:c>
     </x:row>
     <x:row r="8" ht="27">
-      <x:c r="A8" s="1" t="s">
-        <x:v>185</x:v>
-      </x:c>
-      <x:c r="B8" s="1" t="s">
-        <x:v>186</x:v>
-      </x:c>
-      <x:c r="C8" s="1" t="s">
-        <x:v>275</x:v>
-      </x:c>
-      <x:c r="D8" s="1" t="s">
-        <x:v>276</x:v>
-      </x:c>
-      <x:c r="E8" s="1" t="s">
-        <x:v>122</x:v>
-      </x:c>
-      <x:c r="F8" s="1" t="s">
-        <x:v>277</x:v>
-      </x:c>
-      <x:c r="G8" s="1" t="s">
-        <x:v>278</x:v>
-      </x:c>
-      <x:c r="H8" s="4" t="s">
-        <x:v>279</x:v>
-      </x:c>
-      <x:c r="I8" s="4" t="s">
-        <x:v>280</x:v>
-      </x:c>
-      <x:c r="J8" s="4" t="s">
-        <x:v>281</x:v>
-      </x:c>
-      <x:c r="K8" s="4" t="s">
-        <x:v>282</x:v>
-      </x:c>
-      <x:c r="L8" s="1" t="s">
-        <x:v>255</x:v>
-      </x:c>
-      <x:c r="M8" s="4" t="s">
-        <x:v>283</x:v>
+      <x:c r="A8" s="1" t="str">
+        <x:v>kaori</x:v>
+      </x:c>
+      <x:c r="B8" s="1" t="str">
+        <x:v>Kaori Emberheart</x:v>
+      </x:c>
+      <x:c r="C8" s="1" t="str">
+        <x:v>Ohn'ahran Plains / Azj-Kahet placeholder</x:v>
+      </x:c>
+      <x:c r="D8" s="1" t="str">
+        <x:v>Blood Elf</x:v>
+      </x:c>
+      <x:c r="E8" s="1" t="str">
+        <x:v>Female</x:v>
+      </x:c>
+      <x:c r="F8" s="1" t="str">
+        <x:v>Battle senpai</x:v>
+      </x:c>
+      <x:c r="G8" s="1" t="str">
+        <x:v>Confident, fiery, stylish combat mentor</x:v>
+      </x:c>
+      <x:c r="H8" s="4" t="str">
+        <x:v>Placeholder blood elf warrior/mage concept: sharp elegant features, intense eyes, confident battle-ready posture.</x:v>
+      </x:c>
+      <x:c r="I8" s="4" t="str">
+        <x:v>Red/gold combat outfit, elegant armor accents, flame or blade motifs.</x:v>
+      </x:c>
+      <x:c r="J8" s="4" t="str">
+        <x:v>Competitive, teasing, loyal once impressed. Pushes the hero to look cool under pressure.</x:v>
+      </x:c>
+      <x:c r="K8" s="4" t="str">
+        <x:v>Confident anime mentor. Crisp, amused, intense in combat, warmer in bond lines.</x:v>
+      </x:c>
+      <x:c r="L8" s="1" t="str">
+        <x:v>Partial</x:v>
+      </x:c>
+      <x:c r="M8" s="4" t="str">
+        <x:v>Needs final art/voice.</x:v>
       </x:c>
     </x:row>
     <x:row r="9" ht="27">
-      <x:c r="A9" s="1" t="s">
-        <x:v>187</x:v>
-      </x:c>
-      <x:c r="B9" s="1" t="s">
-        <x:v>188</x:v>
-      </x:c>
-      <x:c r="C9" s="1" t="s">
-        <x:v>284</x:v>
-      </x:c>
-      <x:c r="D9" s="1" t="s">
-        <x:v>285</x:v>
-      </x:c>
-      <x:c r="E9" s="1" t="s">
-        <x:v>122</x:v>
-      </x:c>
-      <x:c r="F9" s="1" t="s">
-        <x:v>286</x:v>
-      </x:c>
-      <x:c r="G9" s="1" t="s">
-        <x:v>287</x:v>
-      </x:c>
-      <x:c r="H9" s="4" t="s">
-        <x:v>288</x:v>
-      </x:c>
-      <x:c r="I9" s="4" t="s">
-        <x:v>289</x:v>
-      </x:c>
-      <x:c r="J9" s="4" t="s">
-        <x:v>290</x:v>
-      </x:c>
-      <x:c r="K9" s="4" t="s">
-        <x:v>291</x:v>
-      </x:c>
-      <x:c r="L9" s="1" t="s">
-        <x:v>255</x:v>
-      </x:c>
-      <x:c r="M9" s="4" t="s">
-        <x:v>283</x:v>
+      <x:c r="A9" s="1" t="str">
+        <x:v>rin</x:v>
+      </x:c>
+      <x:c r="B9" s="1" t="str">
+        <x:v>Rin Gearwhisper</x:v>
+      </x:c>
+      <x:c r="C9" s="1" t="str">
+        <x:v>Azure Span / Isle of Dorn placeholder</x:v>
+      </x:c>
+      <x:c r="D9" s="1" t="str">
+        <x:v>Gnome</x:v>
+      </x:c>
+      <x:c r="E9" s="1" t="str">
+        <x:v>Female</x:v>
+      </x:c>
+      <x:c r="F9" s="1" t="str">
+        <x:v>Inventor companion</x:v>
+      </x:c>
+      <x:c r="G9" s="1" t="str">
+        <x:v>Clever, fast-talking, analytical comic relief</x:v>
+      </x:c>
+      <x:c r="H9" s="4" t="str">
+        <x:v>Placeholder gnome inventor concept: compact build, bright eyes, expressive eyebrows, toolbelt energy.</x:v>
+      </x:c>
+      <x:c r="I9" s="4" t="str">
+        <x:v>Engineer goggles, gloves, toolbelt, small gadgets, practical travel boots.</x:v>
+      </x:c>
+      <x:c r="J9" s="4" t="str">
+        <x:v>Brilliant, dry, easily distracted by devices. Affection shows through practical help and nervous jokes.</x:v>
+      </x:c>
+      <x:c r="K9" s="4" t="str">
+        <x:v>Quick, precise, witty. High mental energy without becoming shrill.</x:v>
+      </x:c>
+      <x:c r="L9" s="1" t="str">
+        <x:v>Partial</x:v>
+      </x:c>
+      <x:c r="M9" s="4" t="str">
+        <x:v>Needs final art/voice.</x:v>
       </x:c>
     </x:row>
     <x:row r="10" ht="27">
-      <x:c r="A10" s="1" t="s">
-        <x:v>189</x:v>
-      </x:c>
-      <x:c r="B10" s="1" t="s">
-        <x:v>190</x:v>
-      </x:c>
-      <x:c r="C10" s="1" t="s">
-        <x:v>292</x:v>
-      </x:c>
-      <x:c r="D10" s="1" t="s">
-        <x:v>293</x:v>
-      </x:c>
-      <x:c r="E10" s="1" t="s">
-        <x:v>122</x:v>
-      </x:c>
-      <x:c r="F10" s="1" t="s">
-        <x:v>294</x:v>
-      </x:c>
-      <x:c r="G10" s="1" t="s">
-        <x:v>295</x:v>
-      </x:c>
-      <x:c r="H10" s="4" t="s">
-        <x:v>296</x:v>
-      </x:c>
-      <x:c r="I10" s="4" t="s">
-        <x:v>297</x:v>
-      </x:c>
-      <x:c r="J10" s="4" t="s">
-        <x:v>298</x:v>
-      </x:c>
-      <x:c r="K10" s="4" t="s">
-        <x:v>299</x:v>
-      </x:c>
-      <x:c r="L10" s="1" t="s">
-        <x:v>255</x:v>
-      </x:c>
-      <x:c r="M10" s="4" t="s">
-        <x:v>283</x:v>
+      <x:c r="A10" s="1" t="str">
+        <x:v>lyra</x:v>
+      </x:c>
+      <x:c r="B10" s="1" t="str">
+        <x:v>Lyra Ashpetal</x:v>
+      </x:c>
+      <x:c r="C10" s="1" t="str">
+        <x:v>Thaldraszus placeholder</x:v>
+      </x:c>
+      <x:c r="D10" s="1" t="str">
+        <x:v>Void Elf</x:v>
+      </x:c>
+      <x:c r="E10" s="1" t="str">
+        <x:v>Female</x:v>
+      </x:c>
+      <x:c r="F10" s="1" t="str">
+        <x:v>Mysterious shrine maiden</x:v>
+      </x:c>
+      <x:c r="G10" s="1" t="str">
+        <x:v>Mystical, soft, fate-touched, slightly eerie</x:v>
+      </x:c>
+      <x:c r="H10" s="4" t="str">
+        <x:v>Placeholder void elf mystic concept: pale/lavender tones, long hair, calm eyes, ethereal shrine-maiden silhouette.</x:v>
+      </x:c>
+      <x:c r="I10" s="4" t="str">
+        <x:v>Shrine-inspired robes, subtle void accents, charms or prayer ribbons, twilight color palette.</x:v>
+      </x:c>
+      <x:c r="J10" s="4" t="str">
+        <x:v>Poetic, intuitive, quietly nervous beneath the mysticism. Speaks as if she hears fate whispering nearby.</x:v>
+      </x:c>
+      <x:c r="K10" s="4" t="str">
+        <x:v>Soft mystical cadence. Dreamy but understandable; avoid going too monotone.</x:v>
+      </x:c>
+      <x:c r="L10" s="1" t="str">
+        <x:v>Partial</x:v>
+      </x:c>
+      <x:c r="M10" s="4" t="str">
+        <x:v>Needs final art/voice.</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Raac0ad15a51c42bd"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R1ec9b2f29fdd4e91"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
Add Elune intro narrator
</commit_message>
<xml_diff>
--- a/docs/voice-line-tracker.xlsx
+++ b/docs/voice-line-tracker.xlsx
@@ -2,11 +2,11 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Standards" sheetId="1" r:id="R137c4090c6044359"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Voice Lines" sheetId="2" r:id="R0c165d191a264ed9"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Coverage" sheetId="3" r:id="R70ce7e0f48294414"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Zone Routes" sheetId="4" r:id="Rdeb1bebb959145da"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Character Profiles" sheetId="5" r:id="R0e27b889f0884ee4"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Standards" sheetId="1" r:id="Rfc3cf5f8f6354d16"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Voice Lines" sheetId="2" r:id="Rf50f55d6f3d14921"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Coverage" sheetId="3" r:id="R06055283c5d6493a"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Zone Routes" sheetId="4" r:id="R4c2d550ffdef4d2a"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Character Profiles" sheetId="5" r:id="R3edc5d39854a49ab"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -1915,6 +1915,23 @@
         <x:v>113</x:v>
       </x:c>
     </x:row>
+    <x:row r="39">
+      <x:c r="A39" t="str">
+        <x:v>intro</x:v>
+      </x:c>
+      <x:c r="B39" t="str">
+        <x:v>Opening reincarnation scene</x:v>
+      </x:c>
+      <x:c r="C39" t="n">
+        <x:v>9</x:v>
+      </x:c>
+      <x:c r="D39" t="str">
+        <x:v>Required for Elune narrator</x:v>
+      </x:c>
+      <x:c r="E39" t="str">
+        <x:v>Sequential lines. Filenames: intro_01.mp3 through intro_09.mp3.</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
   <x:mergeCells>
     <x:mergeCell ref="A1:E1"/>
@@ -26620,10 +26637,685 @@
         <x:v>Generated 2026-05-17T23:27:39.293Z (72351 bytes)</x:v>
       </x:c>
     </x:row>
+    <x:row r="325">
+      <x:c r="A325" t="str">
+        <x:v>elune</x:v>
+      </x:c>
+      <x:c r="B325" t="str">
+        <x:v>Elune</x:v>
+      </x:c>
+      <x:c r="C325" t="str">
+        <x:v>Eternal</x:v>
+      </x:c>
+      <x:c r="D325" t="str">
+        <x:v>Female</x:v>
+      </x:c>
+      <x:c r="E325" t="str">
+        <x:v>Intro narrator</x:v>
+      </x:c>
+      <x:c r="F325" t="str">
+        <x:v>intro</x:v>
+      </x:c>
+      <x:c r="G325" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="H325" t="str">
+        <x:v>Required</x:v>
+      </x:c>
+      <x:c r="I325" t="n">
+        <x:v>9</x:v>
+      </x:c>
+      <x:c r="J325" t="str">
+        <x:v>intro_01.mp3</x:v>
+      </x:c>
+      <x:c r="K325" t="n">
+        <x:v>3.2</x:v>
+      </x:c>
+      <x:c r="L325" t="str">
+        <x:v>Needs generation</x:v>
+      </x:c>
+      <x:c r="M325" t="str">
+        <x:v>Awaken, child of another sky.</x:v>
+      </x:c>
+      <x:c r="N325" t="str">
+        <x:v>Media\Voice\Elune\intro_01.mp3</x:v>
+      </x:c>
+      <x:c r="O325" t="str">
+        <x:v>No</x:v>
+      </x:c>
+      <x:c r="P325" t="str"/>
+      <x:c r="Q325" t="str">
+        <x:v>eleven_multilingual_v2</x:v>
+      </x:c>
+      <x:c r="R325" t="str">
+        <x:v>mp3_44100_128</x:v>
+      </x:c>
+      <x:c r="S325" t="n">
+        <x:v>0.48</x:v>
+      </x:c>
+      <x:c r="T325" t="n">
+        <x:v>0.82</x:v>
+      </x:c>
+      <x:c r="U325" t="n">
+        <x:v>0.15</x:v>
+      </x:c>
+      <x:c r="V325" s="5" t="b">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="W325" t="n">
+        <x:v>0.92</x:v>
+      </x:c>
+      <x:c r="X325" s="5" t="b">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="Y325" t="str">
+        <x:v>Opening reincarnation intro; add Elune voice ID before generation.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="326">
+      <x:c r="A326" t="str">
+        <x:v>elune</x:v>
+      </x:c>
+      <x:c r="B326" t="str">
+        <x:v>Elune</x:v>
+      </x:c>
+      <x:c r="C326" t="str">
+        <x:v>Eternal</x:v>
+      </x:c>
+      <x:c r="D326" t="str">
+        <x:v>Female</x:v>
+      </x:c>
+      <x:c r="E326" t="str">
+        <x:v>Intro narrator</x:v>
+      </x:c>
+      <x:c r="F326" t="str">
+        <x:v>intro</x:v>
+      </x:c>
+      <x:c r="G326" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="H326" t="str">
+        <x:v>Required</x:v>
+      </x:c>
+      <x:c r="I326" t="n">
+        <x:v>9</x:v>
+      </x:c>
+      <x:c r="J326" t="str">
+        <x:v>intro_02.mp3</x:v>
+      </x:c>
+      <x:c r="K326" t="n">
+        <x:v>7.2</x:v>
+      </x:c>
+      <x:c r="L326" t="str">
+        <x:v>Needs generation</x:v>
+      </x:c>
+      <x:c r="M326" t="str">
+        <x:v>I am Elune, the moon's eternal light, and I have watched your soul cross a threshold it was never meant to find.</x:v>
+      </x:c>
+      <x:c r="N326" t="str">
+        <x:v>Media\Voice\Elune\intro_02.mp3</x:v>
+      </x:c>
+      <x:c r="O326" t="str">
+        <x:v>No</x:v>
+      </x:c>
+      <x:c r="P326" t="str"/>
+      <x:c r="Q326" t="str">
+        <x:v>eleven_multilingual_v2</x:v>
+      </x:c>
+      <x:c r="R326" t="str">
+        <x:v>mp3_44100_128</x:v>
+      </x:c>
+      <x:c r="S326" t="n">
+        <x:v>0.48</x:v>
+      </x:c>
+      <x:c r="T326" t="n">
+        <x:v>0.82</x:v>
+      </x:c>
+      <x:c r="U326" t="n">
+        <x:v>0.15</x:v>
+      </x:c>
+      <x:c r="V326" s="5" t="b">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="W326" t="n">
+        <x:v>0.92</x:v>
+      </x:c>
+      <x:c r="X326" s="5" t="b">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="Y326" t="str">
+        <x:v>Opening reincarnation intro; add Elune voice ID before generation.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="327">
+      <x:c r="A327" t="str">
+        <x:v>elune</x:v>
+      </x:c>
+      <x:c r="B327" t="str">
+        <x:v>Elune</x:v>
+      </x:c>
+      <x:c r="C327" t="str">
+        <x:v>Eternal</x:v>
+      </x:c>
+      <x:c r="D327" t="str">
+        <x:v>Female</x:v>
+      </x:c>
+      <x:c r="E327" t="str">
+        <x:v>Intro narrator</x:v>
+      </x:c>
+      <x:c r="F327" t="str">
+        <x:v>intro</x:v>
+      </x:c>
+      <x:c r="G327" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="H327" t="str">
+        <x:v>Required</x:v>
+      </x:c>
+      <x:c r="I327" t="n">
+        <x:v>9</x:v>
+      </x:c>
+      <x:c r="J327" t="str">
+        <x:v>intro_03.mp3</x:v>
+      </x:c>
+      <x:c r="K327" t="n">
+        <x:v>6.3</x:v>
+      </x:c>
+      <x:c r="L327" t="str">
+        <x:v>Needs generation</x:v>
+      </x:c>
+      <x:c r="M327" t="str">
+        <x:v>Your thread was severed before its hour. In the world that bore you, your life has ended.</x:v>
+      </x:c>
+      <x:c r="N327" t="str">
+        <x:v>Media\Voice\Elune\intro_03.mp3</x:v>
+      </x:c>
+      <x:c r="O327" t="str">
+        <x:v>No</x:v>
+      </x:c>
+      <x:c r="P327" t="str"/>
+      <x:c r="Q327" t="str">
+        <x:v>eleven_multilingual_v2</x:v>
+      </x:c>
+      <x:c r="R327" t="str">
+        <x:v>mp3_44100_128</x:v>
+      </x:c>
+      <x:c r="S327" t="n">
+        <x:v>0.48</x:v>
+      </x:c>
+      <x:c r="T327" t="n">
+        <x:v>0.82</x:v>
+      </x:c>
+      <x:c r="U327" t="n">
+        <x:v>0.15</x:v>
+      </x:c>
+      <x:c r="V327" s="5" t="b">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="W327" t="n">
+        <x:v>0.92</x:v>
+      </x:c>
+      <x:c r="X327" s="5" t="b">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="Y327" t="str">
+        <x:v>Opening reincarnation intro; add Elune voice ID before generation.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="328">
+      <x:c r="A328" t="str">
+        <x:v>elune</x:v>
+      </x:c>
+      <x:c r="B328" t="str">
+        <x:v>Elune</x:v>
+      </x:c>
+      <x:c r="C328" t="str">
+        <x:v>Eternal</x:v>
+      </x:c>
+      <x:c r="D328" t="str">
+        <x:v>Female</x:v>
+      </x:c>
+      <x:c r="E328" t="str">
+        <x:v>Intro narrator</x:v>
+      </x:c>
+      <x:c r="F328" t="str">
+        <x:v>intro</x:v>
+      </x:c>
+      <x:c r="G328" t="n">
+        <x:v>4</x:v>
+      </x:c>
+      <x:c r="H328" t="str">
+        <x:v>Required</x:v>
+      </x:c>
+      <x:c r="I328" t="n">
+        <x:v>9</x:v>
+      </x:c>
+      <x:c r="J328" t="str">
+        <x:v>intro_04.mp3</x:v>
+      </x:c>
+      <x:c r="K328" t="n">
+        <x:v>7.5</x:v>
+      </x:c>
+      <x:c r="L328" t="str">
+        <x:v>Needs generation</x:v>
+      </x:c>
+      <x:c r="M328" t="str">
+        <x:v>I cannot return you to that place. The path behind you has closed, and to force it open would wound more than fate.</x:v>
+      </x:c>
+      <x:c r="N328" t="str">
+        <x:v>Media\Voice\Elune\intro_04.mp3</x:v>
+      </x:c>
+      <x:c r="O328" t="str">
+        <x:v>No</x:v>
+      </x:c>
+      <x:c r="P328" t="str"/>
+      <x:c r="Q328" t="str">
+        <x:v>eleven_multilingual_v2</x:v>
+      </x:c>
+      <x:c r="R328" t="str">
+        <x:v>mp3_44100_128</x:v>
+      </x:c>
+      <x:c r="S328" t="n">
+        <x:v>0.48</x:v>
+      </x:c>
+      <x:c r="T328" t="n">
+        <x:v>0.82</x:v>
+      </x:c>
+      <x:c r="U328" t="n">
+        <x:v>0.15</x:v>
+      </x:c>
+      <x:c r="V328" s="5" t="b">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="W328" t="n">
+        <x:v>0.92</x:v>
+      </x:c>
+      <x:c r="X328" s="5" t="b">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="Y328" t="str">
+        <x:v>Opening reincarnation intro; add Elune voice ID before generation.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="329">
+      <x:c r="A329" t="str">
+        <x:v>elune</x:v>
+      </x:c>
+      <x:c r="B329" t="str">
+        <x:v>Elune</x:v>
+      </x:c>
+      <x:c r="C329" t="str">
+        <x:v>Eternal</x:v>
+      </x:c>
+      <x:c r="D329" t="str">
+        <x:v>Female</x:v>
+      </x:c>
+      <x:c r="E329" t="str">
+        <x:v>Intro narrator</x:v>
+      </x:c>
+      <x:c r="F329" t="str">
+        <x:v>intro</x:v>
+      </x:c>
+      <x:c r="G329" t="n">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="H329" t="str">
+        <x:v>Required</x:v>
+      </x:c>
+      <x:c r="I329" t="n">
+        <x:v>9</x:v>
+      </x:c>
+      <x:c r="J329" t="str">
+        <x:v>intro_05.mp3</x:v>
+      </x:c>
+      <x:c r="K329" t="n">
+        <x:v>6.2</x:v>
+      </x:c>
+      <x:c r="L329" t="str">
+        <x:v>Needs generation</x:v>
+      </x:c>
+      <x:c r="M329" t="str">
+        <x:v>So I have drawn your soul beneath Azeroth's moon, where broken lives may yet find new light.</x:v>
+      </x:c>
+      <x:c r="N329" t="str">
+        <x:v>Media\Voice\Elune\intro_05.mp3</x:v>
+      </x:c>
+      <x:c r="O329" t="str">
+        <x:v>No</x:v>
+      </x:c>
+      <x:c r="P329" t="str"/>
+      <x:c r="Q329" t="str">
+        <x:v>eleven_multilingual_v2</x:v>
+      </x:c>
+      <x:c r="R329" t="str">
+        <x:v>mp3_44100_128</x:v>
+      </x:c>
+      <x:c r="S329" t="n">
+        <x:v>0.48</x:v>
+      </x:c>
+      <x:c r="T329" t="n">
+        <x:v>0.82</x:v>
+      </x:c>
+      <x:c r="U329" t="n">
+        <x:v>0.15</x:v>
+      </x:c>
+      <x:c r="V329" s="5" t="b">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="W329" t="n">
+        <x:v>0.92</x:v>
+      </x:c>
+      <x:c r="X329" s="5" t="b">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="Y329" t="str">
+        <x:v>Opening reincarnation intro; add Elune voice ID before generation.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="330">
+      <x:c r="A330" t="str">
+        <x:v>elune</x:v>
+      </x:c>
+      <x:c r="B330" t="str">
+        <x:v>Elune</x:v>
+      </x:c>
+      <x:c r="C330" t="str">
+        <x:v>Eternal</x:v>
+      </x:c>
+      <x:c r="D330" t="str">
+        <x:v>Female</x:v>
+      </x:c>
+      <x:c r="E330" t="str">
+        <x:v>Intro narrator</x:v>
+      </x:c>
+      <x:c r="F330" t="str">
+        <x:v>intro</x:v>
+      </x:c>
+      <x:c r="G330" t="n">
+        <x:v>6</x:v>
+      </x:c>
+      <x:c r="H330" t="str">
+        <x:v>Required</x:v>
+      </x:c>
+      <x:c r="I330" t="n">
+        <x:v>9</x:v>
+      </x:c>
+      <x:c r="J330" t="str">
+        <x:v>intro_06.mp3</x:v>
+      </x:c>
+      <x:c r="K330" t="n">
+        <x:v>6.3</x:v>
+      </x:c>
+      <x:c r="L330" t="str">
+        <x:v>Needs generation</x:v>
+      </x:c>
+      <x:c r="M330" t="str">
+        <x:v>This world is beautiful, wounded, and often unkind. You will need more than courage to endure it.</x:v>
+      </x:c>
+      <x:c r="N330" t="str">
+        <x:v>Media\Voice\Elune\intro_06.mp3</x:v>
+      </x:c>
+      <x:c r="O330" t="str">
+        <x:v>No</x:v>
+      </x:c>
+      <x:c r="P330" t="str"/>
+      <x:c r="Q330" t="str">
+        <x:v>eleven_multilingual_v2</x:v>
+      </x:c>
+      <x:c r="R330" t="str">
+        <x:v>mp3_44100_128</x:v>
+      </x:c>
+      <x:c r="S330" t="n">
+        <x:v>0.48</x:v>
+      </x:c>
+      <x:c r="T330" t="n">
+        <x:v>0.82</x:v>
+      </x:c>
+      <x:c r="U330" t="n">
+        <x:v>0.15</x:v>
+      </x:c>
+      <x:c r="V330" s="5" t="b">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="W330" t="n">
+        <x:v>0.92</x:v>
+      </x:c>
+      <x:c r="X330" s="5" t="b">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="Y330" t="str">
+        <x:v>Opening reincarnation intro; add Elune voice ID before generation.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="331">
+      <x:c r="A331" t="str">
+        <x:v>elune</x:v>
+      </x:c>
+      <x:c r="B331" t="str">
+        <x:v>Elune</x:v>
+      </x:c>
+      <x:c r="C331" t="str">
+        <x:v>Eternal</x:v>
+      </x:c>
+      <x:c r="D331" t="str">
+        <x:v>Female</x:v>
+      </x:c>
+      <x:c r="E331" t="str">
+        <x:v>Intro narrator</x:v>
+      </x:c>
+      <x:c r="F331" t="str">
+        <x:v>intro</x:v>
+      </x:c>
+      <x:c r="G331" t="n">
+        <x:v>7</x:v>
+      </x:c>
+      <x:c r="H331" t="str">
+        <x:v>Required</x:v>
+      </x:c>
+      <x:c r="I331" t="n">
+        <x:v>9</x:v>
+      </x:c>
+      <x:c r="J331" t="str">
+        <x:v>intro_07.mp3</x:v>
+      </x:c>
+      <x:c r="K331" t="n">
+        <x:v>7</x:v>
+      </x:c>
+      <x:c r="L331" t="str">
+        <x:v>Needs generation</x:v>
+      </x:c>
+      <x:c r="M331" t="str">
+        <x:v>You shall not walk alone. In each land, a heart will find yours, and beside you learn what shape destiny now takes.</x:v>
+      </x:c>
+      <x:c r="N331" t="str">
+        <x:v>Media\Voice\Elune\intro_07.mp3</x:v>
+      </x:c>
+      <x:c r="O331" t="str">
+        <x:v>No</x:v>
+      </x:c>
+      <x:c r="P331" t="str"/>
+      <x:c r="Q331" t="str">
+        <x:v>eleven_multilingual_v2</x:v>
+      </x:c>
+      <x:c r="R331" t="str">
+        <x:v>mp3_44100_128</x:v>
+      </x:c>
+      <x:c r="S331" t="n">
+        <x:v>0.48</x:v>
+      </x:c>
+      <x:c r="T331" t="n">
+        <x:v>0.82</x:v>
+      </x:c>
+      <x:c r="U331" t="n">
+        <x:v>0.15</x:v>
+      </x:c>
+      <x:c r="V331" s="5" t="b">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="W331" t="n">
+        <x:v>0.92</x:v>
+      </x:c>
+      <x:c r="X331" s="5" t="b">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="Y331" t="str">
+        <x:v>Opening reincarnation intro; add Elune voice ID before generation.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="332">
+      <x:c r="A332" t="str">
+        <x:v>elune</x:v>
+      </x:c>
+      <x:c r="B332" t="str">
+        <x:v>Elune</x:v>
+      </x:c>
+      <x:c r="C332" t="str">
+        <x:v>Eternal</x:v>
+      </x:c>
+      <x:c r="D332" t="str">
+        <x:v>Female</x:v>
+      </x:c>
+      <x:c r="E332" t="str">
+        <x:v>Intro narrator</x:v>
+      </x:c>
+      <x:c r="F332" t="str">
+        <x:v>intro</x:v>
+      </x:c>
+      <x:c r="G332" t="n">
+        <x:v>8</x:v>
+      </x:c>
+      <x:c r="H332" t="str">
+        <x:v>Required</x:v>
+      </x:c>
+      <x:c r="I332" t="n">
+        <x:v>9</x:v>
+      </x:c>
+      <x:c r="J332" t="str">
+        <x:v>intro_08.mp3</x:v>
+      </x:c>
+      <x:c r="K332" t="n">
+        <x:v>5.6</x:v>
+      </x:c>
+      <x:c r="L332" t="str">
+        <x:v>Needs generation</x:v>
+      </x:c>
+      <x:c r="M332" t="str">
+        <x:v>Go gently, reborn one. Let this second life become more than an apology.</x:v>
+      </x:c>
+      <x:c r="N332" t="str">
+        <x:v>Media\Voice\Elune\intro_08.mp3</x:v>
+      </x:c>
+      <x:c r="O332" t="str">
+        <x:v>No</x:v>
+      </x:c>
+      <x:c r="P332" t="str"/>
+      <x:c r="Q332" t="str">
+        <x:v>eleven_multilingual_v2</x:v>
+      </x:c>
+      <x:c r="R332" t="str">
+        <x:v>mp3_44100_128</x:v>
+      </x:c>
+      <x:c r="S332" t="n">
+        <x:v>0.48</x:v>
+      </x:c>
+      <x:c r="T332" t="n">
+        <x:v>0.82</x:v>
+      </x:c>
+      <x:c r="U332" t="n">
+        <x:v>0.15</x:v>
+      </x:c>
+      <x:c r="V332" s="5" t="b">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="W332" t="n">
+        <x:v>0.92</x:v>
+      </x:c>
+      <x:c r="X332" s="5" t="b">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="Y332" t="str">
+        <x:v>Opening reincarnation intro; add Elune voice ID before generation.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="333">
+      <x:c r="A333" t="str">
+        <x:v>elune</x:v>
+      </x:c>
+      <x:c r="B333" t="str">
+        <x:v>Elune</x:v>
+      </x:c>
+      <x:c r="C333" t="str">
+        <x:v>Eternal</x:v>
+      </x:c>
+      <x:c r="D333" t="str">
+        <x:v>Female</x:v>
+      </x:c>
+      <x:c r="E333" t="str">
+        <x:v>Intro narrator</x:v>
+      </x:c>
+      <x:c r="F333" t="str">
+        <x:v>intro</x:v>
+      </x:c>
+      <x:c r="G333" t="n">
+        <x:v>9</x:v>
+      </x:c>
+      <x:c r="H333" t="str">
+        <x:v>Required</x:v>
+      </x:c>
+      <x:c r="I333" t="n">
+        <x:v>9</x:v>
+      </x:c>
+      <x:c r="J333" t="str">
+        <x:v>intro_09.mp3</x:v>
+      </x:c>
+      <x:c r="K333" t="n">
+        <x:v>3.6</x:v>
+      </x:c>
+      <x:c r="L333" t="str">
+        <x:v>Needs generation</x:v>
+      </x:c>
+      <x:c r="M333" t="str">
+        <x:v>Rise now. Azeroth is waiting.</x:v>
+      </x:c>
+      <x:c r="N333" t="str">
+        <x:v>Media\Voice\Elune\intro_09.mp3</x:v>
+      </x:c>
+      <x:c r="O333" t="str">
+        <x:v>No</x:v>
+      </x:c>
+      <x:c r="P333" t="str"/>
+      <x:c r="Q333" t="str">
+        <x:v>eleven_multilingual_v2</x:v>
+      </x:c>
+      <x:c r="R333" t="str">
+        <x:v>mp3_44100_128</x:v>
+      </x:c>
+      <x:c r="S333" t="n">
+        <x:v>0.48</x:v>
+      </x:c>
+      <x:c r="T333" t="n">
+        <x:v>0.82</x:v>
+      </x:c>
+      <x:c r="U333" t="n">
+        <x:v>0.15</x:v>
+      </x:c>
+      <x:c r="V333" s="5" t="b">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="W333" t="n">
+        <x:v>0.92</x:v>
+      </x:c>
+      <x:c r="X333" s="5" t="b">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="Y333" t="str">
+        <x:v>Opening reincarnation intro; add Elune voice ID before generation.</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Ra832edd61ffd412e"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R957108c11897483c"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -37534,10 +38226,36 @@
         <x:v>123</x:v>
       </x:c>
     </x:row>
+    <x:row r="420">
+      <x:c r="A420" t="str">
+        <x:v>elune</x:v>
+      </x:c>
+      <x:c r="B420" t="str">
+        <x:v>Elune</x:v>
+      </x:c>
+      <x:c r="C420" t="str">
+        <x:v>Female</x:v>
+      </x:c>
+      <x:c r="D420" t="str">
+        <x:v>intro</x:v>
+      </x:c>
+      <x:c r="E420" t="n">
+        <x:v>9</x:v>
+      </x:c>
+      <x:c r="F420" t="n">
+        <x:v>9</x:v>
+      </x:c>
+      <x:c r="G420" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="H420" t="str">
+        <x:v>OK</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R36101cf6896341d5"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R289c033c8b1f4d40"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -37937,7 +38655,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R8a291944f22d4493"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R4ab5707a98d2439d"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -38412,10 +39130,51 @@
         <x:v>309</x:v>
       </x:c>
     </x:row>
+    <x:row r="12">
+      <x:c r="A12" t="str">
+        <x:v>elune</x:v>
+      </x:c>
+      <x:c r="B12" t="str">
+        <x:v>Elune</x:v>
+      </x:c>
+      <x:c r="C12" t="str">
+        <x:v>Intro narrator</x:v>
+      </x:c>
+      <x:c r="D12" t="str">
+        <x:v>Eternal</x:v>
+      </x:c>
+      <x:c r="E12" t="str">
+        <x:v>Female</x:v>
+      </x:c>
+      <x:c r="F12" t="str">
+        <x:v>Moon goddess / reincarnation guide</x:v>
+      </x:c>
+      <x:c r="G12" t="str">
+        <x:v>Serene, ancient, compassionate, sacred, quietly sorrowful</x:v>
+      </x:c>
+      <x:c r="H12" t="str">
+        <x:v>A luminous moonlit goddess with night-elf-like elegance, pale lavender skin, silver-white hair, crescent moon ornaments, and a calm celestial presence.</x:v>
+      </x:c>
+      <x:c r="I12" t="str">
+        <x:v>Moon-silver regalia, delicate star jewelry, crescent motifs, soft glowing aura.</x:v>
+      </x:c>
+      <x:c r="J12" t="str">
+        <x:v>Gentle but immense; speaks as someone who can see fate clearly and still grieves the pain inside it.</x:v>
+      </x:c>
+      <x:c r="K12" t="str">
+        <x:v>Slow, reverent, warm, ethereal, maternal without sounding casual; each sentence should feel like moonlight over a sacred place.</x:v>
+      </x:c>
+      <x:c r="L12" t="str">
+        <x:v>Done</x:v>
+      </x:c>
+      <x:c r="M12" t="str">
+        <x:v>Special narrator only. Not a romance/bond companion and not assigned to zone routes.</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R36ea7ac1ad3c4072"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Ra8f6f94c9a8b47de"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
Fix voice line timing
</commit_message>
<xml_diff>
--- a/docs/voice-line-tracker.xlsx
+++ b/docs/voice-line-tracker.xlsx
@@ -2,11 +2,11 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Standards" sheetId="1" r:id="R4ad422cf7ef74508"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Voice Lines" sheetId="2" r:id="Rc28836b758a34499"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Coverage" sheetId="3" r:id="R7154523953db486c"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Zone Routes" sheetId="4" r:id="R5d4d82da837847dc"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Character Profiles" sheetId="5" r:id="R00e6f6546a1f45ec"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Standards" sheetId="1" r:id="R5d72cc7b4d13433d"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Voice Lines" sheetId="2" r:id="Rdb76cf4d0b254a04"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Coverage" sheetId="3" r:id="R94505964be444894"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Zone Routes" sheetId="4" r:id="Raac8f370a49a42cc"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Character Profiles" sheetId="5" r:id="Rc8b5791888c744fc"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -2125,7 +2125,7 @@
         <x:v>zone_intro_01.mp3</x:v>
       </x:c>
       <x:c r="K2" s="1" t="n">
-        <x:v>6.2</x:v>
+        <x:v>9.4</x:v>
       </x:c>
       <x:c r="L2" s="1" t="str">
         <x:v>Audio exists</x:v>
@@ -2200,7 +2200,7 @@
         <x:v>zone_intro_02.mp3</x:v>
       </x:c>
       <x:c r="K3" s="1" t="n">
-        <x:v>5.6</x:v>
+        <x:v>7.5</x:v>
       </x:c>
       <x:c r="L3" s="1" t="str">
         <x:v>Audio exists</x:v>
@@ -2275,7 +2275,7 @@
         <x:v>quest_accept_01.mp3</x:v>
       </x:c>
       <x:c r="K4" s="1" t="n">
-        <x:v>4.4</x:v>
+        <x:v>5.1</x:v>
       </x:c>
       <x:c r="L4" s="1" t="str">
         <x:v>Audio exists</x:v>
@@ -2350,7 +2350,7 @@
         <x:v>quest_accept_02.mp3</x:v>
       </x:c>
       <x:c r="K5" s="1" t="n">
-        <x:v>5.6</x:v>
+        <x:v>7.8</x:v>
       </x:c>
       <x:c r="L5" s="1" t="str">
         <x:v>Audio exists</x:v>
@@ -2425,7 +2425,7 @@
         <x:v>quest_accept_03.mp3</x:v>
       </x:c>
       <x:c r="K6" s="1" t="n">
-        <x:v>5.4</x:v>
+        <x:v>6.4</x:v>
       </x:c>
       <x:c r="L6" s="1" t="str">
         <x:v>Audio exists</x:v>
@@ -2500,7 +2500,7 @@
         <x:v>kill_01.mp3</x:v>
       </x:c>
       <x:c r="K7" s="1" t="n">
-        <x:v>4.3</x:v>
+        <x:v>7.8</x:v>
       </x:c>
       <x:c r="L7" s="1" t="str">
         <x:v>Audio exists</x:v>
@@ -2575,7 +2575,7 @@
         <x:v>kill_02.mp3</x:v>
       </x:c>
       <x:c r="K8" s="1" t="n">
-        <x:v>4</x:v>
+        <x:v>5.7</x:v>
       </x:c>
       <x:c r="L8" s="1" t="str">
         <x:v>Audio exists</x:v>
@@ -2650,7 +2650,7 @@
         <x:v>kill_03.mp3</x:v>
       </x:c>
       <x:c r="K9" s="1" t="n">
-        <x:v>4.5</x:v>
+        <x:v>5</x:v>
       </x:c>
       <x:c r="L9" s="1" t="str">
         <x:v>Audio exists</x:v>
@@ -2725,7 +2725,7 @@
         <x:v>idle_01.mp3</x:v>
       </x:c>
       <x:c r="K10" s="1" t="n">
-        <x:v>4.8</x:v>
+        <x:v>6.9</x:v>
       </x:c>
       <x:c r="L10" s="1" t="str">
         <x:v>Audio exists</x:v>
@@ -2800,7 +2800,7 @@
         <x:v>idle_02.mp3</x:v>
       </x:c>
       <x:c r="K11" s="1" t="n">
-        <x:v>5.2</x:v>
+        <x:v>7.1</x:v>
       </x:c>
       <x:c r="L11" s="1" t="str">
         <x:v>Audio exists</x:v>
@@ -2875,7 +2875,7 @@
         <x:v>idle_03.mp3</x:v>
       </x:c>
       <x:c r="K12" s="1" t="n">
-        <x:v>4.2</x:v>
+        <x:v>6.2</x:v>
       </x:c>
       <x:c r="L12" s="1" t="str">
         <x:v>Audio exists</x:v>
@@ -2950,7 +2950,7 @@
         <x:v>level_up.mp3</x:v>
       </x:c>
       <x:c r="K13" s="1" t="n">
-        <x:v>4.4</x:v>
+        <x:v>6.2</x:v>
       </x:c>
       <x:c r="L13" s="1" t="str">
         <x:v>Audio exists</x:v>
@@ -3025,7 +3025,7 @@
         <x:v>level_up_02.mp3</x:v>
       </x:c>
       <x:c r="K14" s="1" t="n">
-        <x:v>5.6</x:v>
+        <x:v>5.9</x:v>
       </x:c>
       <x:c r="L14" s="1" t="str">
         <x:v>Audio exists</x:v>
@@ -3102,7 +3102,7 @@
         <x:v>summon_01.mp3</x:v>
       </x:c>
       <x:c r="K15" s="1" t="n">
-        <x:v>4.9</x:v>
+        <x:v>6.1</x:v>
       </x:c>
       <x:c r="L15" s="1" t="str">
         <x:v>Audio exists</x:v>
@@ -3177,7 +3177,7 @@
         <x:v>bond_02_01.mp3</x:v>
       </x:c>
       <x:c r="K16" s="1" t="n">
-        <x:v>5.4</x:v>
+        <x:v>6.5</x:v>
       </x:c>
       <x:c r="L16" s="1" t="str">
         <x:v>Audio exists</x:v>
@@ -3254,7 +3254,7 @@
         <x:v>bond_04_01.mp3</x:v>
       </x:c>
       <x:c r="K17" s="1" t="n">
-        <x:v>6</x:v>
+        <x:v>6.4</x:v>
       </x:c>
       <x:c r="L17" s="1" t="str">
         <x:v>Audio exists</x:v>
@@ -3331,7 +3331,7 @@
         <x:v>bond_06_01.mp3</x:v>
       </x:c>
       <x:c r="K18" s="1" t="n">
-        <x:v>5.6</x:v>
+        <x:v>5.9</x:v>
       </x:c>
       <x:c r="L18" s="1" t="str">
         <x:v>Audio exists</x:v>
@@ -3408,7 +3408,7 @@
         <x:v>bond_08_01.mp3</x:v>
       </x:c>
       <x:c r="K19" s="1" t="n">
-        <x:v>5.8</x:v>
+        <x:v>5.3</x:v>
       </x:c>
       <x:c r="L19" s="1" t="str">
         <x:v>Audio exists</x:v>
@@ -3485,7 +3485,7 @@
         <x:v>bond_10_01.mp3</x:v>
       </x:c>
       <x:c r="K20" s="1" t="n">
-        <x:v>6</x:v>
+        <x:v>5.6</x:v>
       </x:c>
       <x:c r="L20" s="1" t="str">
         <x:v>Audio exists</x:v>
@@ -3562,7 +3562,7 @@
         <x:v>romance_02_01.mp3</x:v>
       </x:c>
       <x:c r="K21" s="1" t="n">
-        <x:v>6</x:v>
+        <x:v>7.8</x:v>
       </x:c>
       <x:c r="L21" s="1" t="str">
         <x:v>Audio exists</x:v>
@@ -3639,7 +3639,7 @@
         <x:v>romance_04_01.mp3</x:v>
       </x:c>
       <x:c r="K22" s="1" t="n">
-        <x:v>6.2</x:v>
+        <x:v>6.9</x:v>
       </x:c>
       <x:c r="L22" s="1" t="str">
         <x:v>Audio exists</x:v>
@@ -3716,7 +3716,7 @@
         <x:v>romance_06_01.mp3</x:v>
       </x:c>
       <x:c r="K23" s="1" t="n">
-        <x:v>6.1</x:v>
+        <x:v>7.4</x:v>
       </x:c>
       <x:c r="L23" s="1" t="str">
         <x:v>Audio exists</x:v>
@@ -3793,7 +3793,7 @@
         <x:v>romance_08_01.mp3</x:v>
       </x:c>
       <x:c r="K24" s="1" t="n">
-        <x:v>5.6</x:v>
+        <x:v>4.9</x:v>
       </x:c>
       <x:c r="L24" s="1" t="str">
         <x:v>Audio exists</x:v>
@@ -3870,7 +3870,7 @@
         <x:v>romance_10_01.mp3</x:v>
       </x:c>
       <x:c r="K25" s="1" t="n">
-        <x:v>6.3</x:v>
+        <x:v>7.2</x:v>
       </x:c>
       <x:c r="L25" s="1" t="str">
         <x:v>Audio exists</x:v>
@@ -3947,7 +3947,7 @@
         <x:v>romance_not_ready_01.mp3</x:v>
       </x:c>
       <x:c r="K26" s="1" t="n">
-        <x:v>5.4</x:v>
+        <x:v>5.3</x:v>
       </x:c>
       <x:c r="L26" s="1" t="str">
         <x:v>Audio exists</x:v>
@@ -4024,7 +4024,7 @@
         <x:v>romance_repeat_01.mp3</x:v>
       </x:c>
       <x:c r="K27" s="1" t="n">
-        <x:v>5.4</x:v>
+        <x:v>6.2</x:v>
       </x:c>
       <x:c r="L27" s="1" t="str">
         <x:v>Audio exists</x:v>
@@ -4101,7 +4101,7 @@
         <x:v>romance_stop_01.mp3</x:v>
       </x:c>
       <x:c r="K28" s="1" t="n">
-        <x:v>5.8</x:v>
+        <x:v>6.2</x:v>
       </x:c>
       <x:c r="L28" s="1" t="str">
         <x:v>Audio exists</x:v>
@@ -4178,7 +4178,7 @@
         <x:v>quest_complete_01.mp3</x:v>
       </x:c>
       <x:c r="K29" s="1" t="n">
-        <x:v>5.3</x:v>
+        <x:v>5.7</x:v>
       </x:c>
       <x:c r="L29" s="1" t="str">
         <x:v>Audio exists</x:v>
@@ -4255,7 +4255,7 @@
         <x:v>quest_complete_02.mp3</x:v>
       </x:c>
       <x:c r="K30" s="1" t="n">
-        <x:v>5</x:v>
+        <x:v>5.4</x:v>
       </x:c>
       <x:c r="L30" s="1" t="str">
         <x:v>Audio exists</x:v>
@@ -4409,7 +4409,7 @@
         <x:v>bond_kill_02.mp3</x:v>
       </x:c>
       <x:c r="K32" s="1" t="n">
-        <x:v>4.6</x:v>
+        <x:v>4.5</x:v>
       </x:c>
       <x:c r="L32" s="1" t="str">
         <x:v>Audio exists</x:v>
@@ -4486,7 +4486,7 @@
         <x:v>bond_kill_04.mp3</x:v>
       </x:c>
       <x:c r="K33" s="1" t="n">
-        <x:v>4.7</x:v>
+        <x:v>4.3</x:v>
       </x:c>
       <x:c r="L33" s="1" t="str">
         <x:v>Audio exists</x:v>
@@ -4563,7 +4563,7 @@
         <x:v>bond_kill_06.mp3</x:v>
       </x:c>
       <x:c r="K34" s="1" t="n">
-        <x:v>5</x:v>
+        <x:v>4.9</x:v>
       </x:c>
       <x:c r="L34" s="1" t="str">
         <x:v>Audio exists</x:v>
@@ -4640,7 +4640,7 @@
         <x:v>bond_kill_08.mp3</x:v>
       </x:c>
       <x:c r="K35" s="1" t="n">
-        <x:v>4.9</x:v>
+        <x:v>4.7</x:v>
       </x:c>
       <x:c r="L35" s="1" t="str">
         <x:v>Audio exists</x:v>
@@ -4717,7 +4717,7 @@
         <x:v>bond_kill_10.mp3</x:v>
       </x:c>
       <x:c r="K36" s="1" t="n">
-        <x:v>5.2</x:v>
+        <x:v>5.1</x:v>
       </x:c>
       <x:c r="L36" s="1" t="str">
         <x:v>Audio exists</x:v>
@@ -4794,7 +4794,7 @@
         <x:v>bond_idle_01.mp3</x:v>
       </x:c>
       <x:c r="K37" s="1" t="n">
-        <x:v>5.3</x:v>
+        <x:v>5</x:v>
       </x:c>
       <x:c r="L37" s="1" t="str">
         <x:v>Audio exists</x:v>
@@ -4871,7 +4871,7 @@
         <x:v>bond_idle_03.mp3</x:v>
       </x:c>
       <x:c r="K38" s="1" t="n">
-        <x:v>5.5</x:v>
+        <x:v>5</x:v>
       </x:c>
       <x:c r="L38" s="1" t="str">
         <x:v>Audio exists</x:v>
@@ -4948,7 +4948,7 @@
         <x:v>bond_idle_05.mp3</x:v>
       </x:c>
       <x:c r="K39" s="1" t="n">
-        <x:v>5.1</x:v>
+        <x:v>4.7</x:v>
       </x:c>
       <x:c r="L39" s="1" t="str">
         <x:v>Audio exists</x:v>
@@ -5025,7 +5025,7 @@
         <x:v>bond_idle_07.mp3</x:v>
       </x:c>
       <x:c r="K40" s="1" t="n">
-        <x:v>6.4</x:v>
+        <x:v>7.3</x:v>
       </x:c>
       <x:c r="L40" s="1" t="str">
         <x:v>Audio exists</x:v>
@@ -5102,7 +5102,7 @@
         <x:v>bond_idle_09.mp3</x:v>
       </x:c>
       <x:c r="K41" s="1" t="n">
-        <x:v>5.9</x:v>
+        <x:v>5.3</x:v>
       </x:c>
       <x:c r="L41" s="1" t="str">
         <x:v>Audio exists</x:v>
@@ -5179,7 +5179,7 @@
         <x:v>low_health_01.mp3</x:v>
       </x:c>
       <x:c r="K42" s="1" t="n">
-        <x:v>5.7</x:v>
+        <x:v>5.4</x:v>
       </x:c>
       <x:c r="L42" s="1" t="str">
         <x:v>Audio exists</x:v>
@@ -5256,7 +5256,7 @@
         <x:v>death_01.mp3</x:v>
       </x:c>
       <x:c r="K43" s="1" t="n">
-        <x:v>6.3</x:v>
+        <x:v>5.8</x:v>
       </x:c>
       <x:c r="L43" s="1" t="str">
         <x:v>Audio exists</x:v>
@@ -5333,7 +5333,7 @@
         <x:v>subzone_brackwell_pumpkin_patch.mp3</x:v>
       </x:c>
       <x:c r="K44" s="1" t="n">
-        <x:v>6</x:v>
+        <x:v>7.7</x:v>
       </x:c>
       <x:c r="L44" s="1" t="str">
         <x:v>Audio exists</x:v>
@@ -5410,7 +5410,7 @@
         <x:v>subzone_crystal_lake.mp3</x:v>
       </x:c>
       <x:c r="K45" s="1" t="n">
-        <x:v>5</x:v>
+        <x:v>5.4</x:v>
       </x:c>
       <x:c r="L45" s="1" t="str">
         <x:v>Audio exists</x:v>
@@ -5487,7 +5487,7 @@
         <x:v>subzone_eastvale_logging_camp.mp3</x:v>
       </x:c>
       <x:c r="K46" s="1" t="n">
-        <x:v>5.5</x:v>
+        <x:v>7.1</x:v>
       </x:c>
       <x:c r="L46" s="1" t="str">
         <x:v>Audio exists</x:v>
@@ -5564,7 +5564,7 @@
         <x:v>subzone_echo_ridge_mine.mp3</x:v>
       </x:c>
       <x:c r="K47" s="1" t="n">
-        <x:v>5.4</x:v>
+        <x:v>6.1</x:v>
       </x:c>
       <x:c r="L47" s="1" t="str">
         <x:v>Audio exists</x:v>
@@ -5641,7 +5641,7 @@
         <x:v>subzone_fargodeep_mine.mp3</x:v>
       </x:c>
       <x:c r="K48" s="1" t="n">
-        <x:v>4.8</x:v>
+        <x:v>5.1</x:v>
       </x:c>
       <x:c r="L48" s="1" t="str">
         <x:v>Audio exists</x:v>
@@ -5718,7 +5718,7 @@
         <x:v>subzone_forests_edge.mp3</x:v>
       </x:c>
       <x:c r="K49" s="1" t="n">
-        <x:v>5.3</x:v>
+        <x:v>5.2</x:v>
       </x:c>
       <x:c r="L49" s="1" t="str">
         <x:v>Audio exists</x:v>
@@ -5795,7 +5795,7 @@
         <x:v>subzone_goldshire.mp3</x:v>
       </x:c>
       <x:c r="K50" s="1" t="n">
-        <x:v>5.8</x:v>
+        <x:v>7.3</x:v>
       </x:c>
       <x:c r="L50" s="1" t="str">
         <x:v>Audio exists</x:v>
@@ -5872,7 +5872,7 @@
         <x:v>subzone_goldtooths_den.mp3</x:v>
       </x:c>
       <x:c r="K51" s="1" t="n">
-        <x:v>5</x:v>
+        <x:v>5.5</x:v>
       </x:c>
       <x:c r="L51" s="1" t="str">
         <x:v>Audio exists</x:v>
@@ -5949,7 +5949,7 @@
         <x:v>subzone_hall_of_arms.mp3</x:v>
       </x:c>
       <x:c r="K52" s="1" t="n">
-        <x:v>5.2</x:v>
+        <x:v>7.2</x:v>
       </x:c>
       <x:c r="L52" s="1" t="str">
         <x:v>Audio exists</x:v>
@@ -6026,7 +6026,7 @@
         <x:v>subzone_heroes_vigil.mp3</x:v>
       </x:c>
       <x:c r="K53" s="1" t="n">
-        <x:v>5.1</x:v>
+        <x:v>5.5</x:v>
       </x:c>
       <x:c r="L53" s="1" t="str">
         <x:v>Audio exists</x:v>
@@ -6103,7 +6103,7 @@
         <x:v>subzone_hogger_hill.mp3</x:v>
       </x:c>
       <x:c r="K54" s="1" t="n">
-        <x:v>5.2</x:v>
+        <x:v>6.8</x:v>
       </x:c>
       <x:c r="L54" s="1" t="str">
         <x:v>Audio exists</x:v>
@@ -6180,7 +6180,7 @@
         <x:v>subzone_jasperlode_mine.mp3</x:v>
       </x:c>
       <x:c r="K55" s="1" t="n">
-        <x:v>5.3</x:v>
+        <x:v>6.9</x:v>
       </x:c>
       <x:c r="L55" s="1" t="str">
         <x:v>Audio exists</x:v>
@@ -6257,7 +6257,7 @@
         <x:v>subzone_jerods_landing.mp3</x:v>
       </x:c>
       <x:c r="K56" s="1" t="n">
-        <x:v>5.1</x:v>
+        <x:v>5.3</x:v>
       </x:c>
       <x:c r="L56" s="1" t="str">
         <x:v>Audio exists</x:v>
@@ -6334,7 +6334,7 @@
         <x:v>subzone_library_wing.mp3</x:v>
       </x:c>
       <x:c r="K57" s="1" t="n">
-        <x:v>5.6</x:v>
+        <x:v>5.8</x:v>
       </x:c>
       <x:c r="L57" s="1" t="str">
         <x:v>Audio exists</x:v>
@@ -6411,7 +6411,7 @@
         <x:v>subzone_lions_pride_inn.mp3</x:v>
       </x:c>
       <x:c r="K58" s="1" t="n">
-        <x:v>5.2</x:v>
+        <x:v>5.8</x:v>
       </x:c>
       <x:c r="L58" s="1" t="str">
         <x:v>Audio exists</x:v>
@@ -6488,7 +6488,7 @@
         <x:v>subzone_maclure_vineyards.mp3</x:v>
       </x:c>
       <x:c r="K59" s="1" t="n">
-        <x:v>5.4</x:v>
+        <x:v>6.2</x:v>
       </x:c>
       <x:c r="L59" s="1" t="str">
         <x:v>Audio exists</x:v>
@@ -6565,7 +6565,7 @@
         <x:v>subzone_main_hall.mp3</x:v>
       </x:c>
       <x:c r="K60" s="1" t="n">
-        <x:v>5</x:v>
+        <x:v>6</x:v>
       </x:c>
       <x:c r="L60" s="1" t="str">
         <x:v>Audio exists</x:v>
@@ -6719,7 +6719,7 @@
         <x:v>subzone_mirror_lake_orchard.mp3</x:v>
       </x:c>
       <x:c r="K62" s="1" t="n">
-        <x:v>5.1</x:v>
+        <x:v>6</x:v>
       </x:c>
       <x:c r="L62" s="1" t="str">
         <x:v>Audio exists</x:v>
@@ -6873,7 +6873,7 @@
         <x:v>subzone_northshire_valley.mp3</x:v>
       </x:c>
       <x:c r="K64" s="1" t="n">
-        <x:v>4.8</x:v>
+        <x:v>5</x:v>
       </x:c>
       <x:c r="L64" s="1" t="str">
         <x:v>Audio exists</x:v>
@@ -6950,7 +6950,7 @@
         <x:v>subzone_northshire_vineyards.mp3</x:v>
       </x:c>
       <x:c r="K65" s="1" t="n">
-        <x:v>5</x:v>
+        <x:v>5.4</x:v>
       </x:c>
       <x:c r="L65" s="1" t="str">
         <x:v>Audio exists</x:v>
@@ -7027,7 +7027,7 @@
         <x:v>subzone_ridgepoint_tower.mp3</x:v>
       </x:c>
       <x:c r="K66" s="1" t="n">
-        <x:v>5.8</x:v>
+        <x:v>6.5</x:v>
       </x:c>
       <x:c r="L66" s="1" t="str">
         <x:v>Audio exists</x:v>
@@ -7104,7 +7104,7 @@
         <x:v>subzone_stone_cairn_lake.mp3</x:v>
       </x:c>
       <x:c r="K67" s="1" t="n">
-        <x:v>5.5</x:v>
+        <x:v>6.1</x:v>
       </x:c>
       <x:c r="L67" s="1" t="str">
         <x:v>Audio exists</x:v>
@@ -7181,7 +7181,7 @@
         <x:v>subzone_stonefield_farm.mp3</x:v>
       </x:c>
       <x:c r="K68" s="1" t="n">
-        <x:v>5</x:v>
+        <x:v>5.1</x:v>
       </x:c>
       <x:c r="L68" s="1" t="str">
         <x:v>Audio exists</x:v>
@@ -7258,7 +7258,7 @@
         <x:v>subzone_stormwind_city.mp3</x:v>
       </x:c>
       <x:c r="K69" s="1" t="n">
-        <x:v>5.6</x:v>
+        <x:v>6.3</x:v>
       </x:c>
       <x:c r="L69" s="1" t="str">
         <x:v>Audio exists</x:v>
@@ -7335,7 +7335,7 @@
         <x:v>subzone_stormwind_gate.mp3</x:v>
       </x:c>
       <x:c r="K70" s="1" t="n">
-        <x:v>5.8</x:v>
+        <x:v>7.4</x:v>
       </x:c>
       <x:c r="L70" s="1" t="str">
         <x:v>Audio exists</x:v>
@@ -7412,7 +7412,7 @@
         <x:v>subzone_thunder_falls.mp3</x:v>
       </x:c>
       <x:c r="K71" s="1" t="n">
-        <x:v>4.7</x:v>
+        <x:v>4.8</x:v>
       </x:c>
       <x:c r="L71" s="1" t="str">
         <x:v>Audio exists</x:v>
@@ -7489,7 +7489,7 @@
         <x:v>subzone_tower_of_azora.mp3</x:v>
       </x:c>
       <x:c r="K72" s="1" t="n">
-        <x:v>5.5</x:v>
+        <x:v>6.2</x:v>
       </x:c>
       <x:c r="L72" s="1" t="str">
         <x:v>Audio exists</x:v>
@@ -7566,7 +7566,7 @@
         <x:v>subzone_westbrook_garrison.mp3</x:v>
       </x:c>
       <x:c r="K73" s="1" t="n">
-        <x:v>5.4</x:v>
+        <x:v>5.1</x:v>
       </x:c>
       <x:c r="L73" s="1" t="str">
         <x:v>Audio exists</x:v>
@@ -7643,7 +7643,7 @@
         <x:v>zone_intro_01.mp3</x:v>
       </x:c>
       <x:c r="K74" s="1" t="n">
-        <x:v>6.2</x:v>
+        <x:v>6.7</x:v>
       </x:c>
       <x:c r="L74" s="1" t="str">
         <x:v>Audio exists</x:v>
@@ -7720,7 +7720,7 @@
         <x:v>zone_intro_02.mp3</x:v>
       </x:c>
       <x:c r="K75" s="1" t="n">
-        <x:v>5.8</x:v>
+        <x:v>6.8</x:v>
       </x:c>
       <x:c r="L75" s="1" t="str">
         <x:v>Audio exists</x:v>
@@ -7874,7 +7874,7 @@
         <x:v>quest_accept_02.mp3</x:v>
       </x:c>
       <x:c r="K77" s="1" t="n">
-        <x:v>5.6</x:v>
+        <x:v>6.4</x:v>
       </x:c>
       <x:c r="L77" s="1" t="str">
         <x:v>Audio exists</x:v>
@@ -7951,7 +7951,7 @@
         <x:v>quest_accept_03.mp3</x:v>
       </x:c>
       <x:c r="K78" s="1" t="n">
-        <x:v>4.9</x:v>
+        <x:v>5.3</x:v>
       </x:c>
       <x:c r="L78" s="1" t="str">
         <x:v>Audio exists</x:v>
@@ -8028,7 +8028,7 @@
         <x:v>kill_01.mp3</x:v>
       </x:c>
       <x:c r="K79" s="1" t="n">
-        <x:v>3.4</x:v>
+        <x:v>2.6</x:v>
       </x:c>
       <x:c r="L79" s="1" t="str">
         <x:v>Audio exists</x:v>
@@ -8105,7 +8105,7 @@
         <x:v>kill_02.mp3</x:v>
       </x:c>
       <x:c r="K80" s="1" t="n">
-        <x:v>4.5</x:v>
+        <x:v>5.2</x:v>
       </x:c>
       <x:c r="L80" s="1" t="str">
         <x:v>Audio exists</x:v>
@@ -8182,7 +8182,7 @@
         <x:v>kill_03.mp3</x:v>
       </x:c>
       <x:c r="K81" s="1" t="n">
-        <x:v>4.2</x:v>
+        <x:v>3.9</x:v>
       </x:c>
       <x:c r="L81" s="1" t="str">
         <x:v>Audio exists</x:v>
@@ -8259,7 +8259,7 @@
         <x:v>idle_01.mp3</x:v>
       </x:c>
       <x:c r="K82" s="1" t="n">
-        <x:v>6</x:v>
+        <x:v>6.3</x:v>
       </x:c>
       <x:c r="L82" s="1" t="str">
         <x:v>Audio exists</x:v>
@@ -8336,7 +8336,7 @@
         <x:v>idle_02.mp3</x:v>
       </x:c>
       <x:c r="K83" s="1" t="n">
-        <x:v>6.4</x:v>
+        <x:v>6.1</x:v>
       </x:c>
       <x:c r="L83" s="1" t="str">
         <x:v>Audio exists</x:v>
@@ -8490,7 +8490,7 @@
         <x:v>level_up_01.mp3</x:v>
       </x:c>
       <x:c r="K85" s="1" t="n">
-        <x:v>4.7</x:v>
+        <x:v>5.5</x:v>
       </x:c>
       <x:c r="L85" s="1" t="str">
         <x:v>Audio exists</x:v>
@@ -8567,7 +8567,7 @@
         <x:v>level_up_02.mp3</x:v>
       </x:c>
       <x:c r="K86" s="1" t="n">
-        <x:v>4.7</x:v>
+        <x:v>4</x:v>
       </x:c>
       <x:c r="L86" s="1" t="str">
         <x:v>Audio exists</x:v>
@@ -8644,7 +8644,7 @@
         <x:v>summon_01.mp3</x:v>
       </x:c>
       <x:c r="K87" s="1" t="n">
-        <x:v>6.5</x:v>
+        <x:v>7.7</x:v>
       </x:c>
       <x:c r="L87" s="1" t="str">
         <x:v>Audio exists</x:v>
@@ -8721,7 +8721,7 @@
         <x:v>bond_02_01.mp3</x:v>
       </x:c>
       <x:c r="K88" s="1" t="n">
-        <x:v>5.6</x:v>
+        <x:v>5.5</x:v>
       </x:c>
       <x:c r="L88" s="1" t="str">
         <x:v>Audio exists</x:v>
@@ -8798,7 +8798,7 @@
         <x:v>bond_04_01.mp3</x:v>
       </x:c>
       <x:c r="K89" s="1" t="n">
-        <x:v>5.8</x:v>
+        <x:v>7.1</x:v>
       </x:c>
       <x:c r="L89" s="1" t="str">
         <x:v>Audio exists</x:v>
@@ -8875,7 +8875,7 @@
         <x:v>bond_06_01.mp3</x:v>
       </x:c>
       <x:c r="K90" s="1" t="n">
-        <x:v>6</x:v>
+        <x:v>6.2</x:v>
       </x:c>
       <x:c r="L90" s="1" t="str">
         <x:v>Audio exists</x:v>
@@ -8952,7 +8952,7 @@
         <x:v>bond_08_01.mp3</x:v>
       </x:c>
       <x:c r="K91" s="1" t="n">
-        <x:v>6</x:v>
+        <x:v>5.5</x:v>
       </x:c>
       <x:c r="L91" s="1" t="str">
         <x:v>Audio exists</x:v>
@@ -9029,7 +9029,7 @@
         <x:v>bond_10_01.mp3</x:v>
       </x:c>
       <x:c r="K92" s="1" t="n">
-        <x:v>6.3</x:v>
+        <x:v>6.9</x:v>
       </x:c>
       <x:c r="L92" s="1" t="str">
         <x:v>Audio exists</x:v>
@@ -9106,7 +9106,7 @@
         <x:v>romance_02_01.mp3</x:v>
       </x:c>
       <x:c r="K93" s="1" t="n">
-        <x:v>6.3</x:v>
+        <x:v>6.2</x:v>
       </x:c>
       <x:c r="L93" s="1" t="str">
         <x:v>Audio exists</x:v>
@@ -9183,7 +9183,7 @@
         <x:v>romance_04_01.mp3</x:v>
       </x:c>
       <x:c r="K94" s="1" t="n">
-        <x:v>6</x:v>
+        <x:v>5.9</x:v>
       </x:c>
       <x:c r="L94" s="1" t="str">
         <x:v>Audio exists</x:v>
@@ -9260,7 +9260,7 @@
         <x:v>romance_06_01.mp3</x:v>
       </x:c>
       <x:c r="K95" s="1" t="n">
-        <x:v>5.7</x:v>
+        <x:v>5.5</x:v>
       </x:c>
       <x:c r="L95" s="1" t="str">
         <x:v>Audio exists</x:v>
@@ -9337,7 +9337,7 @@
         <x:v>romance_08_01.mp3</x:v>
       </x:c>
       <x:c r="K96" s="1" t="n">
-        <x:v>6.1</x:v>
+        <x:v>5.7</x:v>
       </x:c>
       <x:c r="L96" s="1" t="str">
         <x:v>Audio exists</x:v>
@@ -9414,7 +9414,7 @@
         <x:v>romance_10_01.mp3</x:v>
       </x:c>
       <x:c r="K97" s="1" t="n">
-        <x:v>6.2</x:v>
+        <x:v>7.2</x:v>
       </x:c>
       <x:c r="L97" s="1" t="str">
         <x:v>Audio exists</x:v>
@@ -9491,7 +9491,7 @@
         <x:v>romance_not_ready_01.mp3</x:v>
       </x:c>
       <x:c r="K98" s="1" t="n">
-        <x:v>5.8</x:v>
+        <x:v>6</x:v>
       </x:c>
       <x:c r="L98" s="1" t="str">
         <x:v>Audio exists</x:v>
@@ -9568,7 +9568,7 @@
         <x:v>romance_repeat_01.mp3</x:v>
       </x:c>
       <x:c r="K99" s="1" t="n">
-        <x:v>4.8</x:v>
+        <x:v>4.3</x:v>
       </x:c>
       <x:c r="L99" s="1" t="str">
         <x:v>Audio exists</x:v>
@@ -9645,7 +9645,7 @@
         <x:v>romance_stop_01.mp3</x:v>
       </x:c>
       <x:c r="K100" s="1" t="n">
-        <x:v>5.8</x:v>
+        <x:v>6.6</x:v>
       </x:c>
       <x:c r="L100" s="1" t="str">
         <x:v>Audio exists</x:v>
@@ -9722,7 +9722,7 @@
         <x:v>quest_complete_01.mp3</x:v>
       </x:c>
       <x:c r="K101" s="1" t="n">
-        <x:v>5</x:v>
+        <x:v>5.4</x:v>
       </x:c>
       <x:c r="L101" s="1" t="str">
         <x:v>Audio exists</x:v>
@@ -9799,7 +9799,7 @@
         <x:v>quest_complete_02.mp3</x:v>
       </x:c>
       <x:c r="K102" s="1" t="n">
-        <x:v>5.2</x:v>
+        <x:v>4.6</x:v>
       </x:c>
       <x:c r="L102" s="1" t="str">
         <x:v>Audio exists</x:v>
@@ -9876,7 +9876,7 @@
         <x:v>quest_complete_03.mp3</x:v>
       </x:c>
       <x:c r="K103" s="1" t="n">
-        <x:v>5.1</x:v>
+        <x:v>5</x:v>
       </x:c>
       <x:c r="L103" s="1" t="str">
         <x:v>Audio exists</x:v>
@@ -9953,7 +9953,7 @@
         <x:v>bond_kill_02.mp3</x:v>
       </x:c>
       <x:c r="K104" s="1" t="n">
-        <x:v>4.8</x:v>
+        <x:v>4</x:v>
       </x:c>
       <x:c r="L104" s="1" t="str">
         <x:v>Audio exists</x:v>
@@ -10030,7 +10030,7 @@
         <x:v>bond_kill_04.mp3</x:v>
       </x:c>
       <x:c r="K105" s="1" t="n">
-        <x:v>5.2</x:v>
+        <x:v>4.7</x:v>
       </x:c>
       <x:c r="L105" s="1" t="str">
         <x:v>Audio exists</x:v>
@@ -10107,7 +10107,7 @@
         <x:v>bond_kill_06.mp3</x:v>
       </x:c>
       <x:c r="K106" s="1" t="n">
-        <x:v>4.4</x:v>
+        <x:v>3.2</x:v>
       </x:c>
       <x:c r="L106" s="1" t="str">
         <x:v>Audio exists</x:v>
@@ -10184,7 +10184,7 @@
         <x:v>bond_kill_08.mp3</x:v>
       </x:c>
       <x:c r="K107" s="1" t="n">
-        <x:v>4.6</x:v>
+        <x:v>3.4</x:v>
       </x:c>
       <x:c r="L107" s="1" t="str">
         <x:v>Audio exists</x:v>
@@ -10261,7 +10261,7 @@
         <x:v>bond_kill_10.mp3</x:v>
       </x:c>
       <x:c r="K108" s="1" t="n">
-        <x:v>4.5</x:v>
+        <x:v>3.8</x:v>
       </x:c>
       <x:c r="L108" s="1" t="str">
         <x:v>Audio exists</x:v>
@@ -10338,7 +10338,7 @@
         <x:v>bond_idle_01.mp3</x:v>
       </x:c>
       <x:c r="K109" s="1" t="n">
-        <x:v>5</x:v>
+        <x:v>4.5</x:v>
       </x:c>
       <x:c r="L109" s="1" t="str">
         <x:v>Audio exists</x:v>
@@ -10415,7 +10415,7 @@
         <x:v>bond_idle_03.mp3</x:v>
       </x:c>
       <x:c r="K110" s="1" t="n">
-        <x:v>5.6</x:v>
+        <x:v>5.9</x:v>
       </x:c>
       <x:c r="L110" s="1" t="str">
         <x:v>Audio exists</x:v>
@@ -10492,7 +10492,7 @@
         <x:v>bond_idle_05.mp3</x:v>
       </x:c>
       <x:c r="K111" s="1" t="n">
-        <x:v>5.7</x:v>
+        <x:v>5</x:v>
       </x:c>
       <x:c r="L111" s="1" t="str">
         <x:v>Audio exists</x:v>
@@ -10569,7 +10569,7 @@
         <x:v>bond_idle_07.mp3</x:v>
       </x:c>
       <x:c r="K112" s="1" t="n">
-        <x:v>4.8</x:v>
+        <x:v>3.4</x:v>
       </x:c>
       <x:c r="L112" s="1" t="str">
         <x:v>Audio exists</x:v>
@@ -10646,7 +10646,7 @@
         <x:v>bond_idle_09.mp3</x:v>
       </x:c>
       <x:c r="K113" s="1" t="n">
-        <x:v>5.7</x:v>
+        <x:v>4.6</x:v>
       </x:c>
       <x:c r="L113" s="1" t="str">
         <x:v>Audio exists</x:v>
@@ -10800,7 +10800,7 @@
         <x:v>death_01.mp3</x:v>
       </x:c>
       <x:c r="K115" s="1" t="n">
-        <x:v>5.8</x:v>
+        <x:v>4.6</x:v>
       </x:c>
       <x:c r="L115" s="1" t="str">
         <x:v>Audio exists</x:v>
@@ -10877,7 +10877,7 @@
         <x:v>subzone_brackwell_pumpkin_patch.mp3</x:v>
       </x:c>
       <x:c r="K116" s="1" t="n">
-        <x:v>5.4</x:v>
+        <x:v>4.9</x:v>
       </x:c>
       <x:c r="L116" s="1" t="str">
         <x:v>Audio exists</x:v>
@@ -10954,7 +10954,7 @@
         <x:v>subzone_crystal_lake.mp3</x:v>
       </x:c>
       <x:c r="K117" s="1" t="n">
-        <x:v>4.8</x:v>
+        <x:v>4.9</x:v>
       </x:c>
       <x:c r="L117" s="1" t="str">
         <x:v>Audio exists</x:v>
@@ -11031,7 +11031,7 @@
         <x:v>subzone_eastvale_logging_camp.mp3</x:v>
       </x:c>
       <x:c r="K118" s="1" t="n">
-        <x:v>5.7</x:v>
+        <x:v>5.3</x:v>
       </x:c>
       <x:c r="L118" s="1" t="str">
         <x:v>Audio exists</x:v>
@@ -11108,7 +11108,7 @@
         <x:v>subzone_echo_ridge_mine.mp3</x:v>
       </x:c>
       <x:c r="K119" s="1" t="n">
-        <x:v>5.1</x:v>
+        <x:v>4.9</x:v>
       </x:c>
       <x:c r="L119" s="1" t="str">
         <x:v>Audio exists</x:v>
@@ -11185,7 +11185,7 @@
         <x:v>subzone_fargodeep_mine.mp3</x:v>
       </x:c>
       <x:c r="K120" s="1" t="n">
-        <x:v>5</x:v>
+        <x:v>5.4</x:v>
       </x:c>
       <x:c r="L120" s="1" t="str">
         <x:v>Audio exists</x:v>
@@ -11262,7 +11262,7 @@
         <x:v>subzone_forests_edge.mp3</x:v>
       </x:c>
       <x:c r="K121" s="1" t="n">
-        <x:v>4.6</x:v>
+        <x:v>4</x:v>
       </x:c>
       <x:c r="L121" s="1" t="str">
         <x:v>Audio exists</x:v>
@@ -11339,7 +11339,7 @@
         <x:v>subzone_goldshire.mp3</x:v>
       </x:c>
       <x:c r="K122" s="1" t="n">
-        <x:v>5.3</x:v>
+        <x:v>5.4</x:v>
       </x:c>
       <x:c r="L122" s="1" t="str">
         <x:v>Audio exists</x:v>
@@ -11416,7 +11416,7 @@
         <x:v>subzone_goldtooths_den.mp3</x:v>
       </x:c>
       <x:c r="K123" s="1" t="n">
-        <x:v>5.5</x:v>
+        <x:v>7.2</x:v>
       </x:c>
       <x:c r="L123" s="1" t="str">
         <x:v>Audio exists</x:v>
@@ -11493,7 +11493,7 @@
         <x:v>subzone_hall_of_arms.mp3</x:v>
       </x:c>
       <x:c r="K124" s="1" t="n">
-        <x:v>5</x:v>
+        <x:v>4.7</x:v>
       </x:c>
       <x:c r="L124" s="1" t="str">
         <x:v>Audio exists</x:v>
@@ -11570,7 +11570,7 @@
         <x:v>subzone_heroes_vigil.mp3</x:v>
       </x:c>
       <x:c r="K125" s="1" t="n">
-        <x:v>5.8</x:v>
+        <x:v>6</x:v>
       </x:c>
       <x:c r="L125" s="1" t="str">
         <x:v>Audio exists</x:v>
@@ -11647,7 +11647,7 @@
         <x:v>subzone_hogger_hill.mp3</x:v>
       </x:c>
       <x:c r="K126" s="1" t="n">
-        <x:v>5.1</x:v>
+        <x:v>5.8</x:v>
       </x:c>
       <x:c r="L126" s="1" t="str">
         <x:v>Audio exists</x:v>
@@ -11724,7 +11724,7 @@
         <x:v>subzone_jasperlode_mine.mp3</x:v>
       </x:c>
       <x:c r="K127" s="1" t="n">
-        <x:v>5.4</x:v>
+        <x:v>5.2</x:v>
       </x:c>
       <x:c r="L127" s="1" t="str">
         <x:v>Audio exists</x:v>
@@ -11801,7 +11801,7 @@
         <x:v>subzone_jerods_landing.mp3</x:v>
       </x:c>
       <x:c r="K128" s="1" t="n">
-        <x:v>4.8</x:v>
+        <x:v>4.1</x:v>
       </x:c>
       <x:c r="L128" s="1" t="str">
         <x:v>Audio exists</x:v>
@@ -11878,7 +11878,7 @@
         <x:v>subzone_library_wing.mp3</x:v>
       </x:c>
       <x:c r="K129" s="1" t="n">
-        <x:v>4.6</x:v>
+        <x:v>3.6</x:v>
       </x:c>
       <x:c r="L129" s="1" t="str">
         <x:v>Audio exists</x:v>
@@ -11955,7 +11955,7 @@
         <x:v>subzone_lions_pride_inn.mp3</x:v>
       </x:c>
       <x:c r="K130" s="1" t="n">
-        <x:v>5.1</x:v>
+        <x:v>4.6</x:v>
       </x:c>
       <x:c r="L130" s="1" t="str">
         <x:v>Audio exists</x:v>
@@ -12032,7 +12032,7 @@
         <x:v>subzone_maclure_vineyards.mp3</x:v>
       </x:c>
       <x:c r="K131" s="1" t="n">
-        <x:v>5.5</x:v>
+        <x:v>5.7</x:v>
       </x:c>
       <x:c r="L131" s="1" t="str">
         <x:v>Audio exists</x:v>
@@ -12263,7 +12263,7 @@
         <x:v>subzone_mirror_lake_orchard.mp3</x:v>
       </x:c>
       <x:c r="K134" s="1" t="n">
-        <x:v>5</x:v>
+        <x:v>4.1</x:v>
       </x:c>
       <x:c r="L134" s="1" t="str">
         <x:v>Audio exists</x:v>
@@ -12340,7 +12340,7 @@
         <x:v>subzone_northshire_abbey.mp3</x:v>
       </x:c>
       <x:c r="K135" s="1" t="n">
-        <x:v>5.9</x:v>
+        <x:v>5.3</x:v>
       </x:c>
       <x:c r="L135" s="1" t="str">
         <x:v>Audio exists</x:v>
@@ -12417,7 +12417,7 @@
         <x:v>subzone_northshire_valley.mp3</x:v>
       </x:c>
       <x:c r="K136" s="1" t="n">
-        <x:v>5.6</x:v>
+        <x:v>4.9</x:v>
       </x:c>
       <x:c r="L136" s="1" t="str">
         <x:v>Audio exists</x:v>
@@ -12494,7 +12494,7 @@
         <x:v>subzone_northshire_vineyards.mp3</x:v>
       </x:c>
       <x:c r="K137" s="1" t="n">
-        <x:v>5.1</x:v>
+        <x:v>4.6</x:v>
       </x:c>
       <x:c r="L137" s="1" t="str">
         <x:v>Audio exists</x:v>
@@ -12571,7 +12571,7 @@
         <x:v>subzone_ridgepoint_tower.mp3</x:v>
       </x:c>
       <x:c r="K138" s="1" t="n">
-        <x:v>5</x:v>
+        <x:v>4.8</x:v>
       </x:c>
       <x:c r="L138" s="1" t="str">
         <x:v>Audio exists</x:v>
@@ -12648,7 +12648,7 @@
         <x:v>subzone_stone_cairn_lake.mp3</x:v>
       </x:c>
       <x:c r="K139" s="1" t="n">
-        <x:v>4.7</x:v>
+        <x:v>3.3</x:v>
       </x:c>
       <x:c r="L139" s="1" t="str">
         <x:v>Audio exists</x:v>
@@ -12725,7 +12725,7 @@
         <x:v>subzone_stonefield_farm.mp3</x:v>
       </x:c>
       <x:c r="K140" s="1" t="n">
-        <x:v>4.9</x:v>
+        <x:v>4.1</x:v>
       </x:c>
       <x:c r="L140" s="1" t="str">
         <x:v>Audio exists</x:v>
@@ -12802,7 +12802,7 @@
         <x:v>subzone_stormwind_city.mp3</x:v>
       </x:c>
       <x:c r="K141" s="1" t="n">
-        <x:v>5.5</x:v>
+        <x:v>7.5</x:v>
       </x:c>
       <x:c r="L141" s="1" t="str">
         <x:v>Audio exists</x:v>
@@ -12879,7 +12879,7 @@
         <x:v>subzone_stormwind_gate.mp3</x:v>
       </x:c>
       <x:c r="K142" s="1" t="n">
-        <x:v>5</x:v>
+        <x:v>4.3</x:v>
       </x:c>
       <x:c r="L142" s="1" t="str">
         <x:v>Audio exists</x:v>
@@ -12956,7 +12956,7 @@
         <x:v>subzone_thunder_falls.mp3</x:v>
       </x:c>
       <x:c r="K143" s="1" t="n">
-        <x:v>5</x:v>
+        <x:v>4.6</x:v>
       </x:c>
       <x:c r="L143" s="1" t="str">
         <x:v>Audio exists</x:v>
@@ -13033,7 +13033,7 @@
         <x:v>subzone_tower_of_azora.mp3</x:v>
       </x:c>
       <x:c r="K144" s="1" t="n">
-        <x:v>5.8</x:v>
+        <x:v>6.6</x:v>
       </x:c>
       <x:c r="L144" s="1" t="str">
         <x:v>Audio exists</x:v>
@@ -13110,7 +13110,7 @@
         <x:v>subzone_westbrook_garrison.mp3</x:v>
       </x:c>
       <x:c r="K145" s="1" t="n">
-        <x:v>4.9</x:v>
+        <x:v>4.5</x:v>
       </x:c>
       <x:c r="L145" s="1" t="str">
         <x:v>Audio exists</x:v>
@@ -13187,7 +13187,7 @@
         <x:v>zone_intro_01.mp3</x:v>
       </x:c>
       <x:c r="K146" s="1" t="n">
-        <x:v>6.2</x:v>
+        <x:v>7.3</x:v>
       </x:c>
       <x:c r="L146" s="1" t="str">
         <x:v>Audio exists</x:v>
@@ -13262,7 +13262,7 @@
         <x:v>zone_intro_02.mp3</x:v>
       </x:c>
       <x:c r="K147" s="1" t="n">
-        <x:v>6.4</x:v>
+        <x:v>9.6</x:v>
       </x:c>
       <x:c r="L147" s="1" t="str">
         <x:v>Audio exists</x:v>
@@ -13337,7 +13337,7 @@
         <x:v>quest_accept_01.mp3</x:v>
       </x:c>
       <x:c r="K148" s="1" t="n">
-        <x:v>6.2</x:v>
+        <x:v>8.9</x:v>
       </x:c>
       <x:c r="L148" s="1" t="str">
         <x:v>Audio exists</x:v>
@@ -13412,7 +13412,7 @@
         <x:v>quest_accept_02.mp3</x:v>
       </x:c>
       <x:c r="K149" s="1" t="n">
-        <x:v>6.3</x:v>
+        <x:v>9.4</x:v>
       </x:c>
       <x:c r="L149" s="1" t="str">
         <x:v>Audio exists</x:v>
@@ -13487,7 +13487,7 @@
         <x:v>quest_accept_03.mp3</x:v>
       </x:c>
       <x:c r="K150" s="1" t="n">
-        <x:v>5.2</x:v>
+        <x:v>6.9</x:v>
       </x:c>
       <x:c r="L150" s="1" t="str">
         <x:v>Audio exists</x:v>
@@ -13562,7 +13562,7 @@
         <x:v>kill_01.mp3</x:v>
       </x:c>
       <x:c r="K151" s="1" t="n">
-        <x:v>3.7</x:v>
+        <x:v>5.1</x:v>
       </x:c>
       <x:c r="L151" s="1" t="str">
         <x:v>Audio exists</x:v>
@@ -13637,7 +13637,7 @@
         <x:v>kill_02.mp3</x:v>
       </x:c>
       <x:c r="K152" s="1" t="n">
-        <x:v>4.6</x:v>
+        <x:v>6.7</x:v>
       </x:c>
       <x:c r="L152" s="1" t="str">
         <x:v>Audio exists</x:v>
@@ -13712,7 +13712,7 @@
         <x:v>kill_03.mp3</x:v>
       </x:c>
       <x:c r="K153" s="1" t="n">
-        <x:v>4.5</x:v>
+        <x:v>7.1</x:v>
       </x:c>
       <x:c r="L153" s="1" t="str">
         <x:v>Audio exists</x:v>
@@ -13787,7 +13787,7 @@
         <x:v>idle_01.mp3</x:v>
       </x:c>
       <x:c r="K154" s="1" t="n">
-        <x:v>5.8</x:v>
+        <x:v>7.5</x:v>
       </x:c>
       <x:c r="L154" s="1" t="str">
         <x:v>Audio exists</x:v>
@@ -13862,7 +13862,7 @@
         <x:v>idle_02.mp3</x:v>
       </x:c>
       <x:c r="K155" s="1" t="n">
-        <x:v>6.1</x:v>
+        <x:v>7.9</x:v>
       </x:c>
       <x:c r="L155" s="1" t="str">
         <x:v>Audio exists</x:v>
@@ -13937,7 +13937,7 @@
         <x:v>idle_03.mp3</x:v>
       </x:c>
       <x:c r="K156" s="1" t="n">
-        <x:v>5.4</x:v>
+        <x:v>7</x:v>
       </x:c>
       <x:c r="L156" s="1" t="str">
         <x:v>Audio exists</x:v>
@@ -14012,7 +14012,7 @@
         <x:v>level_up_01.mp3</x:v>
       </x:c>
       <x:c r="K157" s="1" t="n">
-        <x:v>5.4</x:v>
+        <x:v>8.7</x:v>
       </x:c>
       <x:c r="L157" s="1" t="str">
         <x:v>Audio exists</x:v>
@@ -14087,7 +14087,7 @@
         <x:v>level_up_02.mp3</x:v>
       </x:c>
       <x:c r="K158" s="1" t="n">
-        <x:v>4.7</x:v>
+        <x:v>7.3</x:v>
       </x:c>
       <x:c r="L158" s="1" t="str">
         <x:v>Audio exists</x:v>
@@ -14162,7 +14162,7 @@
         <x:v>summon_01.mp3</x:v>
       </x:c>
       <x:c r="K159" s="1" t="n">
-        <x:v>6</x:v>
+        <x:v>8.7</x:v>
       </x:c>
       <x:c r="L159" s="1" t="str">
         <x:v>Audio exists</x:v>
@@ -14237,7 +14237,7 @@
         <x:v>bond_02_01.mp3</x:v>
       </x:c>
       <x:c r="K160" s="1" t="n">
-        <x:v>5.4</x:v>
+        <x:v>5.8</x:v>
       </x:c>
       <x:c r="L160" s="1" t="str">
         <x:v>Audio exists</x:v>
@@ -14314,7 +14314,7 @@
         <x:v>bond_04_01.mp3</x:v>
       </x:c>
       <x:c r="K161" s="1" t="n">
-        <x:v>5.4</x:v>
+        <x:v>5.1</x:v>
       </x:c>
       <x:c r="L161" s="1" t="str">
         <x:v>Audio exists</x:v>
@@ -14391,7 +14391,7 @@
         <x:v>bond_06_01.mp3</x:v>
       </x:c>
       <x:c r="K162" s="1" t="n">
-        <x:v>6.2</x:v>
+        <x:v>6.5</x:v>
       </x:c>
       <x:c r="L162" s="1" t="str">
         <x:v>Audio exists</x:v>
@@ -14468,7 +14468,7 @@
         <x:v>bond_08_01.mp3</x:v>
       </x:c>
       <x:c r="K163" s="1" t="n">
-        <x:v>5.7</x:v>
+        <x:v>5.9</x:v>
       </x:c>
       <x:c r="L163" s="1" t="str">
         <x:v>Audio exists</x:v>
@@ -14545,7 +14545,7 @@
         <x:v>bond_10_01.mp3</x:v>
       </x:c>
       <x:c r="K164" s="1" t="n">
-        <x:v>6.5</x:v>
+        <x:v>6.3</x:v>
       </x:c>
       <x:c r="L164" s="1" t="str">
         <x:v>Audio exists</x:v>
@@ -14622,7 +14622,7 @@
         <x:v>romance_02_01.mp3</x:v>
       </x:c>
       <x:c r="K165" s="1" t="n">
-        <x:v>4.8</x:v>
+        <x:v>5.3</x:v>
       </x:c>
       <x:c r="L165" s="1" t="str">
         <x:v>Audio exists</x:v>
@@ -14699,7 +14699,7 @@
         <x:v>romance_04_01.mp3</x:v>
       </x:c>
       <x:c r="K166" s="1" t="n">
-        <x:v>5</x:v>
+        <x:v>4.1</x:v>
       </x:c>
       <x:c r="L166" s="1" t="str">
         <x:v>Audio exists</x:v>
@@ -14853,7 +14853,7 @@
         <x:v>romance_08_01.mp3</x:v>
       </x:c>
       <x:c r="K168" s="1" t="n">
-        <x:v>5.7</x:v>
+        <x:v>5.3</x:v>
       </x:c>
       <x:c r="L168" s="1" t="str">
         <x:v>Audio exists</x:v>
@@ -14930,7 +14930,7 @@
         <x:v>romance_10_01.mp3</x:v>
       </x:c>
       <x:c r="K169" s="1" t="n">
-        <x:v>5.8</x:v>
+        <x:v>5.5</x:v>
       </x:c>
       <x:c r="L169" s="1" t="str">
         <x:v>Audio exists</x:v>
@@ -15007,7 +15007,7 @@
         <x:v>romance_not_ready_01.mp3</x:v>
       </x:c>
       <x:c r="K170" s="1" t="n">
-        <x:v>6</x:v>
+        <x:v>6.2</x:v>
       </x:c>
       <x:c r="L170" s="1" t="str">
         <x:v>Audio exists</x:v>
@@ -15084,7 +15084,7 @@
         <x:v>romance_repeat_01.mp3</x:v>
       </x:c>
       <x:c r="K171" s="1" t="n">
-        <x:v>4.5</x:v>
+        <x:v>3.1</x:v>
       </x:c>
       <x:c r="L171" s="1" t="str">
         <x:v>Audio exists</x:v>
@@ -15161,7 +15161,7 @@
         <x:v>romance_stop_01.mp3</x:v>
       </x:c>
       <x:c r="K172" s="1" t="n">
-        <x:v>5</x:v>
+        <x:v>4.4</x:v>
       </x:c>
       <x:c r="L172" s="1" t="str">
         <x:v>Audio exists</x:v>
@@ -15238,7 +15238,7 @@
         <x:v>quest_complete_01.mp3</x:v>
       </x:c>
       <x:c r="K173" s="1" t="n">
-        <x:v>4.6</x:v>
+        <x:v>3.5</x:v>
       </x:c>
       <x:c r="L173" s="1" t="str">
         <x:v>Audio exists</x:v>
@@ -15315,7 +15315,7 @@
         <x:v>quest_complete_02.mp3</x:v>
       </x:c>
       <x:c r="K174" s="1" t="n">
-        <x:v>5</x:v>
+        <x:v>4.4</x:v>
       </x:c>
       <x:c r="L174" s="1" t="str">
         <x:v>Audio exists</x:v>
@@ -15392,7 +15392,7 @@
         <x:v>quest_complete_03.mp3</x:v>
       </x:c>
       <x:c r="K175" s="1" t="n">
-        <x:v>5.4</x:v>
+        <x:v>4.4</x:v>
       </x:c>
       <x:c r="L175" s="1" t="str">
         <x:v>Audio exists</x:v>
@@ -15469,7 +15469,7 @@
         <x:v>bond_kill_02.mp3</x:v>
       </x:c>
       <x:c r="K176" s="1" t="n">
-        <x:v>4.2</x:v>
+        <x:v>3.4</x:v>
       </x:c>
       <x:c r="L176" s="1" t="str">
         <x:v>Audio exists</x:v>
@@ -15546,7 +15546,7 @@
         <x:v>bond_kill_04.mp3</x:v>
       </x:c>
       <x:c r="K177" s="1" t="n">
-        <x:v>4.6</x:v>
+        <x:v>3.9</x:v>
       </x:c>
       <x:c r="L177" s="1" t="str">
         <x:v>Audio exists</x:v>
@@ -15623,7 +15623,7 @@
         <x:v>bond_kill_06.mp3</x:v>
       </x:c>
       <x:c r="K178" s="1" t="n">
-        <x:v>5.6</x:v>
+        <x:v>6.1</x:v>
       </x:c>
       <x:c r="L178" s="1" t="str">
         <x:v>Audio exists</x:v>
@@ -15700,7 +15700,7 @@
         <x:v>bond_kill_08.mp3</x:v>
       </x:c>
       <x:c r="K179" s="1" t="n">
-        <x:v>5.3</x:v>
+        <x:v>4.2</x:v>
       </x:c>
       <x:c r="L179" s="1" t="str">
         <x:v>Audio exists</x:v>
@@ -15777,7 +15777,7 @@
         <x:v>bond_kill_10.mp3</x:v>
       </x:c>
       <x:c r="K180" s="1" t="n">
-        <x:v>4.4</x:v>
+        <x:v>3.9</x:v>
       </x:c>
       <x:c r="L180" s="1" t="str">
         <x:v>Audio exists</x:v>
@@ -15854,7 +15854,7 @@
         <x:v>bond_idle_01.mp3</x:v>
       </x:c>
       <x:c r="K181" s="1" t="n">
-        <x:v>5.5</x:v>
+        <x:v>5</x:v>
       </x:c>
       <x:c r="L181" s="1" t="str">
         <x:v>Audio exists</x:v>
@@ -15931,7 +15931,7 @@
         <x:v>bond_idle_03.mp3</x:v>
       </x:c>
       <x:c r="K182" s="1" t="n">
-        <x:v>5</x:v>
+        <x:v>4.9</x:v>
       </x:c>
       <x:c r="L182" s="1" t="str">
         <x:v>Audio exists</x:v>
@@ -16008,7 +16008,7 @@
         <x:v>bond_idle_05.mp3</x:v>
       </x:c>
       <x:c r="K183" s="1" t="n">
-        <x:v>5.3</x:v>
+        <x:v>4.8</x:v>
       </x:c>
       <x:c r="L183" s="1" t="str">
         <x:v>Audio exists</x:v>
@@ -16085,7 +16085,7 @@
         <x:v>bond_idle_07.mp3</x:v>
       </x:c>
       <x:c r="K184" s="1" t="n">
-        <x:v>4.8</x:v>
+        <x:v>5.1</x:v>
       </x:c>
       <x:c r="L184" s="1" t="str">
         <x:v>Audio exists</x:v>
@@ -16162,7 +16162,7 @@
         <x:v>bond_idle_09.mp3</x:v>
       </x:c>
       <x:c r="K185" s="1" t="n">
-        <x:v>5.1</x:v>
+        <x:v>4.2</x:v>
       </x:c>
       <x:c r="L185" s="1" t="str">
         <x:v>Audio exists</x:v>
@@ -16239,7 +16239,7 @@
         <x:v>low_health_01.mp3</x:v>
       </x:c>
       <x:c r="K186" s="1" t="n">
-        <x:v>3.7</x:v>
+        <x:v>2.7</x:v>
       </x:c>
       <x:c r="L186" s="1" t="str">
         <x:v>Audio exists</x:v>
@@ -16316,7 +16316,7 @@
         <x:v>death_01.mp3</x:v>
       </x:c>
       <x:c r="K187" s="1" t="n">
-        <x:v>5</x:v>
+        <x:v>4.3</x:v>
       </x:c>
       <x:c r="L187" s="1" t="str">
         <x:v>Audio exists</x:v>
@@ -16393,7 +16393,7 @@
         <x:v>subzone_alexston_farmstead.mp3</x:v>
       </x:c>
       <x:c r="K188" s="1" t="n">
-        <x:v>5.4</x:v>
+        <x:v>5</x:v>
       </x:c>
       <x:c r="L188" s="1" t="str">
         <x:v>Audio exists</x:v>
@@ -16470,7 +16470,7 @@
         <x:v>subzone_dagger_hills.mp3</x:v>
       </x:c>
       <x:c r="K189" s="1" t="n">
-        <x:v>4.8</x:v>
+        <x:v>4.6</x:v>
       </x:c>
       <x:c r="L189" s="1" t="str">
         <x:v>Audio exists</x:v>
@@ -16547,7 +16547,7 @@
         <x:v>subzone_dawning_wood_catacombs.mp3</x:v>
       </x:c>
       <x:c r="K190" s="1" t="n">
-        <x:v>5.1</x:v>
+        <x:v>5.2</x:v>
       </x:c>
       <x:c r="L190" s="1" t="str">
         <x:v>Audio exists</x:v>
@@ -16624,7 +16624,7 @@
         <x:v>subzone_dead_acre.mp3</x:v>
       </x:c>
       <x:c r="K191" s="1" t="n">
-        <x:v>4.8</x:v>
+        <x:v>4.4</x:v>
       </x:c>
       <x:c r="L191" s="1" t="str">
         <x:v>Audio exists</x:v>
@@ -16701,7 +16701,7 @@
         <x:v>subzone_demonts_place.mp3</x:v>
       </x:c>
       <x:c r="K192" s="1" t="n">
-        <x:v>5</x:v>
+        <x:v>4.5</x:v>
       </x:c>
       <x:c r="L192" s="1" t="str">
         <x:v>Audio exists</x:v>
@@ -16778,7 +16778,7 @@
         <x:v>subzone_dust_plains.mp3</x:v>
       </x:c>
       <x:c r="K193" s="1" t="n">
-        <x:v>4.8</x:v>
+        <x:v>3.8</x:v>
       </x:c>
       <x:c r="L193" s="1" t="str">
         <x:v>Audio exists</x:v>
@@ -16855,7 +16855,7 @@
         <x:v>subzone_furlbrows_pumpkin_farm.mp3</x:v>
       </x:c>
       <x:c r="K194" s="1" t="n">
-        <x:v>5.3</x:v>
+        <x:v>4.8</x:v>
       </x:c>
       <x:c r="L194" s="1" t="str">
         <x:v>Audio exists</x:v>
@@ -16932,7 +16932,7 @@
         <x:v>subzone_gold_coast_quarry.mp3</x:v>
       </x:c>
       <x:c r="K195" s="1" t="n">
-        <x:v>5.6</x:v>
+        <x:v>6.1</x:v>
       </x:c>
       <x:c r="L195" s="1" t="str">
         <x:v>Audio exists</x:v>
@@ -17009,7 +17009,7 @@
         <x:v>subzone_jansen_stead.mp3</x:v>
       </x:c>
       <x:c r="K196" s="1" t="n">
-        <x:v>5.2</x:v>
+        <x:v>4.3</x:v>
       </x:c>
       <x:c r="L196" s="1" t="str">
         <x:v>Audio exists</x:v>
@@ -17086,7 +17086,7 @@
         <x:v>subzone_jangolode_mine.mp3</x:v>
       </x:c>
       <x:c r="K197" s="1" t="n">
-        <x:v>5</x:v>
+        <x:v>4.8</x:v>
       </x:c>
       <x:c r="L197" s="1" t="str">
         <x:v>Audio exists</x:v>
@@ -17163,7 +17163,7 @@
         <x:v>subzone_molsen_farm.mp3</x:v>
       </x:c>
       <x:c r="K198" s="1" t="n">
-        <x:v>4.5</x:v>
+        <x:v>4.1</x:v>
       </x:c>
       <x:c r="L198" s="1" t="str">
         <x:v>Audio exists</x:v>
@@ -17240,7 +17240,7 @@
         <x:v>subzone_moonbrook.mp3</x:v>
       </x:c>
       <x:c r="K199" s="1" t="n">
-        <x:v>4.7</x:v>
+        <x:v>4.3</x:v>
       </x:c>
       <x:c r="L199" s="1" t="str">
         <x:v>Audio exists</x:v>
@@ -17317,7 +17317,7 @@
         <x:v>subzone_raging_chasm.mp3</x:v>
       </x:c>
       <x:c r="K200" s="1" t="n">
-        <x:v>5.2</x:v>
+        <x:v>4.4</x:v>
       </x:c>
       <x:c r="L200" s="1" t="str">
         <x:v>Audio exists</x:v>
@@ -17394,7 +17394,7 @@
         <x:v>subzone_saldeans_farm.mp3</x:v>
       </x:c>
       <x:c r="K201" s="1" t="n">
-        <x:v>4.9</x:v>
+        <x:v>4.3</x:v>
       </x:c>
       <x:c r="L201" s="1" t="str">
         <x:v>Audio exists</x:v>
@@ -17471,7 +17471,7 @@
         <x:v>subzone_sentinel_hill.mp3</x:v>
       </x:c>
       <x:c r="K202" s="1" t="n">
-        <x:v>5.1</x:v>
+        <x:v>4.5</x:v>
       </x:c>
       <x:c r="L202" s="1" t="str">
         <x:v>Audio exists</x:v>
@@ -17548,7 +17548,7 @@
         <x:v>subzone_shattered_strand.mp3</x:v>
       </x:c>
       <x:c r="K203" s="1" t="n">
-        <x:v>5.2</x:v>
+        <x:v>4.8</x:v>
       </x:c>
       <x:c r="L203" s="1" t="str">
         <x:v>Audio exists</x:v>
@@ -17625,7 +17625,7 @@
         <x:v>subzone_sludge_fields.mp3</x:v>
       </x:c>
       <x:c r="K204" s="1" t="n">
-        <x:v>4.8</x:v>
+        <x:v>3.9</x:v>
       </x:c>
       <x:c r="L204" s="1" t="str">
         <x:v>Audio exists</x:v>
@@ -17702,7 +17702,7 @@
         <x:v>subzone_writhing_haunt.mp3</x:v>
       </x:c>
       <x:c r="K205" s="1" t="n">
-        <x:v>4.7</x:v>
+        <x:v>4.6</x:v>
       </x:c>
       <x:c r="L205" s="1" t="str">
         <x:v>Audio exists</x:v>
@@ -17779,7 +17779,7 @@
         <x:v>subzone_westfall_lighthouse.mp3</x:v>
       </x:c>
       <x:c r="K206" s="1" t="n">
-        <x:v>4.8</x:v>
+        <x:v>4.4</x:v>
       </x:c>
       <x:c r="L206" s="1" t="str">
         <x:v>Audio exists</x:v>
@@ -22017,7 +22017,7 @@
         <x:v>zone_intro_01.mp3</x:v>
       </x:c>
       <x:c r="K264" t="n">
-        <x:v>6</x:v>
+        <x:v>5.6</x:v>
       </x:c>
       <x:c r="L264" t="str">
         <x:v>Audio exists</x:v>
@@ -22094,7 +22094,7 @@
         <x:v>zone_intro_02.mp3</x:v>
       </x:c>
       <x:c r="K265" t="n">
-        <x:v>6.1</x:v>
+        <x:v>6.5</x:v>
       </x:c>
       <x:c r="L265" t="str">
         <x:v>Audio exists</x:v>
@@ -22171,7 +22171,7 @@
         <x:v>quest_accept_01.mp3</x:v>
       </x:c>
       <x:c r="K266" t="n">
-        <x:v>5.4</x:v>
+        <x:v>5.2</x:v>
       </x:c>
       <x:c r="L266" t="str">
         <x:v>Audio exists</x:v>
@@ -22248,7 +22248,7 @@
         <x:v>quest_accept_02.mp3</x:v>
       </x:c>
       <x:c r="K267" t="n">
-        <x:v>4.9</x:v>
+        <x:v>4.5</x:v>
       </x:c>
       <x:c r="L267" t="str">
         <x:v>Audio exists</x:v>
@@ -22325,7 +22325,7 @@
         <x:v>quest_accept_03.mp3</x:v>
       </x:c>
       <x:c r="K268" t="n">
-        <x:v>5</x:v>
+        <x:v>4.2</x:v>
       </x:c>
       <x:c r="L268" t="str">
         <x:v>Audio exists</x:v>
@@ -22402,7 +22402,7 @@
         <x:v>kill_01.mp3</x:v>
       </x:c>
       <x:c r="K269" t="n">
-        <x:v>3.4</x:v>
+        <x:v>2.8</x:v>
       </x:c>
       <x:c r="L269" t="str">
         <x:v>Audio exists</x:v>
@@ -22556,7 +22556,7 @@
         <x:v>kill_03.mp3</x:v>
       </x:c>
       <x:c r="K271" t="n">
-        <x:v>4.6</x:v>
+        <x:v>5</x:v>
       </x:c>
       <x:c r="L271" t="str">
         <x:v>Audio exists</x:v>
@@ -22633,7 +22633,7 @@
         <x:v>idle_01.mp3</x:v>
       </x:c>
       <x:c r="K272" t="n">
-        <x:v>5.8</x:v>
+        <x:v>5</x:v>
       </x:c>
       <x:c r="L272" t="str">
         <x:v>Audio exists</x:v>
@@ -22710,7 +22710,7 @@
         <x:v>idle_02.mp3</x:v>
       </x:c>
       <x:c r="K273" t="n">
-        <x:v>6.1</x:v>
+        <x:v>5.2</x:v>
       </x:c>
       <x:c r="L273" t="str">
         <x:v>Audio exists</x:v>
@@ -22787,7 +22787,7 @@
         <x:v>idle_03.mp3</x:v>
       </x:c>
       <x:c r="K274" t="n">
-        <x:v>5.1</x:v>
+        <x:v>4.9</x:v>
       </x:c>
       <x:c r="L274" t="str">
         <x:v>Audio exists</x:v>
@@ -22864,7 +22864,7 @@
         <x:v>level_up_01.mp3</x:v>
       </x:c>
       <x:c r="K275" t="n">
-        <x:v>4.2</x:v>
+        <x:v>3.3</x:v>
       </x:c>
       <x:c r="L275" t="str">
         <x:v>Audio exists</x:v>
@@ -22941,7 +22941,7 @@
         <x:v>level_up_02.mp3</x:v>
       </x:c>
       <x:c r="K276" t="n">
-        <x:v>4.7</x:v>
+        <x:v>4.6</x:v>
       </x:c>
       <x:c r="L276" t="str">
         <x:v>Audio exists</x:v>
@@ -23018,7 +23018,7 @@
         <x:v>summon_01.mp3</x:v>
       </x:c>
       <x:c r="K277" t="n">
-        <x:v>6</x:v>
+        <x:v>6.9</x:v>
       </x:c>
       <x:c r="L277" t="str">
         <x:v>Audio exists</x:v>
@@ -23095,7 +23095,7 @@
         <x:v>bond_02_01.mp3</x:v>
       </x:c>
       <x:c r="K278" t="n">
-        <x:v>5.4</x:v>
+        <x:v>5.9</x:v>
       </x:c>
       <x:c r="L278" t="str">
         <x:v>Audio exists</x:v>
@@ -23172,7 +23172,7 @@
         <x:v>bond_04_01.mp3</x:v>
       </x:c>
       <x:c r="K279" t="n">
-        <x:v>5.4</x:v>
+        <x:v>5</x:v>
       </x:c>
       <x:c r="L279" t="str">
         <x:v>Audio exists</x:v>
@@ -23249,7 +23249,7 @@
         <x:v>bond_06_01.mp3</x:v>
       </x:c>
       <x:c r="K280" t="n">
-        <x:v>6.2</x:v>
+        <x:v>5.7</x:v>
       </x:c>
       <x:c r="L280" t="str">
         <x:v>Audio exists</x:v>
@@ -23403,7 +23403,7 @@
         <x:v>bond_10_01.mp3</x:v>
       </x:c>
       <x:c r="K282" t="n">
-        <x:v>6.5</x:v>
+        <x:v>6.7</x:v>
       </x:c>
       <x:c r="L282" t="str">
         <x:v>Audio exists</x:v>
@@ -23480,7 +23480,7 @@
         <x:v>romance_02_01.mp3</x:v>
       </x:c>
       <x:c r="K283" t="n">
-        <x:v>4.8</x:v>
+        <x:v>4.9</x:v>
       </x:c>
       <x:c r="L283" t="str">
         <x:v>Audio exists</x:v>
@@ -23557,7 +23557,7 @@
         <x:v>romance_04_01.mp3</x:v>
       </x:c>
       <x:c r="K284" t="n">
-        <x:v>5</x:v>
+        <x:v>4.2</x:v>
       </x:c>
       <x:c r="L284" t="str">
         <x:v>Audio exists</x:v>
@@ -23634,7 +23634,7 @@
         <x:v>romance_06_01.mp3</x:v>
       </x:c>
       <x:c r="K285" t="n">
-        <x:v>6</x:v>
+        <x:v>6.4</x:v>
       </x:c>
       <x:c r="L285" t="str">
         <x:v>Audio exists</x:v>
@@ -23711,7 +23711,7 @@
         <x:v>romance_08_01.mp3</x:v>
       </x:c>
       <x:c r="K286" t="n">
-        <x:v>5.7</x:v>
+        <x:v>5.1</x:v>
       </x:c>
       <x:c r="L286" t="str">
         <x:v>Audio exists</x:v>
@@ -23788,7 +23788,7 @@
         <x:v>romance_10_01.mp3</x:v>
       </x:c>
       <x:c r="K287" t="n">
-        <x:v>5.8</x:v>
+        <x:v>5.5</x:v>
       </x:c>
       <x:c r="L287" t="str">
         <x:v>Audio exists</x:v>
@@ -23865,7 +23865,7 @@
         <x:v>romance_not_ready_01.mp3</x:v>
       </x:c>
       <x:c r="K288" t="n">
-        <x:v>6</x:v>
+        <x:v>7.2</x:v>
       </x:c>
       <x:c r="L288" t="str">
         <x:v>Audio exists</x:v>
@@ -23942,7 +23942,7 @@
         <x:v>romance_repeat_01.mp3</x:v>
       </x:c>
       <x:c r="K289" t="n">
-        <x:v>4.5</x:v>
+        <x:v>3.7</x:v>
       </x:c>
       <x:c r="L289" t="str">
         <x:v>Audio exists</x:v>
@@ -24019,7 +24019,7 @@
         <x:v>romance_stop_01.mp3</x:v>
       </x:c>
       <x:c r="K290" t="n">
-        <x:v>5</x:v>
+        <x:v>3.8</x:v>
       </x:c>
       <x:c r="L290" t="str">
         <x:v>Audio exists</x:v>
@@ -24096,7 +24096,7 @@
         <x:v>quest_complete_01.mp3</x:v>
       </x:c>
       <x:c r="K291" t="n">
-        <x:v>4.6</x:v>
+        <x:v>3.5</x:v>
       </x:c>
       <x:c r="L291" t="str">
         <x:v>Audio exists</x:v>
@@ -24173,7 +24173,7 @@
         <x:v>quest_complete_02.mp3</x:v>
       </x:c>
       <x:c r="K292" t="n">
-        <x:v>5</x:v>
+        <x:v>4.4</x:v>
       </x:c>
       <x:c r="L292" t="str">
         <x:v>Audio exists</x:v>
@@ -24250,7 +24250,7 @@
         <x:v>quest_complete_03.mp3</x:v>
       </x:c>
       <x:c r="K293" t="n">
-        <x:v>5.3</x:v>
+        <x:v>4.5</x:v>
       </x:c>
       <x:c r="L293" t="str">
         <x:v>Audio exists</x:v>
@@ -24327,7 +24327,7 @@
         <x:v>bond_kill_02.mp3</x:v>
       </x:c>
       <x:c r="K294" t="n">
-        <x:v>4.2</x:v>
+        <x:v>3.4</x:v>
       </x:c>
       <x:c r="L294" t="str">
         <x:v>Audio exists</x:v>
@@ -24404,7 +24404,7 @@
         <x:v>bond_kill_04.mp3</x:v>
       </x:c>
       <x:c r="K295" t="n">
-        <x:v>4.6</x:v>
+        <x:v>3.7</x:v>
       </x:c>
       <x:c r="L295" t="str">
         <x:v>Audio exists</x:v>
@@ -24481,7 +24481,7 @@
         <x:v>bond_kill_06.mp3</x:v>
       </x:c>
       <x:c r="K296" t="n">
-        <x:v>5.6</x:v>
+        <x:v>6</x:v>
       </x:c>
       <x:c r="L296" t="str">
         <x:v>Audio exists</x:v>
@@ -24558,7 +24558,7 @@
         <x:v>bond_kill_08.mp3</x:v>
       </x:c>
       <x:c r="K297" t="n">
-        <x:v>5.3</x:v>
+        <x:v>4.7</x:v>
       </x:c>
       <x:c r="L297" t="str">
         <x:v>Audio exists</x:v>
@@ -24635,7 +24635,7 @@
         <x:v>bond_kill_10.mp3</x:v>
       </x:c>
       <x:c r="K298" t="n">
-        <x:v>4.4</x:v>
+        <x:v>4.1</x:v>
       </x:c>
       <x:c r="L298" t="str">
         <x:v>Audio exists</x:v>
@@ -24712,7 +24712,7 @@
         <x:v>bond_idle_01.mp3</x:v>
       </x:c>
       <x:c r="K299" t="n">
-        <x:v>5.5</x:v>
+        <x:v>5.1</x:v>
       </x:c>
       <x:c r="L299" t="str">
         <x:v>Audio exists</x:v>
@@ -24789,7 +24789,7 @@
         <x:v>bond_idle_03.mp3</x:v>
       </x:c>
       <x:c r="K300" t="n">
-        <x:v>5</x:v>
+        <x:v>4.2</x:v>
       </x:c>
       <x:c r="L300" t="str">
         <x:v>Audio exists</x:v>
@@ -24866,7 +24866,7 @@
         <x:v>bond_idle_05.mp3</x:v>
       </x:c>
       <x:c r="K301" t="n">
-        <x:v>5.3</x:v>
+        <x:v>4</x:v>
       </x:c>
       <x:c r="L301" t="str">
         <x:v>Audio exists</x:v>
@@ -24943,7 +24943,7 @@
         <x:v>bond_idle_07.mp3</x:v>
       </x:c>
       <x:c r="K302" t="n">
-        <x:v>4.8</x:v>
+        <x:v>4.4</x:v>
       </x:c>
       <x:c r="L302" t="str">
         <x:v>Audio exists</x:v>
@@ -25020,7 +25020,7 @@
         <x:v>bond_idle_09.mp3</x:v>
       </x:c>
       <x:c r="K303" t="n">
-        <x:v>5.1</x:v>
+        <x:v>5</x:v>
       </x:c>
       <x:c r="L303" t="str">
         <x:v>Audio exists</x:v>
@@ -25097,7 +25097,7 @@
         <x:v>low_health_01.mp3</x:v>
       </x:c>
       <x:c r="K304" t="n">
-        <x:v>3.6</x:v>
+        <x:v>2.9</x:v>
       </x:c>
       <x:c r="L304" t="str">
         <x:v>Audio exists</x:v>
@@ -25174,7 +25174,7 @@
         <x:v>death_01.mp3</x:v>
       </x:c>
       <x:c r="K305" t="n">
-        <x:v>5</x:v>
+        <x:v>4</x:v>
       </x:c>
       <x:c r="L305" t="str">
         <x:v>Audio exists</x:v>
@@ -25251,7 +25251,7 @@
         <x:v>subzone_alexston_farmstead.mp3</x:v>
       </x:c>
       <x:c r="K306" t="n">
-        <x:v>5.4</x:v>
+        <x:v>4.8</x:v>
       </x:c>
       <x:c r="L306" t="str">
         <x:v>Audio exists</x:v>
@@ -25328,7 +25328,7 @@
         <x:v>subzone_dagger_hills.mp3</x:v>
       </x:c>
       <x:c r="K307" t="n">
-        <x:v>4.8</x:v>
+        <x:v>4.5</x:v>
       </x:c>
       <x:c r="L307" t="str">
         <x:v>Audio exists</x:v>
@@ -25482,7 +25482,7 @@
         <x:v>subzone_dead_acre.mp3</x:v>
       </x:c>
       <x:c r="K309" t="n">
-        <x:v>4.8</x:v>
+        <x:v>4.5</x:v>
       </x:c>
       <x:c r="L309" t="str">
         <x:v>Audio exists</x:v>
@@ -25559,7 +25559,7 @@
         <x:v>subzone_demonts_place.mp3</x:v>
       </x:c>
       <x:c r="K310" t="n">
-        <x:v>5</x:v>
+        <x:v>4.5</x:v>
       </x:c>
       <x:c r="L310" t="str">
         <x:v>Audio exists</x:v>
@@ -25636,7 +25636,7 @@
         <x:v>subzone_dust_plains.mp3</x:v>
       </x:c>
       <x:c r="K311" t="n">
-        <x:v>4.8</x:v>
+        <x:v>3.6</x:v>
       </x:c>
       <x:c r="L311" t="str">
         <x:v>Audio exists</x:v>
@@ -25713,7 +25713,7 @@
         <x:v>subzone_furlbrows_pumpkin_farm.mp3</x:v>
       </x:c>
       <x:c r="K312" t="n">
-        <x:v>5.3</x:v>
+        <x:v>4.4</x:v>
       </x:c>
       <x:c r="L312" t="str">
         <x:v>Audio exists</x:v>
@@ -25790,7 +25790,7 @@
         <x:v>subzone_gold_coast_quarry.mp3</x:v>
       </x:c>
       <x:c r="K313" t="n">
-        <x:v>5.6</x:v>
+        <x:v>5.5</x:v>
       </x:c>
       <x:c r="L313" t="str">
         <x:v>Audio exists</x:v>
@@ -25867,7 +25867,7 @@
         <x:v>subzone_jansen_stead.mp3</x:v>
       </x:c>
       <x:c r="K314" t="n">
-        <x:v>5.2</x:v>
+        <x:v>4</x:v>
       </x:c>
       <x:c r="L314" t="str">
         <x:v>Audio exists</x:v>
@@ -25944,7 +25944,7 @@
         <x:v>subzone_jangolode_mine.mp3</x:v>
       </x:c>
       <x:c r="K315" t="n">
-        <x:v>5</x:v>
+        <x:v>4.3</x:v>
       </x:c>
       <x:c r="L315" t="str">
         <x:v>Audio exists</x:v>
@@ -26021,7 +26021,7 @@
         <x:v>subzone_molsen_farm.mp3</x:v>
       </x:c>
       <x:c r="K316" t="n">
-        <x:v>4.5</x:v>
+        <x:v>4.2</x:v>
       </x:c>
       <x:c r="L316" t="str">
         <x:v>Audio exists</x:v>
@@ -26098,7 +26098,7 @@
         <x:v>subzone_moonbrook.mp3</x:v>
       </x:c>
       <x:c r="K317" t="n">
-        <x:v>4.7</x:v>
+        <x:v>4.3</x:v>
       </x:c>
       <x:c r="L317" t="str">
         <x:v>Audio exists</x:v>
@@ -26175,7 +26175,7 @@
         <x:v>subzone_raging_chasm.mp3</x:v>
       </x:c>
       <x:c r="K318" t="n">
-        <x:v>5.2</x:v>
+        <x:v>4.3</x:v>
       </x:c>
       <x:c r="L318" t="str">
         <x:v>Audio exists</x:v>
@@ -26252,7 +26252,7 @@
         <x:v>subzone_saldeans_farm.mp3</x:v>
       </x:c>
       <x:c r="K319" t="n">
-        <x:v>4.9</x:v>
+        <x:v>4.2</x:v>
       </x:c>
       <x:c r="L319" t="str">
         <x:v>Audio exists</x:v>
@@ -26329,7 +26329,7 @@
         <x:v>subzone_sentinel_hill.mp3</x:v>
       </x:c>
       <x:c r="K320" t="n">
-        <x:v>5.1</x:v>
+        <x:v>4.4</x:v>
       </x:c>
       <x:c r="L320" t="str">
         <x:v>Audio exists</x:v>
@@ -26406,7 +26406,7 @@
         <x:v>subzone_shattered_strand.mp3</x:v>
       </x:c>
       <x:c r="K321" t="n">
-        <x:v>5.2</x:v>
+        <x:v>4.9</x:v>
       </x:c>
       <x:c r="L321" t="str">
         <x:v>Audio exists</x:v>
@@ -26483,7 +26483,7 @@
         <x:v>subzone_sludge_fields.mp3</x:v>
       </x:c>
       <x:c r="K322" t="n">
-        <x:v>4.8</x:v>
+        <x:v>3.7</x:v>
       </x:c>
       <x:c r="L322" t="str">
         <x:v>Audio exists</x:v>
@@ -26560,7 +26560,7 @@
         <x:v>subzone_writhing_haunt.mp3</x:v>
       </x:c>
       <x:c r="K323" t="n">
-        <x:v>4.7</x:v>
+        <x:v>4.3</x:v>
       </x:c>
       <x:c r="L323" t="str">
         <x:v>Audio exists</x:v>
@@ -26637,7 +26637,7 @@
         <x:v>subzone_westfall_lighthouse.mp3</x:v>
       </x:c>
       <x:c r="K324" t="n">
-        <x:v>4.8</x:v>
+        <x:v>4.6</x:v>
       </x:c>
       <x:c r="L324" t="str">
         <x:v>Audio exists</x:v>
@@ -26714,7 +26714,7 @@
         <x:v>intro_01.mp3</x:v>
       </x:c>
       <x:c r="K325" t="n">
-        <x:v>3.2</x:v>
+        <x:v>3.9</x:v>
       </x:c>
       <x:c r="L325" t="str">
         <x:v>Audio exists</x:v>
@@ -26791,7 +26791,7 @@
         <x:v>intro_02.mp3</x:v>
       </x:c>
       <x:c r="K326" t="n">
-        <x:v>7.2</x:v>
+        <x:v>14.1</x:v>
       </x:c>
       <x:c r="L326" t="str">
         <x:v>Audio exists</x:v>
@@ -26868,7 +26868,7 @@
         <x:v>intro_03.mp3</x:v>
       </x:c>
       <x:c r="K327" t="n">
-        <x:v>6.3</x:v>
+        <x:v>9.5</x:v>
       </x:c>
       <x:c r="L327" t="str">
         <x:v>Audio exists</x:v>
@@ -26945,7 +26945,7 @@
         <x:v>intro_04.mp3</x:v>
       </x:c>
       <x:c r="K328" t="n">
-        <x:v>7.5</x:v>
+        <x:v>13.8</x:v>
       </x:c>
       <x:c r="L328" t="str">
         <x:v>Audio exists</x:v>
@@ -27022,7 +27022,7 @@
         <x:v>intro_05.mp3</x:v>
       </x:c>
       <x:c r="K329" t="n">
-        <x:v>6.2</x:v>
+        <x:v>12.3</x:v>
       </x:c>
       <x:c r="L329" t="str">
         <x:v>Audio exists</x:v>
@@ -27099,7 +27099,7 @@
         <x:v>intro_06.mp3</x:v>
       </x:c>
       <x:c r="K330" t="n">
-        <x:v>6.3</x:v>
+        <x:v>11.3</x:v>
       </x:c>
       <x:c r="L330" t="str">
         <x:v>Audio exists</x:v>
@@ -27176,7 +27176,7 @@
         <x:v>intro_07.mp3</x:v>
       </x:c>
       <x:c r="K331" t="n">
-        <x:v>7</x:v>
+        <x:v>14.6</x:v>
       </x:c>
       <x:c r="L331" t="str">
         <x:v>Audio exists</x:v>
@@ -27253,7 +27253,7 @@
         <x:v>intro_08.mp3</x:v>
       </x:c>
       <x:c r="K332" t="n">
-        <x:v>5.6</x:v>
+        <x:v>8.3</x:v>
       </x:c>
       <x:c r="L332" t="str">
         <x:v>Audio exists</x:v>
@@ -27330,7 +27330,7 @@
         <x:v>intro_09.mp3</x:v>
       </x:c>
       <x:c r="K333" t="n">
-        <x:v>3.6</x:v>
+        <x:v>3.7</x:v>
       </x:c>
       <x:c r="L333" t="str">
         <x:v>Audio exists</x:v>
@@ -27378,7 +27378,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R9d9a82876c3946be"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rea9019dc1da148e9"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -38318,7 +38318,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Ra210a8e46fd74c4a"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R77d86192ab3342d3"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -38718,7 +38718,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R4749140f6bb24612"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rfee06f48fe024f81"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -39237,7 +39237,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R00cb5a824f704d34"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Re2b33100b3ec479c"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>